<commit_message>
feat: update UI components and internationalization
</commit_message>
<xml_diff>
--- a/i18n_export.xlsx
+++ b/i18n_export.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -274,567 +274,567 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">onboarding_starting</t>
+          <t xml:space="preserve">pet_dog</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Starting</t>
+          <t xml:space="preserve">Dog</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">開始中</t>
+          <t xml:space="preserve">犬</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">启动中</t>
+          <t xml:space="preserve">狗</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">啟動中</t>
+          <t xml:space="preserve">狗</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">시작 중</t>
+          <t xml:space="preserve">강아지</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">กำลังเริ่ม</t>
+          <t xml:space="preserve">สุนัข</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">pet_dog</t>
+          <t xml:space="preserve">pet_cat</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dog</t>
+          <t xml:space="preserve">Cat</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">犬</t>
+          <t xml:space="preserve">猫</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">狗</t>
+          <t xml:space="preserve">猫</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">狗</t>
+          <t xml:space="preserve">貓</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">강아지</t>
+          <t xml:space="preserve">고양이</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">สุนัข</t>
+          <t xml:space="preserve">แมว</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">pet_cat</t>
+          <t xml:space="preserve">pet_other</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cat</t>
+          <t xml:space="preserve">Other</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">猫</t>
+          <t xml:space="preserve">その他</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">猫</t>
+          <t xml:space="preserve">其他</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">貓</t>
+          <t xml:space="preserve">其他</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">고양이</t>
+          <t xml:space="preserve">기타</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">แมว</t>
+          <t xml:space="preserve">อื่นๆ</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">pet_squirrel</t>
+          <t xml:space="preserve">home_nav_change_pet</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Squirrel</t>
+          <t xml:space="preserve">Change pet</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">リス</t>
+          <t xml:space="preserve">ペット変更</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">松鼠</t>
+          <t xml:space="preserve">更换宠物</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">松鼠</t>
+          <t xml:space="preserve">更換寵物</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">다람쥐</t>
+          <t xml:space="preserve">반려동물 변경</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">กระรอก</t>
+          <t xml:space="preserve">เปลี่ยนสัตว์เลี้ยง</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">pet_hamster</t>
+          <t xml:space="preserve">home_status_temperature</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hamster</t>
+          <t xml:space="preserve">Temperature</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">ハムスター</t>
+          <t xml:space="preserve">気温</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">仓鼠</t>
+          <t xml:space="preserve">温度</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">倉鼠</t>
+          <t xml:space="preserve">溫度</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">햄스터</t>
+          <t xml:space="preserve">온도</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">แฮมสเตอร์</t>
+          <t xml:space="preserve">อุณหภูมิ</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">pet_rabbit</t>
+          <t xml:space="preserve">home_status_humidity</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rabbit</t>
+          <t xml:space="preserve">Humidity</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">兎</t>
+          <t xml:space="preserve">湿度</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">兔子</t>
+          <t xml:space="preserve">湿度</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">兔子</t>
+          <t xml:space="preserve">濕度</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">토끼</t>
+          <t xml:space="preserve">습도</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">กระต่าย</t>
+          <t xml:space="preserve">ความชื้น</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">pet_other</t>
+          <t xml:space="preserve">home_status_device</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other</t>
+          <t xml:space="preserve">Device status</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他</t>
+          <t xml:space="preserve">デバイス検出</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">其他</t>
+          <t xml:space="preserve">设备状态</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">其他</t>
+          <t xml:space="preserve">設備狀態</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타</t>
+          <t xml:space="preserve">기기 상태</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve">อื่นๆ</t>
+          <t xml:space="preserve">สถานะอุปกรณ์</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_nav_change_pet</t>
+          <t xml:space="preserve">home_temperature_good</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Change pet</t>
+          <t xml:space="preserve">Comfortable</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">ペット変更</t>
+          <t xml:space="preserve">環境が良い</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">更换宠物</t>
+          <t xml:space="preserve">环境良好</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">更換寵物</t>
+          <t xml:space="preserve">環境良好</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">반려동물 변경</t>
+          <t xml:space="preserve">쾌적함</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">เปลี่ยนสัตว์เลี้ยง</t>
+          <t xml:space="preserve">สบาย</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_status_temperature</t>
+          <t xml:space="preserve">home_temperature_high</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Temperature</t>
+          <t xml:space="preserve">Hot</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">気温</t>
+          <t xml:space="preserve">高温</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">温度</t>
+          <t xml:space="preserve">高温</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">溫度</t>
+          <t xml:space="preserve">高溫</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">온도</t>
+          <t xml:space="preserve">더움</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve">อุณหภูมิ</t>
+          <t xml:space="preserve">ร้อน</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_status_humidity</t>
+          <t xml:space="preserve">home_temperature_low</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Humidity</t>
+          <t xml:space="preserve">Cold</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">湿度</t>
+          <t xml:space="preserve">寒い</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">湿度</t>
+          <t xml:space="preserve">寒冷</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">濕度</t>
+          <t xml:space="preserve">寒冷</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">습도</t>
+          <t xml:space="preserve">추움</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ความชื้น</t>
+          <t xml:space="preserve">หนาว</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_status_device</t>
+          <t xml:space="preserve">home_tab_climate</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Device status</t>
+          <t xml:space="preserve">Climate</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">デバイス検出</t>
+          <t xml:space="preserve">ミストファン</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">设备状态</t>
+          <t xml:space="preserve">温湿度管理</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">設備狀態</t>
+          <t xml:space="preserve">溫濕度管理</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">기기 상태</t>
+          <t xml:space="preserve">기후</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">สถานะอุปกรณ์</t>
+          <t xml:space="preserve">สภาพอากาศ</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_temperature_good</t>
+          <t xml:space="preserve">home_tab_disinfection</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comfortable</t>
+          <t xml:space="preserve">Quick disinfection</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境が良い</t>
+          <t xml:space="preserve">スピード消毒</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">环境良好</t>
+          <t xml:space="preserve">快速消毒</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境良好</t>
+          <t xml:space="preserve">快速消毒</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">쾌적함</t>
+          <t xml:space="preserve">빠른 살균</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t xml:space="preserve">สบาย</t>
+          <t xml:space="preserve">ฆ่าเชื้อด่วน</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_temperature_high</t>
+          <t xml:space="preserve">home_tab_light</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hot</t>
+          <t xml:space="preserve">Light</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">高温</t>
+          <t xml:space="preserve">ライト</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">高温</t>
+          <t xml:space="preserve">灯光</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">高溫</t>
+          <t xml:space="preserve">燈光</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">더움</t>
+          <t xml:space="preserve">조명</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t xml:space="preserve">ร้อน</t>
+          <t xml:space="preserve">ไฟ</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_temperature_low</t>
+          <t xml:space="preserve">home_action_mist</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cold</t>
+          <t xml:space="preserve">Mist</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">寒い</t>
+          <t xml:space="preserve">ミスト</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">寒冷</t>
+          <t xml:space="preserve">喷雾</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">寒冷</t>
+          <t xml:space="preserve">噴霧</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">추움</t>
+          <t xml:space="preserve">미스트</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t xml:space="preserve">หนาว</t>
+          <t xml:space="preserve">ละอองน้ำ</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_tab_climate</t>
+          <t xml:space="preserve">home_action_fan</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Climate</t>
+          <t xml:space="preserve">Fan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミストファン</t>
+          <t xml:space="preserve">風量設定</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">温湿度管理</t>
+          <t xml:space="preserve">风扇</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">溫濕度管理</t>
+          <t xml:space="preserve">風扇</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">기후</t>
+          <t xml:space="preserve">팬</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t xml:space="preserve">สภาพอากาศ</t>
+          <t xml:space="preserve">พัดลม</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_tab_disinfection</t>
+          <t xml:space="preserve">home_action_disinfection_quick</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quick disinfection</t>
+          <t xml:space="preserve">Quick</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -854,1157 +854,1009 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">빠른 살균</t>
+          <t xml:space="preserve">빠르게</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t xml:space="preserve">ฆ่าเชื้อด่วน</t>
+          <t xml:space="preserve">ด่วน</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_tab_light</t>
+          <t xml:space="preserve">home_action_disinfection_deep</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light</t>
+          <t xml:space="preserve">Deep</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">灯</t>
+          <t xml:space="preserve">通常消毒</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">灯光</t>
+          <t xml:space="preserve">彻底消毒</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">燈光</t>
+          <t xml:space="preserve">徹底消毒</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">조명</t>
+          <t xml:space="preserve">집중</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve">ไฟ</t>
+          <t xml:space="preserve">ลึก</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_mist</t>
+          <t xml:space="preserve">home_action_light_red</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mist</t>
+          <t xml:space="preserve">Red</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミスト</t>
+          <t xml:space="preserve">赤色</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">喷雾</t>
+          <t xml:space="preserve">红色</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">噴霧</t>
+          <t xml:space="preserve">紅色</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">미스트</t>
+          <t xml:space="preserve">빨간색</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t xml:space="preserve">ละอองน้ำ</t>
+          <t xml:space="preserve">สีแดง</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_fan</t>
+          <t xml:space="preserve">home_action_light_blue</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fan</t>
+          <t xml:space="preserve">Blue</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">風量設定</t>
+          <t xml:space="preserve">青色</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">风扇</t>
+          <t xml:space="preserve">蓝色</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">風扇</t>
+          <t xml:space="preserve">藍色</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">팬</t>
+          <t xml:space="preserve">파란색</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t xml:space="preserve">พัดลม</t>
+          <t xml:space="preserve">สีน้ำเงิน</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_disinfection_quick</t>
+          <t xml:space="preserve">home_action_light_green</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quick</t>
+          <t xml:space="preserve">Green</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">スピード消毒</t>
+          <t xml:space="preserve">緑色</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">快速消毒</t>
+          <t xml:space="preserve">绿色</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">快速消毒</t>
+          <t xml:space="preserve">綠色</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">빠르게</t>
+          <t xml:space="preserve">초록색</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">ด่วน</t>
+          <t xml:space="preserve">สีเขียว</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_disinfection_deep</t>
+          <t xml:space="preserve">scene_title</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deep</t>
+          <t xml:space="preserve">Scene</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">通常消毒</t>
+          <t xml:space="preserve">シーン</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">彻底消毒</t>
+          <t xml:space="preserve">场景</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">徹底消毒</t>
+          <t xml:space="preserve">場景</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">집중</t>
+          <t xml:space="preserve">장면</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve">ลึก</t>
+          <t xml:space="preserve">ฉาก</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_light_red</t>
+          <t xml:space="preserve">scene_action_auto</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Red</t>
+          <t xml:space="preserve">Auto</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">赤色</t>
+          <t xml:space="preserve">自動</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">红色</t>
+          <t xml:space="preserve">自动</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">紅色</t>
+          <t xml:space="preserve">自動</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">빨간색</t>
+          <t xml:space="preserve">자동</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t xml:space="preserve">สีแดง</t>
+          <t xml:space="preserve">อัตโนมัติ</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_light_blue</t>
+          <t xml:space="preserve">home_o3_toast_pause</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blue</t>
+          <t xml:space="preserve">Human/animal detected. Disinfection paused. Resume after cleared.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">青色</t>
+          <t xml:space="preserve">人・動物検知、消毒停止。解除後、再開。</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">蓝色</t>
+          <t xml:space="preserve">检测到人/动物，消毒已暂停。解除后恢复。</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">藍色</t>
+          <t xml:space="preserve">檢測到人/動物，消毒已暫停。解除後恢復。</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">파란색</t>
+          <t xml:space="preserve">사람/동물이 감지되어 살균이 일시 중지되었습니다. 해제 후 재개됩니다.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t xml:space="preserve">สีน้ำเงิน</t>
+          <t xml:space="preserve">ตรวจพบคน/สัตว์ การฆ่าเชื้อถูกหยุดชั่วคราว และจะทำงานต่อเมื่อพื้นที่ปลอดภัย</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_light_green</t>
+          <t xml:space="preserve">home_o3_toast_running</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green</t>
+          <t xml:space="preserve">Disinfecting. Keep people/animals away.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">緑色</t>
+          <t xml:space="preserve">消毒中、人・動物は遠ざけてください。</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">绿色</t>
+          <t xml:space="preserve">消毒中，请远离人/动物。</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">綠色</t>
+          <t xml:space="preserve">消毒中，請遠離人/動物。</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">초록색</t>
+          <t xml:space="preserve">살균 중입니다. 사람/동물은 가까이 오지 마세요.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t xml:space="preserve">สีเขียว</t>
+          <t xml:space="preserve">กำลังฆ่าเชื้อ โปรดอยู่ห่างจากคน/สัตว์</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">scene_action_auto</t>
+          <t xml:space="preserve">home_o3_status_recovery</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Auto</t>
+          <t xml:space="preserve">Recovery after emergency stop</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">自動</t>
+          <t xml:space="preserve">緊急停止後の回復フェーズ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">自动</t>
+          <t xml:space="preserve">紧急停止后的恢复阶段</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">自動</t>
+          <t xml:space="preserve">緊急停止後的恢復階段</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">자동</t>
+          <t xml:space="preserve">긴급 정지 후 복구 단계</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">อัตโนมัติ</t>
+          <t xml:space="preserve">ช่วงฟื้นตัวหลังหยุดฉุกเฉิน</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_toast_pause</t>
+          <t xml:space="preserve">home_o3_status_diffuse</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Human/animal detected. Disinfection paused. Resume after cleared.</t>
+          <t xml:space="preserve">Dispersing with strong airflow</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">人・動物検知、消毒停止。解除後、再開。</t>
+          <t xml:space="preserve">オゾン消毒後待機中</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">检测到人/动物，消毒已暂停。解除后恢复。</t>
+          <t xml:space="preserve">强风扩散中</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">檢測到人/動物，消毒已暫停。解除後恢復。</t>
+          <t xml:space="preserve">強風擴散中</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">사람/동물이 감지되어 살균이 일시 중지되었습니다. 해제 후 재개됩니다.</t>
+          <t xml:space="preserve">강한 바람으로 확산 중</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">ตรวจพบคน/สัตว์ การฆ่าเชื้อถูกหยุดชั่วคราว และจะทำงานต่อเมื่อพื้นที่ปลอดภัย</t>
+          <t xml:space="preserve">กำลังกระจายด้วยลมแรง</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_toast_running</t>
+          <t xml:space="preserve">disinfection_title</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Disinfecting. Keep people/animals away.</t>
+          <t xml:space="preserve">Ozone disinfection</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">消毒中、人・動物は遠ざけてください。</t>
+          <t xml:space="preserve">オゾン消毒</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">消毒中，请远离人/动物。</t>
+          <t xml:space="preserve">臭氧消毒</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">消毒中，請遠離人/動物。</t>
+          <t xml:space="preserve">臭氧消毒</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">살균 중입니다. 사람/동물은 가까이 오지 마세요.</t>
+          <t xml:space="preserve">오존 살균</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">กำลังฆ่าเชื้อ โปรดอยู่ห่างจากคน/สัตว์</t>
+          <t xml:space="preserve">ฆ่าเชื้อด้วยโอโซน</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_status_recovery</t>
+          <t xml:space="preserve">disinfection_status_paused</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recovery after emergency stop</t>
+          <t xml:space="preserve">Paused</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">緊急停止後の回復フェーズ</t>
+          <t xml:space="preserve">停止</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">紧急停止后的恢复阶段</t>
+          <t xml:space="preserve">已暂停</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">緊急停止後的恢復階段</t>
+          <t xml:space="preserve">已暫停</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">긴급 정지 후 복구 단계</t>
+          <t xml:space="preserve">일시 중지됨</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">ช่วงฟื้นตัวหลังหยุดฉุกเฉิน</t>
+          <t xml:space="preserve">หยุดชั่วคราว</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_status_diffuse</t>
+          <t xml:space="preserve">disinfection_note_stopped</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dispersing with strong airflow</t>
+          <t xml:space="preserve">People or animals are still active in the area. Ozone has stopped.</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">オゾン消毒後待機中</t>
+          <t xml:space="preserve">人や動物の活動が続いているため、オゾンを停止しました。</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">强风扩散中</t>
+          <t xml:space="preserve">环境持续有人员活动，臭氧已停止。</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">強風擴散中</t>
+          <t xml:space="preserve">環境持續有人員活動，臭氧已停止。</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">강한 바람으로 확산 중</t>
+          <t xml:space="preserve">주변에 사람이나 동물의 움직임이 계속 감지되어 오존이 중지되었습니다.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve">กำลังกระจายด้วยลมแรง</t>
+          <t xml:space="preserve">ยังตรวจพบการเคลื่อนไหวของคนหรือสัตว์ในพื้นที่ โอโซนจึงหยุดทำงาน</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_title</t>
+          <t xml:space="preserve">disinfection_note_paused</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ozone disinfection</t>
+          <t xml:space="preserve">Person or pet detected. Ozone has paused.</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">オゾン消毒</t>
+          <t xml:space="preserve">人やペットを検知したため、オゾンを一時停止しました。</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">臭氧消毒</t>
+          <t xml:space="preserve">检测到人员或宠物，臭氧已暂停。</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">臭氧消毒</t>
+          <t xml:space="preserve">偵測到人員或寵物，臭氧已暫停。</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">오존 살균</t>
+          <t xml:space="preserve">사람 또는 반려동물이 감지되어 오존이 일시 중지되었습니다.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve">ฆ่าเชื้อด้วยโอโซน</t>
+          <t xml:space="preserve">ตรวจพบคนหรือสัตว์เลี้ยง โอโซนจึงหยุดชั่วคราว</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_status_paused</t>
+          <t xml:space="preserve">disinfection_note_running</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paused</t>
+          <t xml:space="preserve">Area is clear. Ozone has restarted.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">停止</t>
+          <t xml:space="preserve">環境がクリアになったため、オゾンを再起動しました。</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">已暂停</t>
+          <t xml:space="preserve">环境已清空，臭氧重新启动。</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">已暫停</t>
+          <t xml:space="preserve">環境已清空，臭氧重新啟動。</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">일시 중지됨</t>
+          <t xml:space="preserve">주변이 비어 있어 오존이 다시 시작되었습니다.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve">หยุดชั่วคราว</t>
+          <t xml:space="preserve">พื้นที่ปลอดคนแล้ว โอโซนเริ่มทำงานอีกครั้ง</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_remaining_minutes</t>
+          <t xml:space="preserve">disinfection_detected</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Remaining {0} min</t>
+          <t xml:space="preserve">● People/animals detected.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">残り{0}分</t>
+          <t xml:space="preserve">● 人や動物を検知しました。</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">剩余{0}分钟</t>
+          <t xml:space="preserve">● 检测到人/动物。</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">剩餘{0}分鐘</t>
+          <t xml:space="preserve">● 檢測到人/動物。</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">{0}분 남음</t>
+          <t xml:space="preserve">● 사람/동물이 감지되었습니다.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">เหลืออีก {0} นาที</t>
+          <t xml:space="preserve">● ตรวจพบคน/สัตว์</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_note_stopped</t>
+          <t xml:space="preserve">disinfection_not_detected</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">People or animals are still active in the area. Ozone has stopped.</t>
+          <t xml:space="preserve">● No people/pets detected.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">人や動物の活動が続いているため、オゾンを停止しました。</t>
+          <t xml:space="preserve">● 人や動物は検知されていません</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">环境持续有人员活动，臭氧已停止。</t>
+          <t xml:space="preserve">● 未检测到人/宠物。</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境持續有人員活動，臭氧已停止。</t>
+          <t xml:space="preserve">● 未檢測到人/寵物。</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">주변에 사람이나 동물의 움직임이 계속 감지되어 오존이 중지되었습니다.</t>
+          <t xml:space="preserve">● 사람/반려동물이 감지되지 않았습니다.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve">ยังตรวจพบการเคลื่อนไหวของคนหรือสัตว์ในพื้นที่ โอโซนจึงหยุดทำงาน</t>
+          <t xml:space="preserve">● ไม่พบคน/สัตว์เลี้ยง</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_note_paused</t>
+          <t xml:space="preserve">mist_title</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Person or pet detected. Ozone has paused.</t>
+          <t xml:space="preserve">Mist level</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">人やペットを検知したため、オゾンを一時停止しました。</t>
+          <t xml:space="preserve">ミスト設定</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">检测到人员或宠物，臭氧已暂停。</t>
+          <t xml:space="preserve">喷雾量设置</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">偵測到人員或寵物，臭氧已暫停。</t>
+          <t xml:space="preserve">噴霧量設定</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">사람 또는 반려동물이 감지되어 오존이 일시 중지되었습니다.</t>
+          <t xml:space="preserve">미스트 단계</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">ตรวจพบคนหรือสัตว์เลี้ยง โอโซนจึงหยุดชั่วคราว</t>
+          <t xml:space="preserve">ระดับละอองน้ำ</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_note_running</t>
+          <t xml:space="preserve">mist_nozzle_1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Area is clear. Ozone has restarted.</t>
+          <t xml:space="preserve">Nozzle 1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境がクリアになったため、オゾンを再起動しました。</t>
+          <t xml:space="preserve">ミスト1</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">环境已清空，臭氧重新启动。</t>
+          <t xml:space="preserve">喷嘴1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境已清空，臭氧重新啟動。</t>
+          <t xml:space="preserve">噴嘴1</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">주변이 비어 있어 오존이 다시 시작되었습니다.</t>
+          <t xml:space="preserve">노즐 1</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นที่ปลอดคนแล้ว โอโซนเริ่มทำงานอีกครั้ง</t>
+          <t xml:space="preserve">หัวพ่น 1</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_detected</t>
+          <t xml:space="preserve">mist_nozzle_2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">● People/animals detected.</t>
+          <t xml:space="preserve">Nozzle 2</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 人や動物を検知しました。</t>
+          <t xml:space="preserve">ミスト2</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 检测到人/动物。</t>
+          <t xml:space="preserve">喷嘴2</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 檢測到人/動物。</t>
+          <t xml:space="preserve">噴嘴2</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 사람/동물이 감지되었습니다.</t>
+          <t xml:space="preserve">노즐 2</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">● ตรวจพบคน/สัตว์</t>
+          <t xml:space="preserve">หัวพ่น 2</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_not_detected</t>
+          <t xml:space="preserve">fan_title</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">● No people/pets detected.</t>
+          <t xml:space="preserve">Fan level</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 人や動物は検知されていません</t>
+          <t xml:space="preserve">風量設定</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 未检测到人/宠物。</t>
+          <t xml:space="preserve">风量设置</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 未檢測到人/寵物。</t>
+          <t xml:space="preserve">風量設定</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 사람/반려동물이 감지되지 않았습니다.</t>
+          <t xml:space="preserve">팬 단계</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t xml:space="preserve">● ไม่พบคน/สัตว์เลี้ยง</t>
+          <t xml:space="preserve">ระดับพัดลม</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">mist_title</t>
+          <t xml:space="preserve">cooling_title</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mist level</t>
+          <t xml:space="preserve">Cooling mode</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミスト設定</t>
+          <t xml:space="preserve">冷房モード</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">喷雾量设置</t>
+          <t xml:space="preserve">制冷模式</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">噴霧量設定</t>
+          <t xml:space="preserve">製冷模式</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t xml:space="preserve">미스트 단계</t>
+          <t xml:space="preserve">냉각 모드</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">ระดับละอองน้ำ</t>
+          <t xml:space="preserve">โหมดทำความเย็น</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">mist_nozzle_1</t>
+          <t xml:space="preserve">cooling_mode_intermittent</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nozzle 1</t>
+          <t xml:space="preserve">Intermittent</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミスト1</t>
+          <t xml:space="preserve">クーリングモード断続</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">喷嘴1</t>
+          <t xml:space="preserve">间歇</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">噴嘴1</t>
+          <t xml:space="preserve">間歇</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">노즐 1</t>
+          <t xml:space="preserve">간헐</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t xml:space="preserve">หัวพ่น 1</t>
+          <t xml:space="preserve">เป็นช่วง</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">mist_nozzle_2</t>
+          <t xml:space="preserve">cooling_mode_continuous</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nozzle 2</t>
+          <t xml:space="preserve">Continuous</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミスト2</t>
+          <t xml:space="preserve">クーリングモード継続</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">喷嘴2</t>
+          <t xml:space="preserve">持续</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">噴嘴2</t>
+          <t xml:space="preserve">持續</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">노즐 2</t>
+          <t xml:space="preserve">연속</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t xml:space="preserve">หัวพ่น 2</t>
+          <t xml:space="preserve">ต่อเนื่อง</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">fan_title</t>
+          <t xml:space="preserve">light_title</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fan level</t>
+          <t xml:space="preserve">Light</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">風量設定</t>
+          <t xml:space="preserve">ライト</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">风量设置</t>
+          <t xml:space="preserve">灯光</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">風量設定</t>
+          <t xml:space="preserve">燈光</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve">팬 단계</t>
+          <t xml:space="preserve">조명</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t xml:space="preserve">ระดับพัดลม</t>
+          <t xml:space="preserve">ไฟ</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">cooling_title</t>
+          <t xml:space="preserve">power_hint_off</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cooling mode</t>
+          <t xml:space="preserve">≪ Power off</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">冷房モード</t>
+          <t xml:space="preserve">≪ 電源を切る</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">制冷模式</t>
+          <t xml:space="preserve">≪ 关闭电源</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">製冷模式</t>
+          <t xml:space="preserve">≪ 關閉電源</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t xml:space="preserve">냉각 모드</t>
+          <t xml:space="preserve">≪ 전원 끄기</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t xml:space="preserve">โหมดทำความเย็น</t>
+          <t xml:space="preserve">≪ ปิดเครื่อง</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">cooling_mode_intermittent</t>
+          <t xml:space="preserve">power_hint_on</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Intermittent</t>
+          <t xml:space="preserve">Power on ≫</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">クーリングモード断続</t>
+          <t xml:space="preserve">電源を入れる ≫</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">间歇</t>
+          <t xml:space="preserve">开启电源 ≫</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">間歇</t>
+          <t xml:space="preserve">開啟電源 ≫</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t xml:space="preserve">간헐</t>
+          <t xml:space="preserve">전원 켜기 ≫</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">เป็นช่วง</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cooling_mode_continuous</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Continuous</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">クーリングモード継続</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">持续</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">持續</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">연속</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ต่อเนื่อง</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">light_title</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Light</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ライト</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">灯光</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">燈光</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조명</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ไฟ</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">power_hint_off</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">≪ Power off</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">≪ 電源を切る</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">≪ 关闭电源</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">≪ 關閉電源</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">≪ 전원 끄기</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">≪ ปิดเครื่อง</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">power_hint_on</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Power on ≫</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">電源を入れる ≫</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">开启电源 ≫</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">開啟電源 ≫</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">전원 켜기 ≫</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
         <is>
           <t xml:space="preserve">เปิดเครื่อง ≫</t>
         </is>

</xml_diff>

<commit_message>
feat: update home controls and cleanup legacy pages
Adjust light and disinfection behavior, refresh i18n, and remove onboarding and mist modal flows.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/i18n_export.xlsx
+++ b/i18n_export.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -903,37 +903,37 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_light_red</t>
+          <t xml:space="preserve">home_action_light_white</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Red</t>
+          <t xml:space="preserve">White</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">赤色</t>
+          <t xml:space="preserve">白色</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">红色</t>
+          <t xml:space="preserve">白色</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">紅色</t>
+          <t xml:space="preserve">白色</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">빨간색</t>
+          <t xml:space="preserve">흰색</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t xml:space="preserve">สีแดง</t>
+          <t xml:space="preserve">สีขาว</t>
         </is>
       </c>
     </row>
@@ -1236,627 +1236,738 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_title</t>
+          <t xml:space="preserve">home_o3_status_fan_remaining_minutes</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ozone disinfection</t>
+          <t xml:space="preserve">Fan remaining: {0} min</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">オゾン消毒</t>
+          <t xml:space="preserve">送風の残り時間：{0}分</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">臭氧消毒</t>
+          <t xml:space="preserve">吹风剩余：{0}分钟</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">臭氧消毒</t>
+          <t xml:space="preserve">吹風剩餘：{0}分鐘</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">오존 살균</t>
+          <t xml:space="preserve">송풍 남은 시간: {0}분</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">ฆ่าเชื้อด้วยโอโซน</t>
+          <t xml:space="preserve">เวลาพัดลมคงเหลือ: {0} นาที</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_status_paused</t>
+          <t xml:space="preserve">home_o3_status_fan_finished</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paused</t>
+          <t xml:space="preserve">Fan finished</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">停止</t>
+          <t xml:space="preserve">送風終了</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">已暂停</t>
+          <t xml:space="preserve">吹风结束</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">已暫停</t>
+          <t xml:space="preserve">吹風結束</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">일시 중지됨</t>
+          <t xml:space="preserve">송풍 종료</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">หยุดชั่วคราว</t>
+          <t xml:space="preserve">พัดลมสิ้นสุดแล้ว</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_note_stopped</t>
+          <t xml:space="preserve">disinfection_title</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">People or animals are still active in the area. Ozone has stopped.</t>
+          <t xml:space="preserve">Ozone disinfection</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">人や動物の活動が続いているため、オゾンを停止しました。</t>
+          <t xml:space="preserve">オゾン消毒</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">环境持续有人员活动，臭氧已停止。</t>
+          <t xml:space="preserve">臭氧消毒</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境持續有人員活動，臭氧已停止。</t>
+          <t xml:space="preserve">臭氧消毒</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">주변에 사람이나 동물의 움직임이 계속 감지되어 오존이 중지되었습니다.</t>
+          <t xml:space="preserve">오존 살균</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve">ยังตรวจพบการเคลื่อนไหวของคนหรือสัตว์ในพื้นที่ โอโซนจึงหยุดทำงาน</t>
+          <t xml:space="preserve">ฆ่าเชื้อด้วยโอโซน</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_note_paused</t>
+          <t xml:space="preserve">disinfection_status_paused</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Person or pet detected. Ozone has paused.</t>
+          <t xml:space="preserve">Paused</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">人やペットを検知したため、オゾンを一時停止しました。</t>
+          <t xml:space="preserve">停止</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">检测到人员或宠物，臭氧已暂停。</t>
+          <t xml:space="preserve">已暂停</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">偵測到人員或寵物，臭氧已暫停。</t>
+          <t xml:space="preserve">已暫停</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">사람 또는 반려동물이 감지되어 오존이 일시 중지되었습니다.</t>
+          <t xml:space="preserve">일시 중지됨</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve">ตรวจพบคนหรือสัตว์เลี้ยง โอโซนจึงหยุดชั่วคราว</t>
+          <t xml:space="preserve">หยุดชั่วคราว</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_note_running</t>
+          <t xml:space="preserve">disinfection_remaining_minutes</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Area is clear. Ozone has restarted.</t>
+          <t xml:space="preserve">{0} min remaining</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境がクリアになったため、オゾンを再起動しました。</t>
+          <t xml:space="preserve">残り{0}分</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">环境已清空，臭氧重新启动。</t>
+          <t xml:space="preserve">剩余{0}分钟</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境已清空，臭氧重新啟動。</t>
+          <t xml:space="preserve">剩餘{0}分鐘</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">주변이 비어 있어 오존이 다시 시작되었습니다.</t>
+          <t xml:space="preserve">{0}분 남음</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นที่ปลอดคนแล้ว โอโซนเริ่มทำงานอีกครั้ง</t>
+          <t xml:space="preserve">เหลืออีก {0} นาที</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_detected</t>
+          <t xml:space="preserve">disinfection_note_stopped</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">● People/animals detected.</t>
+          <t xml:space="preserve">People or animals are still active in the area. Ozone has stopped.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 人や動物を検知しました。</t>
+          <t xml:space="preserve">人や動物の活動が続いているため、オゾンを停止しました。</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 检测到人/动物。</t>
+          <t xml:space="preserve">环境持续有人员活动，臭氧已停止。</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 檢測到人/動物。</t>
+          <t xml:space="preserve">環境持續有人員活動，臭氧已停止。</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 사람/동물이 감지되었습니다.</t>
+          <t xml:space="preserve">주변에 사람이나 동물의 움직임이 계속 감지되어 오존이 중지되었습니다.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">● ตรวจพบคน/สัตว์</t>
+          <t xml:space="preserve">ยังตรวจพบการเคลื่อนไหวของคนหรือสัตว์ในพื้นที่ โอโซนจึงหยุดทำงาน</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_not_detected</t>
+          <t xml:space="preserve">disinfection_note_paused</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">● No people/pets detected.</t>
+          <t xml:space="preserve">Person or pet detected. Ozone has paused.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 人や動物は検知されていません</t>
+          <t xml:space="preserve">人やペットを検知したため、オゾンを一時停止しました。</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 未检测到人/宠物。</t>
+          <t xml:space="preserve">检测到人员或宠物，臭氧已暂停。</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 未檢測到人/寵物。</t>
+          <t xml:space="preserve">偵測到人員或寵物，臭氧已暫停。</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 사람/반려동물이 감지되지 않았습니다.</t>
+          <t xml:space="preserve">사람 또는 반려동물이 감지되어 오존이 일시 중지되었습니다.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve">● ไม่พบคน/สัตว์เลี้ยง</t>
+          <t xml:space="preserve">ตรวจพบคนหรือสัตว์เลี้ยง โอโซนจึงหยุดชั่วคราว</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">mist_title</t>
+          <t xml:space="preserve">disinfection_note_running</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mist level</t>
+          <t xml:space="preserve">Area is clear. Ozone has restarted.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミスト設定</t>
+          <t xml:space="preserve">環境がクリアになったため、オゾンを再起動しました。</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">喷雾量设置</t>
+          <t xml:space="preserve">环境已清空，臭氧重新启动。</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">噴霧量設定</t>
+          <t xml:space="preserve">環境已清空，臭氧重新啟動。</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">미스트 단계</t>
+          <t xml:space="preserve">주변이 비어 있어 오존이 다시 시작되었습니다.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">ระดับละอองน้ำ</t>
+          <t xml:space="preserve">พื้นที่ปลอดคนแล้ว โอโซนเริ่มทำงานอีกครั้ง</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">mist_nozzle_1</t>
+          <t xml:space="preserve">disinfection_detected</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nozzle 1</t>
+          <t xml:space="preserve">● People/animals detected.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミスト1</t>
+          <t xml:space="preserve">● 人や動物を検知しました。</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">喷嘴1</t>
+          <t xml:space="preserve">● 检测到人/动物。</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">噴嘴1</t>
+          <t xml:space="preserve">● 檢測到人/動物。</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">노즐 1</t>
+          <t xml:space="preserve">● 사람/동물이 감지되었습니다.</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve">หัวพ่น 1</t>
+          <t xml:space="preserve">● ตรวจพบคน/สัตว์</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">mist_nozzle_2</t>
+          <t xml:space="preserve">disinfection_not_detected</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nozzle 2</t>
+          <t xml:space="preserve">● No people/pets detected.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミスト2</t>
+          <t xml:space="preserve">● 人や動物は検知されていません</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">喷嘴2</t>
+          <t xml:space="preserve">● 未检测到人/宠物。</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">噴嘴2</t>
+          <t xml:space="preserve">● 未檢測到人/寵物。</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">노즐 2</t>
+          <t xml:space="preserve">● 사람/반려동물이 감지되지 않았습니다.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">หัวพ่น 2</t>
+          <t xml:space="preserve">● ไม่พบคน/สัตว์เลี้ยง</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">fan_title</t>
+          <t xml:space="preserve">mist_title</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fan level</t>
+          <t xml:space="preserve">Mist level</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">風量設定</t>
+          <t xml:space="preserve">ミスト設定</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">风量设置</t>
+          <t xml:space="preserve">喷雾量设置</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">風量設定</t>
+          <t xml:space="preserve">噴霧量設定</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">팬 단계</t>
+          <t xml:space="preserve">미스트 단계</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t xml:space="preserve">ระดับพัดลม</t>
+          <t xml:space="preserve">ระดับละอองน้ำ</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">cooling_title</t>
+          <t xml:space="preserve">mist_nozzle_1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cooling mode</t>
+          <t xml:space="preserve">Nozzle 1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">冷房モード</t>
+          <t xml:space="preserve">ミスト1</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">制冷模式</t>
+          <t xml:space="preserve">喷嘴1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">製冷模式</t>
+          <t xml:space="preserve">噴嘴1</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t xml:space="preserve">냉각 모드</t>
+          <t xml:space="preserve">노즐 1</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">โหมดทำความเย็น</t>
+          <t xml:space="preserve">หัวพ่น 1</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">cooling_mode_intermittent</t>
+          <t xml:space="preserve">mist_nozzle_2</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Intermittent</t>
+          <t xml:space="preserve">Nozzle 2</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">クーリングモード断続</t>
+          <t xml:space="preserve">ミスト2</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">间歇</t>
+          <t xml:space="preserve">喷嘴2</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">間歇</t>
+          <t xml:space="preserve">噴嘴2</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">간헐</t>
+          <t xml:space="preserve">노즐 2</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t xml:space="preserve">เป็นช่วง</t>
+          <t xml:space="preserve">หัวพ่น 2</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">cooling_mode_continuous</t>
+          <t xml:space="preserve">fan_title</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Continuous</t>
+          <t xml:space="preserve">Fan level</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">クーリングモード継続</t>
+          <t xml:space="preserve">風量設定</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">持续</t>
+          <t xml:space="preserve">风量设置</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">持續</t>
+          <t xml:space="preserve">風量設定</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">연속</t>
+          <t xml:space="preserve">팬 단계</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t xml:space="preserve">ต่อเนื่อง</t>
+          <t xml:space="preserve">ระดับพัดลม</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">light_title</t>
+          <t xml:space="preserve">cooling_title</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light</t>
+          <t xml:space="preserve">Cooling mode</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">ライト</t>
+          <t xml:space="preserve">冷房モード</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">灯光</t>
+          <t xml:space="preserve">制冷模式</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">燈光</t>
+          <t xml:space="preserve">製冷模式</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve">조명</t>
+          <t xml:space="preserve">냉각 모드</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t xml:space="preserve">ไฟ</t>
+          <t xml:space="preserve">โหมดทำความเย็น</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">power_hint_off</t>
+          <t xml:space="preserve">cooling_mode_intermittent</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">≪ Power off</t>
+          <t xml:space="preserve">Intermittent</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">≪ 電源を切る</t>
+          <t xml:space="preserve">クーリングモード断続</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">≪ 关闭电源</t>
+          <t xml:space="preserve">间歇</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">≪ 關閉電源</t>
+          <t xml:space="preserve">間歇</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t xml:space="preserve">≪ 전원 끄기</t>
+          <t xml:space="preserve">간헐</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t xml:space="preserve">≪ ปิดเครื่อง</t>
+          <t xml:space="preserve">เป็นช่วง</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t xml:space="preserve">cooling_mode_continuous</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Continuous</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">クーリングモード継続</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">持续</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">持續</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">연속</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ต่อเนื่อง</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">light_title</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Light</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ライト</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">灯光</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">燈光</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조명</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ไฟ</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">power_hint_off</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">≪ Power off</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">≪ 電源を切る</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">≪ 关闭电源</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">≪ 關閉電源</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">≪ 전원 끄기</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">≪ ปิดเครื่อง</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t xml:space="preserve">power_hint_on</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t xml:space="preserve">Power on ≫</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t xml:space="preserve">電源を入れる ≫</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t xml:space="preserve">开启电源 ≫</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t xml:space="preserve">開啟電源 ≫</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t xml:space="preserve">전원 켜기 ≫</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
+      <c r="G53" t="inlineStr">
         <is>
           <t xml:space="preserve">เปิดเครื่อง ≫</t>
         </is>

</xml_diff>

<commit_message>
refactor: simplify home tabs and refine disinfection controls
Remove the light tab and show 60/90 minute disinfection labels.
Lock climate controls while ozone is running.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/i18n_export.xlsx
+++ b/i18n_export.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -686,1288 +686,1103 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quick disinfection</t>
+          <t xml:space="preserve">Disinfection</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">スピード消毒</t>
+          <t xml:space="preserve">消毒</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">快速消毒</t>
+          <t xml:space="preserve">消毒</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">快速消毒</t>
+          <t xml:space="preserve">消毒</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">빠른 살균</t>
+          <t xml:space="preserve">살균</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ฆ่าเชื้อด่วน</t>
+          <t xml:space="preserve">ฆ่าเชื้อ</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_tab_light</t>
+          <t xml:space="preserve">home_action_mist</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light</t>
+          <t xml:space="preserve">Mist</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">ライト</t>
+          <t xml:space="preserve">ミスト</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">灯光</t>
+          <t xml:space="preserve">喷雾</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">燈光</t>
+          <t xml:space="preserve">噴霧</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">조명</t>
+          <t xml:space="preserve">미스트</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t xml:space="preserve">ไฟ</t>
+          <t xml:space="preserve">ละอองน้ำ</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_mist</t>
+          <t xml:space="preserve">home_action_fan</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mist</t>
+          <t xml:space="preserve">Fan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミスト</t>
+          <t xml:space="preserve">風量設定</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">喷雾</t>
+          <t xml:space="preserve">风扇</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">噴霧</t>
+          <t xml:space="preserve">風扇</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">미스트</t>
+          <t xml:space="preserve">팬</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t xml:space="preserve">ละอองน้ำ</t>
+          <t xml:space="preserve">พัดลม</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_fan</t>
+          <t xml:space="preserve">home_action_disinfection_quick</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fan</t>
+          <t xml:space="preserve">60 min</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">風量設定</t>
+          <t xml:space="preserve">60分</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">风扇</t>
+          <t xml:space="preserve">60分钟</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">風扇</t>
+          <t xml:space="preserve">60分鐘</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">팬</t>
+          <t xml:space="preserve">60분</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t xml:space="preserve">พัดลม</t>
+          <t xml:space="preserve">60 นาที</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_disinfection_quick</t>
+          <t xml:space="preserve">home_action_disinfection_deep</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quick</t>
+          <t xml:space="preserve">90 min</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">スピード消毒</t>
+          <t xml:space="preserve">90分</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">快速消毒</t>
+          <t xml:space="preserve">90分钟</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">快速消毒</t>
+          <t xml:space="preserve">90分鐘</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">빠르게</t>
+          <t xml:space="preserve">90분</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t xml:space="preserve">ด่วน</t>
+          <t xml:space="preserve">90 นาที</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_disinfection_deep</t>
+          <t xml:space="preserve">scene_title</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deep</t>
+          <t xml:space="preserve">Scene</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">通常消毒</t>
+          <t xml:space="preserve">シーン</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">彻底消毒</t>
+          <t xml:space="preserve">场景</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">徹底消毒</t>
+          <t xml:space="preserve">場景</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">집중</t>
+          <t xml:space="preserve">장면</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve">ลึก</t>
+          <t xml:space="preserve">ฉาก</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_light_white</t>
+          <t xml:space="preserve">scene_action_auto</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">White</t>
+          <t xml:space="preserve">Auto</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">白色</t>
+          <t xml:space="preserve">自動</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">白色</t>
+          <t xml:space="preserve">自动</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">白色</t>
+          <t xml:space="preserve">自動</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">흰색</t>
+          <t xml:space="preserve">자동</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t xml:space="preserve">สีขาว</t>
+          <t xml:space="preserve">อัตโนมัติ</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_light_blue</t>
+          <t xml:space="preserve">home_o3_toast_pause</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blue</t>
+          <t xml:space="preserve">Human/animal detected. Disinfection paused. Resume after cleared.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">青色</t>
+          <t xml:space="preserve">人・動物検知、消毒停止。解除後、再開。</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">蓝色</t>
+          <t xml:space="preserve">检测到人/动物，消毒已暂停。解除后恢复。</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">藍色</t>
+          <t xml:space="preserve">檢測到人/動物，消毒已暫停。解除後恢復。</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">파란색</t>
+          <t xml:space="preserve">사람/동물이 감지되어 살균이 일시 중지되었습니다. 해제 후 재개됩니다.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t xml:space="preserve">สีน้ำเงิน</t>
+          <t xml:space="preserve">ตรวจพบคน/สัตว์ การฆ่าเชื้อถูกหยุดชั่วคราว และจะทำงานต่อเมื่อพื้นที่ปลอดภัย</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_light_green</t>
+          <t xml:space="preserve">home_o3_toast_running</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green</t>
+          <t xml:space="preserve">Disinfecting. Keep people/animals away.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">緑色</t>
+          <t xml:space="preserve">消毒中、人・動物は遠ざけてください。</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">绿色</t>
+          <t xml:space="preserve">消毒中，请远离人/动物。</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">綠色</t>
+          <t xml:space="preserve">消毒中，請遠離人/動物。</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">초록색</t>
+          <t xml:space="preserve">살균 중입니다. 사람/동물은 가까이 오지 마세요.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">สีเขียว</t>
+          <t xml:space="preserve">กำลังฆ่าเชื้อ โปรดอยู่ห่างจากคน/สัตว์</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">scene_title</t>
+          <t xml:space="preserve">home_o3_status_recovery</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scene</t>
+          <t xml:space="preserve">Recovery after emergency stop</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">シーン</t>
+          <t xml:space="preserve">緊急停止後の回復フェーズ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">场景</t>
+          <t xml:space="preserve">紧急停止后的恢复阶段</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">場景</t>
+          <t xml:space="preserve">緊急停止後的恢復階段</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">장면</t>
+          <t xml:space="preserve">긴급 정지 후 복구 단계</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve">ฉาก</t>
+          <t xml:space="preserve">ช่วงฟื้นตัวหลังหยุดฉุกเฉิน</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">scene_action_auto</t>
+          <t xml:space="preserve">home_o3_status_diffuse</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Auto</t>
+          <t xml:space="preserve">Dispersing with strong airflow</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">自動</t>
+          <t xml:space="preserve">オゾン消毒後待機中</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">自动</t>
+          <t xml:space="preserve">强风扩散中</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">自動</t>
+          <t xml:space="preserve">強風擴散中</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">자동</t>
+          <t xml:space="preserve">강한 바람으로 확산 중</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t xml:space="preserve">อัตโนมัติ</t>
+          <t xml:space="preserve">กำลังกระจายด้วยลมแรง</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_toast_pause</t>
+          <t xml:space="preserve">home_o3_status_fan_remaining_minutes</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Human/animal detected. Disinfection paused. Resume after cleared.</t>
+          <t xml:space="preserve">Fan remaining: {0} min</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">人・動物検知、消毒停止。解除後、再開。</t>
+          <t xml:space="preserve">送風の残り時間：{0}分</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">检测到人/动物，消毒已暂停。解除后恢复。</t>
+          <t xml:space="preserve">吹风剩余：{0}分钟</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">檢測到人/動物，消毒已暫停。解除後恢復。</t>
+          <t xml:space="preserve">吹風剩餘：{0}分鐘</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">사람/동물이 감지되어 살균이 일시 중지되었습니다. 해제 후 재개됩니다.</t>
+          <t xml:space="preserve">송풍 남은 시간: {0}분</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t xml:space="preserve">ตรวจพบคน/สัตว์ การฆ่าเชื้อถูกหยุดชั่วคราว และจะทำงานต่อเมื่อพื้นที่ปลอดภัย</t>
+          <t xml:space="preserve">เวลาพัดลมคงเหลือ: {0} นาที</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_toast_running</t>
+          <t xml:space="preserve">home_o3_status_fan_finished</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Disinfecting. Keep people/animals away.</t>
+          <t xml:space="preserve">Fan finished</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">消毒中、人・動物は遠ざけてください。</t>
+          <t xml:space="preserve">送風終了</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">消毒中，请远离人/动物。</t>
+          <t xml:space="preserve">吹风结束</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">消毒中，請遠離人/動物。</t>
+          <t xml:space="preserve">吹風結束</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">살균 중입니다. 사람/동물은 가까이 오지 마세요.</t>
+          <t xml:space="preserve">송풍 종료</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t xml:space="preserve">กำลังฆ่าเชื้อ โปรดอยู่ห่างจากคน/สัตว์</t>
+          <t xml:space="preserve">พัดลมสิ้นสุดแล้ว</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_status_recovery</t>
+          <t xml:space="preserve">disinfection_title</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recovery after emergency stop</t>
+          <t xml:space="preserve">Ozone disinfection</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">緊急停止後の回復フェーズ</t>
+          <t xml:space="preserve">オゾン消毒</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">紧急停止后的恢复阶段</t>
+          <t xml:space="preserve">臭氧消毒</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">緊急停止後的恢復階段</t>
+          <t xml:space="preserve">臭氧消毒</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">긴급 정지 후 복구 단계</t>
+          <t xml:space="preserve">오존 살균</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">ช่วงฟื้นตัวหลังหยุดฉุกเฉิน</t>
+          <t xml:space="preserve">ฆ่าเชื้อด้วยโอโซน</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_status_diffuse</t>
+          <t xml:space="preserve">disinfection_status_paused</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dispersing with strong airflow</t>
+          <t xml:space="preserve">Paused</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">オゾン消毒後待機中</t>
+          <t xml:space="preserve">停止</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">强风扩散中</t>
+          <t xml:space="preserve">已暂停</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">強風擴散中</t>
+          <t xml:space="preserve">已暫停</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">강한 바람으로 확산 중</t>
+          <t xml:space="preserve">일시 중지됨</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">กำลังกระจายด้วยลมแรง</t>
+          <t xml:space="preserve">หยุดชั่วคราว</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_status_fan_remaining_minutes</t>
+          <t xml:space="preserve">disinfection_remaining_minutes</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fan remaining: {0} min</t>
+          <t xml:space="preserve">{0} min remaining</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">送風の残り時間：{0}分</t>
+          <t xml:space="preserve">残り{0}分</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">吹风剩余：{0}分钟</t>
+          <t xml:space="preserve">剩余{0}分钟</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">吹風剩餘：{0}分鐘</t>
+          <t xml:space="preserve">剩餘{0}分鐘</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">송풍 남은 시간: {0}분</t>
+          <t xml:space="preserve">{0}분 남음</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">เวลาพัดลมคงเหลือ: {0} นาที</t>
+          <t xml:space="preserve">เหลืออีก {0} นาที</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_status_fan_finished</t>
+          <t xml:space="preserve">disinfection_note_stopped</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fan finished</t>
+          <t xml:space="preserve">People or animals are still active in the area. Ozone has stopped.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">送風終了</t>
+          <t xml:space="preserve">人や動物の活動が続いているため、オゾンを停止しました。</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">吹风结束</t>
+          <t xml:space="preserve">环境持续有人员活动，臭氧已停止。</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">吹風結束</t>
+          <t xml:space="preserve">環境持續有人員活動，臭氧已停止。</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">송풍 종료</t>
+          <t xml:space="preserve">주변에 사람이나 동물의 움직임이 계속 감지되어 오존이 중지되었습니다.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">พัดลมสิ้นสุดแล้ว</t>
+          <t xml:space="preserve">ยังตรวจพบการเคลื่อนไหวของคนหรือสัตว์ในพื้นที่ โอโซนจึงหยุดทำงาน</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_title</t>
+          <t xml:space="preserve">disinfection_note_paused</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ozone disinfection</t>
+          <t xml:space="preserve">Person or pet detected. Ozone has paused.</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">オゾン消毒</t>
+          <t xml:space="preserve">人やペットを検知したため、オゾンを一時停止しました。</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">臭氧消毒</t>
+          <t xml:space="preserve">检测到人员或宠物，臭氧已暂停。</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">臭氧消毒</t>
+          <t xml:space="preserve">偵測到人員或寵物，臭氧已暫停。</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">오존 살균</t>
+          <t xml:space="preserve">사람 또는 반려동물이 감지되어 오존이 일시 중지되었습니다.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve">ฆ่าเชื้อด้วยโอโซน</t>
+          <t xml:space="preserve">ตรวจพบคนหรือสัตว์เลี้ยง โอโซนจึงหยุดชั่วคราว</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_status_paused</t>
+          <t xml:space="preserve">disinfection_note_running</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paused</t>
+          <t xml:space="preserve">Area is clear. Ozone has restarted.</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">停止</t>
+          <t xml:space="preserve">環境がクリアになったため、オゾンを再起動しました。</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">已暂停</t>
+          <t xml:space="preserve">环境已清空，臭氧重新启动。</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">已暫停</t>
+          <t xml:space="preserve">環境已清空，臭氧重新啟動。</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">일시 중지됨</t>
+          <t xml:space="preserve">주변이 비어 있어 오존이 다시 시작되었습니다.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve">หยุดชั่วคราว</t>
+          <t xml:space="preserve">พื้นที่ปลอดคนแล้ว โอโซนเริ่มทำงานอีกครั้ง</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_remaining_minutes</t>
+          <t xml:space="preserve">disinfection_detected</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">{0} min remaining</t>
+          <t xml:space="preserve">● People/animals detected.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">残り{0}分</t>
+          <t xml:space="preserve">● 人や動物を検知しました。</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">剩余{0}分钟</t>
+          <t xml:space="preserve">● 检测到人/动物。</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">剩餘{0}分鐘</t>
+          <t xml:space="preserve">● 檢測到人/動物。</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">{0}분 남음</t>
+          <t xml:space="preserve">● 사람/동물이 감지되었습니다.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve">เหลืออีก {0} นาที</t>
+          <t xml:space="preserve">● ตรวจพบคน/สัตว์</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_note_stopped</t>
+          <t xml:space="preserve">disinfection_not_detected</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">People or animals are still active in the area. Ozone has stopped.</t>
+          <t xml:space="preserve">● No people/pets detected.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">人や動物の活動が続いているため、オゾンを停止しました。</t>
+          <t xml:space="preserve">● 人や動物は検知されていません</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">环境持续有人员活动，臭氧已停止。</t>
+          <t xml:space="preserve">● 未检测到人/宠物。</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境持續有人員活動，臭氧已停止。</t>
+          <t xml:space="preserve">● 未檢測到人/寵物。</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">주변에 사람이나 동물의 움직임이 계속 감지되어 오존이 중지되었습니다.</t>
+          <t xml:space="preserve">● 사람/반려동물이 감지되지 않았습니다.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">ยังตรวจพบการเคลื่อนไหวของคนหรือสัตว์ในพื้นที่ โอโซนจึงหยุดทำงาน</t>
+          <t xml:space="preserve">● ไม่พบคน/สัตว์เลี้ยง</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_note_paused</t>
+          <t xml:space="preserve">mist_title</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Person or pet detected. Ozone has paused.</t>
+          <t xml:space="preserve">Mist level</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">人やペットを検知したため、オゾンを一時停止しました。</t>
+          <t xml:space="preserve">ミスト設定</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">检测到人员或宠物，臭氧已暂停。</t>
+          <t xml:space="preserve">喷雾量设置</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">偵測到人員或寵物，臭氧已暫停。</t>
+          <t xml:space="preserve">噴霧量設定</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">사람 또는 반려동물이 감지되어 오존이 일시 중지되었습니다.</t>
+          <t xml:space="preserve">미스트 단계</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve">ตรวจพบคนหรือสัตว์เลี้ยง โอโซนจึงหยุดชั่วคราว</t>
+          <t xml:space="preserve">ระดับละอองน้ำ</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_note_running</t>
+          <t xml:space="preserve">mist_nozzle_1</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Area is clear. Ozone has restarted.</t>
+          <t xml:space="preserve">Nozzle 1</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境がクリアになったため、オゾンを再起動しました。</t>
+          <t xml:space="preserve">ミスト1</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">环境已清空，臭氧重新启动。</t>
+          <t xml:space="preserve">喷嘴1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境已清空，臭氧重新啟動。</t>
+          <t xml:space="preserve">噴嘴1</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">주변이 비어 있어 오존이 다시 시작되었습니다.</t>
+          <t xml:space="preserve">노즐 1</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นที่ปลอดคนแล้ว โอโซนเริ่มทำงานอีกครั้ง</t>
+          <t xml:space="preserve">หัวพ่น 1</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_detected</t>
+          <t xml:space="preserve">mist_nozzle_2</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">● People/animals detected.</t>
+          <t xml:space="preserve">Nozzle 2</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 人や動物を検知しました。</t>
+          <t xml:space="preserve">ミスト2</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 检测到人/动物。</t>
+          <t xml:space="preserve">喷嘴2</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 檢測到人/動物。</t>
+          <t xml:space="preserve">噴嘴2</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 사람/동물이 감지되었습니다.</t>
+          <t xml:space="preserve">노즐 2</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve">● ตรวจพบคน/สัตว์</t>
+          <t xml:space="preserve">หัวพ่น 2</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_not_detected</t>
+          <t xml:space="preserve">fan_title</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">● No people/pets detected.</t>
+          <t xml:space="preserve">Fan level</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 人や動物は検知されていません</t>
+          <t xml:space="preserve">風量設定</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 未检测到人/宠物。</t>
+          <t xml:space="preserve">风量设置</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 未檢測到人/寵物。</t>
+          <t xml:space="preserve">風量設定</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 사람/반려동물이 감지되지 않았습니다.</t>
+          <t xml:space="preserve">팬 단계</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">● ไม่พบคน/สัตว์เลี้ยง</t>
+          <t xml:space="preserve">ระดับพัดลม</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">mist_title</t>
+          <t xml:space="preserve">cooling_title</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mist level</t>
+          <t xml:space="preserve">Cooling mode</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミスト設定</t>
+          <t xml:space="preserve">冷房モード</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">喷雾量设置</t>
+          <t xml:space="preserve">制冷模式</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">噴霧量設定</t>
+          <t xml:space="preserve">製冷模式</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">미스트 단계</t>
+          <t xml:space="preserve">냉각 모드</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t xml:space="preserve">ระดับละอองน้ำ</t>
+          <t xml:space="preserve">โหมดทำความเย็น</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">mist_nozzle_1</t>
+          <t xml:space="preserve">cooling_mode_intermittent</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nozzle 1</t>
+          <t xml:space="preserve">Intermittent</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミスト1</t>
+          <t xml:space="preserve">クーリングモード断続</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">喷嘴1</t>
+          <t xml:space="preserve">间歇</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">噴嘴1</t>
+          <t xml:space="preserve">間歇</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t xml:space="preserve">노즐 1</t>
+          <t xml:space="preserve">간헐</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">หัวพ่น 1</t>
+          <t xml:space="preserve">เป็นช่วง</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">mist_nozzle_2</t>
+          <t xml:space="preserve">cooling_mode_continuous</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nozzle 2</t>
+          <t xml:space="preserve">Continuous</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミスト2</t>
+          <t xml:space="preserve">クーリングモード継続</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">喷嘴2</t>
+          <t xml:space="preserve">持续</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">噴嘴2</t>
+          <t xml:space="preserve">持續</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">노즐 2</t>
+          <t xml:space="preserve">연속</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t xml:space="preserve">หัวพ่น 2</t>
+          <t xml:space="preserve">ต่อเนื่อง</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">fan_title</t>
+          <t xml:space="preserve">power_hint_off</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fan level</t>
+          <t xml:space="preserve">≪ Power off</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">風量設定</t>
+          <t xml:space="preserve">≪ 電源を切る</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">风量设置</t>
+          <t xml:space="preserve">≪ 关闭电源</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">風量設定</t>
+          <t xml:space="preserve">≪ 關閉電源</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">팬 단계</t>
+          <t xml:space="preserve">≪ 전원 끄기</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t xml:space="preserve">ระดับพัดลม</t>
+          <t xml:space="preserve">≪ ปิดเครื่อง</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">cooling_title</t>
+          <t xml:space="preserve">power_hint_on</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cooling mode</t>
+          <t xml:space="preserve">Power on ≫</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">冷房モード</t>
+          <t xml:space="preserve">電源を入れる ≫</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">制冷模式</t>
+          <t xml:space="preserve">开启电源 ≫</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">製冷模式</t>
+          <t xml:space="preserve">開啟電源 ≫</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve">냉각 모드</t>
+          <t xml:space="preserve">전원 켜기 ≫</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">โหมดทำความเย็น</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cooling_mode_intermittent</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Intermittent</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">クーリングモード断続</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">间歇</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">間歇</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">간헐</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">เป็นช่วง</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cooling_mode_continuous</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Continuous</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">クーリングモード継続</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">持续</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">持續</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">연속</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ต่อเนื่อง</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">light_title</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Light</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ライト</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">灯光</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">燈光</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">조명</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ไฟ</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">power_hint_off</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">≪ Power off</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">≪ 電源を切る</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">≪ 关闭电源</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">≪ 關閉電源</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">≪ 전원 끄기</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">≪ ปิดเครื่อง</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">power_hint_on</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Power on ≫</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">電源を入れる ≫</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">开启电源 ≫</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">開啟電源 ≫</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">전원 켜기 ≫</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
         <is>
           <t xml:space="preserve">เปิดเครื่อง ≫</t>
         </is>

</xml_diff>

<commit_message>
feat(i18n): localize smart bottle maker panel strings
Replace the legacy fan panel copy with bottle maker strings for home,
making flows, powder brand management, and baby diary integration.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/i18n_export.xlsx
+++ b/i18n_export.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -67,22 +67,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">关闭</t>
+          <t xml:space="preserve">OFF</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">關閉</t>
+          <t xml:space="preserve">OFF</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">끄기</t>
+          <t xml:space="preserve">OFF</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ปิด</t>
+          <t xml:space="preserve">OFF</t>
         </is>
       </c>
     </row>
@@ -114,12 +114,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">닫기</t>
+          <t xml:space="preserve">Close</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ปิด</t>
+          <t xml:space="preserve">Close</t>
         </is>
       </c>
     </row>
@@ -151,1640 +151,4353 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">창 닫기</t>
+          <t xml:space="preserve">Close window</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ปิดหน้าต่าง</t>
+          <t xml:space="preserve">Close window</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">onboarding_step_title</t>
+          <t xml:space="preserve">common_cancel</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Setup</t>
+          <t xml:space="preserve">Cancel</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">セットアップ中</t>
+          <t xml:space="preserve">キャンセル</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">准备工作</t>
+          <t xml:space="preserve">取消</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">準備工作</t>
+          <t xml:space="preserve">取消</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">설정</t>
+          <t xml:space="preserve">Cancel</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">ตั้งค่า</t>
+          <t xml:space="preserve">Cancel</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">onboarding_step_desc</t>
+          <t xml:space="preserve">common_confirm</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Before we start, please tell us your pet type.</t>
+          <t xml:space="preserve">Confirm</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">開始する前に、まずペットの種類を教えてください。</t>
+          <t xml:space="preserve">確認</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">开始前，请先告诉我们宠物的种类。</t>
+          <t xml:space="preserve">确认</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">開始前，請先告訴我們寵物的種類。</t>
+          <t xml:space="preserve">確認</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">시작하기 전에 반려동물 종류를 알려주세요.</t>
+          <t xml:space="preserve">Confirm</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">ก่อนเริ่ม โปรดบอกประเภทสัตว์เลี้ยงของคุณ</t>
+          <t xml:space="preserve">Confirm</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">onboarding_start</t>
+          <t xml:space="preserve">common_yes</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Start</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">開始</t>
+          <t xml:space="preserve">はい</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">开始</t>
+          <t xml:space="preserve">是</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">開始</t>
+          <t xml:space="preserve">是</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">시작</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">เริ่ม</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">pet_dog</t>
+          <t xml:space="preserve">common_save</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dog</t>
+          <t xml:space="preserve">Save</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">犬</t>
+          <t xml:space="preserve">保存</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">狗</t>
+          <t xml:space="preserve">保存</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">狗</t>
+          <t xml:space="preserve">儲存</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">강아지</t>
+          <t xml:space="preserve">Save</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">สุนัข</t>
+          <t xml:space="preserve">Save</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">pet_cat</t>
+          <t xml:space="preserve">custom_mode_title</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cat</t>
+          <t xml:space="preserve">Custom Mode Settings</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">猫</t>
+          <t xml:space="preserve">カスタムモード設定</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">猫</t>
+          <t xml:space="preserve">自定义模式设置</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">貓</t>
+          <t xml:space="preserve">自訂模式設定</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">고양이</t>
+          <t xml:space="preserve">Custom Mode Settings</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">แมว</t>
+          <t xml:space="preserve">Custom Mode Settings</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">pet_other</t>
+          <t xml:space="preserve">custom_mode_note</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other</t>
+          <t xml:space="preserve">Note: The machine will mix milk powder according to your preset powder-to-water ratio. The final volume of the milk will be slightly higher than the set water output.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">その他</t>
+          <t xml:space="preserve">注：機器は設定した粉水比でミルクパウダーを調合します。完成したミルクの量は、設定した出水量よりやや多くなります。</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">其他</t>
+          <t xml:space="preserve">说明：设备将按您预设的粉水比冲调奶粉，成品奶量会略高于设定出水量。</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">其他</t>
+          <t xml:space="preserve">說明：設備將依您預設的粉水比沖調奶粉，成品奶量會略高於設定出水量。</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">기타</t>
+          <t xml:space="preserve">Note: The machine will mix milk powder according to your preset powder-to-water ratio. The final volume of the milk will be slightly higher than the set water output.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">อื่นๆ</t>
+          <t xml:space="preserve">Note: The machine will mix milk powder according to your preset powder-to-water ratio. The final volume of the milk will be slightly higher than the set water output.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_nav_change_pet</t>
+          <t xml:space="preserve">custom_mode_water</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Change pet</t>
+          <t xml:space="preserve">Water</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">ペット変更</t>
+          <t xml:space="preserve">水</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">更换宠物</t>
+          <t xml:space="preserve">水量</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">更換寵物</t>
+          <t xml:space="preserve">水量</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">반려동물 변경</t>
+          <t xml:space="preserve">Water</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">เปลี่ยนสัตว์เลี้ยง</t>
+          <t xml:space="preserve">Water</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_status_temperature</t>
+          <t xml:space="preserve">custom_mode_powder</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Temperature</t>
+          <t xml:space="preserve">Powder</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">気温</t>
+          <t xml:space="preserve">粉ミルク</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">温度</t>
+          <t xml:space="preserve">奶粉</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">溫度</t>
+          <t xml:space="preserve">奶粉</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">온도</t>
+          <t xml:space="preserve">Powder</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">อุณหภูมิ</t>
+          <t xml:space="preserve">Powder</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_status_humidity</t>
+          <t xml:space="preserve">custom_mode_temperature</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Humidity</t>
+          <t xml:space="preserve">Temperature</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">湿度</t>
+          <t xml:space="preserve">温度</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">湿度</t>
+          <t xml:space="preserve">温度</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">濕度</t>
+          <t xml:space="preserve">溫度</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">습도</t>
+          <t xml:space="preserve">Temperature</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">ความชื้น</t>
+          <t xml:space="preserve">Temperature</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_status_device</t>
+          <t xml:space="preserve">app_title</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Device status</t>
+          <t xml:space="preserve">SMART BOTTLER MAKER</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">デバイス検出</t>
+          <t xml:space="preserve">SMART BOTTLER MAKER</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">设备状态</t>
+          <t xml:space="preserve">SMART BOTTLER MAKER</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">設備狀態</t>
+          <t xml:space="preserve">SMART BOTTLER MAKER</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">기기 상태</t>
+          <t xml:space="preserve">SMART BOTTLER MAKER</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve">สถานะอุปกรณ์</t>
+          <t xml:space="preserve">SMART BOTTLER MAKER</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_temperature_good</t>
+          <t xml:space="preserve">status_online</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comfortable</t>
+          <t xml:space="preserve">Online</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境が良い</t>
+          <t xml:space="preserve">オンライン</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">环境良好</t>
+          <t xml:space="preserve">在线</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境良好</t>
+          <t xml:space="preserve">在線</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">쾌적함</t>
+          <t xml:space="preserve">Online</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">สบาย</t>
+          <t xml:space="preserve">Online</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_temperature_high</t>
+          <t xml:space="preserve">status_offline</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hot</t>
+          <t xml:space="preserve">Offline</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">高温</t>
+          <t xml:space="preserve">オフライン</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">高温</t>
+          <t xml:space="preserve">离线</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">高溫</t>
+          <t xml:space="preserve">離線</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">더움</t>
+          <t xml:space="preserve">Offline</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve">ร้อน</t>
+          <t xml:space="preserve">Offline</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_temperature_low</t>
+          <t xml:space="preserve">status_connecting</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cold</t>
+          <t xml:space="preserve">Connecting</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">寒い</t>
+          <t xml:space="preserve">接続中</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">寒冷</t>
+          <t xml:space="preserve">连接中</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">寒冷</t>
+          <t xml:space="preserve">連線中</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">추움</t>
+          <t xml:space="preserve">Connecting</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t xml:space="preserve">หนาว</t>
+          <t xml:space="preserve">Connecting</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_tab_climate</t>
+          <t xml:space="preserve">gauge_water_amount</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Climate</t>
+          <t xml:space="preserve">WATER AMOUNT</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミストファン</t>
+          <t xml:space="preserve">水量</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">温湿度管理</t>
+          <t xml:space="preserve">水量</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">溫濕度管理</t>
+          <t xml:space="preserve">水量</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">기후</t>
+          <t xml:space="preserve">WATER AMOUNT</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">สภาพอากาศ</t>
+          <t xml:space="preserve">WATER AMOUNT</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_tab_disinfection</t>
+          <t xml:space="preserve">gauge_powder_amount</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Disinfection</t>
+          <t xml:space="preserve">MILK POWDER AMOUNT</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">消毒</t>
+          <t xml:space="preserve">ミルクパウダー量</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">消毒</t>
+          <t xml:space="preserve">奶粉量</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">消毒</t>
+          <t xml:space="preserve">奶粉量</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">살균</t>
+          <t xml:space="preserve">MILK POWDER AMOUNT</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ฆ่าเชื้อ</t>
+          <t xml:space="preserve">MILK POWDER AMOUNT</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_mist</t>
+          <t xml:space="preserve">metric_water</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mist</t>
+          <t xml:space="preserve">WATER</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミスト</t>
+          <t xml:space="preserve">水</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">喷雾</t>
+          <t xml:space="preserve">水</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">噴霧</t>
+          <t xml:space="preserve">水</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">미스트</t>
+          <t xml:space="preserve">WATER</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t xml:space="preserve">ละอองน้ำ</t>
+          <t xml:space="preserve">WATER</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_fan</t>
+          <t xml:space="preserve">metric_powder</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fan</t>
+          <t xml:space="preserve">POWDER</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">風量設定</t>
+          <t xml:space="preserve">粉ミルク</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">风扇</t>
+          <t xml:space="preserve">奶粉</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">風扇</t>
+          <t xml:space="preserve">奶粉</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">팬</t>
+          <t xml:space="preserve">POWDER</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t xml:space="preserve">พัดลม</t>
+          <t xml:space="preserve">POWDER</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_disinfection_quick</t>
+          <t xml:space="preserve">metric_temp</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">60 min</t>
+          <t xml:space="preserve">TEMP</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">60分</t>
+          <t xml:space="preserve">温度</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">60分钟</t>
+          <t xml:space="preserve">温度</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">60分鐘</t>
+          <t xml:space="preserve">溫度</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">60분</t>
+          <t xml:space="preserve">TEMP</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t xml:space="preserve">60 นาที</t>
+          <t xml:space="preserve">TEMP</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_action_disinfection_deep</t>
+          <t xml:space="preserve">metric_stir</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">90 min</t>
+          <t xml:space="preserve">STIR</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">90分</t>
+          <t xml:space="preserve">攪拌</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">90分钟</t>
+          <t xml:space="preserve">搅拌</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">90分鐘</t>
+          <t xml:space="preserve">攪拌</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">90분</t>
+          <t xml:space="preserve">STIR</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t xml:space="preserve">90 นาที</t>
+          <t xml:space="preserve">STIR</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">scene_title</t>
+          <t xml:space="preserve">metric_stir_level</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scene</t>
+          <t xml:space="preserve">Lv.{0}</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">シーン</t>
+          <t xml:space="preserve">Lv.{0}</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">场景</t>
+          <t xml:space="preserve">Lv.{0}</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">場景</t>
+          <t xml:space="preserve">Lv.{0}</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">장면</t>
+          <t xml:space="preserve">Lv.{0}</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve">ฉาก</t>
+          <t xml:space="preserve">Lv.{0}</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">scene_action_auto</t>
+          <t xml:space="preserve">metric_edit</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Auto</t>
+          <t xml:space="preserve">Edit</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">自動</t>
+          <t xml:space="preserve">編集</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">自动</t>
+          <t xml:space="preserve">编辑</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">自動</t>
+          <t xml:space="preserve">編輯</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">자동</t>
+          <t xml:space="preserve">Edit</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t xml:space="preserve">อัตโนมัติ</t>
+          <t xml:space="preserve">Edit</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_toast_pause</t>
+          <t xml:space="preserve">warn_set_brand</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Human/animal detected. Disinfection paused. Resume after cleared.</t>
+          <t xml:space="preserve">Please set a milk powder brand and ratio.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">人・動物検知、消毒停止。解除後、再開。</t>
+          <t xml:space="preserve">粉ミルクブランドと比率を設定してください。</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">检测到人/动物，消毒已暂停。解除后恢复。</t>
+          <t xml:space="preserve">请设置奶粉品牌与配比。</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">檢測到人/動物，消毒已暫停。解除後恢復。</t>
+          <t xml:space="preserve">請設定奶粉品牌與配比。</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">사람/동물이 감지되어 살균이 일시 중지되었습니다. 해제 후 재개됩니다.</t>
+          <t xml:space="preserve">Please set a milk powder brand and ratio.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t xml:space="preserve">ตรวจพบคน/สัตว์ การฆ่าเชื้อถูกหยุดชั่วคราว และจะทำงานต่อเมื่อพื้นที่ปลอดภัย</t>
+          <t xml:space="preserve">Please set a milk powder brand and ratio.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_toast_running</t>
+          <t xml:space="preserve">brand_banner_intro</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Disinfecting. Keep people/animals away.</t>
+          <t xml:space="preserve">Let's mix every formula brand the smart way.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">消毒中、人・動物は遠ざけてください。</t>
+          <t xml:space="preserve">すべてのフォーミュラブランドをスマートにミックスしましょう。</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">消毒中，请远离人/动物。</t>
+          <t xml:space="preserve">智能调配每一款配方奶粉。</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">消毒中，請遠離人/動物。</t>
+          <t xml:space="preserve">智慧調配每一款配方奶粉。</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">살균 중입니다. 사람/동물은 가까이 오지 마세요.</t>
+          <t xml:space="preserve">Let's mix every formula brand the smart way.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">กำลังฆ่าเชื้อ โปรดอยู่ห่างจากคน/สัตว์</t>
+          <t xml:space="preserve">Let's mix every formula brand the smart way.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_status_recovery</t>
+          <t xml:space="preserve">brand_row_hint</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recovery after emergency stop</t>
+          <t xml:space="preserve">Please set a milk powder brand.</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">緊急停止後の回復フェーズ</t>
+          <t xml:space="preserve">粉ミルクブランドを設定してください。</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">紧急停止后的恢复阶段</t>
+          <t xml:space="preserve">请设置奶粉品牌。</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">緊急停止後的恢復階段</t>
+          <t xml:space="preserve">請設定奶粉品牌。</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">긴급 정지 후 복구 단계</t>
+          <t xml:space="preserve">Please set a milk powder brand.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve">ช่วงฟื้นตัวหลังหยุดฉุกเฉิน</t>
+          <t xml:space="preserve">Please set a milk powder brand.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_status_diffuse</t>
+          <t xml:space="preserve">brand_row_custom_ratio</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dispersing with strong airflow</t>
+          <t xml:space="preserve">Custom Mixing Ratio: {0}ml / {1}g</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">オゾン消毒後待機中</t>
+          <t xml:space="preserve">カスタムミックス比率: {0}ml / {1}g</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">强风扩散中</t>
+          <t xml:space="preserve">自定义配比: {0}ml / {1}g</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">強風擴散中</t>
+          <t xml:space="preserve">自訂配比: {0}ml / {1}g</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">강한 바람으로 확산 중</t>
+          <t xml:space="preserve">Custom Mixing Ratio: {0}ml / {1}g</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t xml:space="preserve">กำลังกระจายด้วยลมแรง</t>
+          <t xml:space="preserve">Custom Mixing Ratio: {0}ml / {1}g</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_status_fan_remaining_minutes</t>
+          <t xml:space="preserve">brand_row_brand_summary</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fan remaining: {0} min</t>
+          <t xml:space="preserve">{0} / {1} / {2}</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">送風の残り時間：{0}分</t>
+          <t xml:space="preserve">{0} / {1} / {2}</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">吹风剩余：{0}分钟</t>
+          <t xml:space="preserve">{0} / {1} / {2}</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">吹風剩餘：{0}分鐘</t>
+          <t xml:space="preserve">{0} / {1} / {2}</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">송풍 남은 시간: {0}분</t>
+          <t xml:space="preserve">{0} / {1} / {2}</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t xml:space="preserve">เวลาพัดลมคงเหลือ: {0} นาที</t>
+          <t xml:space="preserve">{0} / {1} / {2}</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">home_o3_status_fan_finished</t>
+          <t xml:space="preserve">mode_standard</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fan finished</t>
+          <t xml:space="preserve">Standard</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">送風終了</t>
+          <t xml:space="preserve">標準</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">吹风结束</t>
+          <t xml:space="preserve">标准</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">吹風結束</t>
+          <t xml:space="preserve">標準</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">송풍 종료</t>
+          <t xml:space="preserve">Standard</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t xml:space="preserve">พัดลมสิ้นสุดแล้ว</t>
+          <t xml:space="preserve">Standard</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_title</t>
+          <t xml:space="preserve">mode_nighttime</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ozone disinfection</t>
+          <t xml:space="preserve">Nighttime</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">オゾン消毒</t>
+          <t xml:space="preserve">夜間</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">臭氧消毒</t>
+          <t xml:space="preserve">夜间</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">臭氧消毒</t>
+          <t xml:space="preserve">夜間</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">오존 살균</t>
+          <t xml:space="preserve">Nighttime</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">ฆ่าเชื้อด้วยโอโซน</t>
+          <t xml:space="preserve">Nighttime</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_status_paused</t>
+          <t xml:space="preserve">mode_go_out</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paused</t>
+          <t xml:space="preserve">Go Out</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">停止</t>
+          <t xml:space="preserve">お出かけ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">已暂停</t>
+          <t xml:space="preserve">外出</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">已暫停</t>
+          <t xml:space="preserve">外出</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">일시 중지됨</t>
+          <t xml:space="preserve">Go Out</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">หยุดชั่วคราว</t>
+          <t xml:space="preserve">Go Out</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_remaining_minutes</t>
+          <t xml:space="preserve">mode_double</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">{0} min remaining</t>
+          <t xml:space="preserve">Double</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">残り{0}分</t>
+          <t xml:space="preserve">二度盛り</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">剩余{0}分钟</t>
+          <t xml:space="preserve">双倍</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">剩餘{0}分鐘</t>
+          <t xml:space="preserve">雙倍</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">{0}분 남음</t>
+          <t xml:space="preserve">Double</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">เหลืออีก {0} นาที</t>
+          <t xml:space="preserve">Double</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_note_stopped</t>
+          <t xml:space="preserve">mode_custom</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">People or animals are still active in the area. Ozone has stopped.</t>
+          <t xml:space="preserve">Custom</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">人や動物の活動が続いているため、オゾンを停止しました。</t>
+          <t xml:space="preserve">カスタム</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">环境持续有人员活动，臭氧已停止。</t>
+          <t xml:space="preserve">自定义</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境持續有人員活動，臭氧已停止。</t>
+          <t xml:space="preserve">自訂</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">주변에 사람이나 동물의 움직임이 계속 감지되어 오존이 중지되었습니다.</t>
+          <t xml:space="preserve">Custom</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">ยังตรวจพบการเคลื่อนไหวของคนหรือสัตว์ในพื้นที่ โอโซนจึงหยุดทำงาน</t>
+          <t xml:space="preserve">Custom</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_note_paused</t>
+          <t xml:space="preserve">action_water_only</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Person or pet detected. Ozone has paused.</t>
+          <t xml:space="preserve">Water Only</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">人やペットを検知したため、オゾンを一時停止しました。</t>
+          <t xml:space="preserve">水のみ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">检测到人员或宠物，臭氧已暂停。</t>
+          <t xml:space="preserve">仅出水</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">偵測到人員或寵物，臭氧已暫停。</t>
+          <t xml:space="preserve">僅出水</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">사람 또는 반려동물이 감지되어 오존이 일시 중지되었습니다.</t>
+          <t xml:space="preserve">Water Only</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve">ตรวจพบคนหรือสัตว์เลี้ยง โอโซนจึงหยุดชั่วคราว</t>
+          <t xml:space="preserve">Water Only</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_note_running</t>
+          <t xml:space="preserve">action_powder_only</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Area is clear. Ozone has restarted.</t>
+          <t xml:space="preserve">Powder Only</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境がクリアになったため、オゾンを再起動しました。</t>
+          <t xml:space="preserve">粉のみ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">环境已清空，臭氧重新启动。</t>
+          <t xml:space="preserve">仅出粉</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">環境已清空，臭氧重新啟動。</t>
+          <t xml:space="preserve">僅出粉</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">주변이 비어 있어 오존이 다시 시작되었습니다.</t>
+          <t xml:space="preserve">Powder Only</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นที่ปลอดคนแล้ว โอโซนเริ่มทำงานอีกครั้ง</t>
+          <t xml:space="preserve">Powder Only</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_detected</t>
+          <t xml:space="preserve">action_start</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">● People/animals detected.</t>
+          <t xml:space="preserve">Start</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 人や動物を検知しました。</t>
+          <t xml:space="preserve">開始</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 检测到人/动物。</t>
+          <t xml:space="preserve">开始</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 檢測到人/動物。</t>
+          <t xml:space="preserve">開始</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 사람/동물이 감지되었습니다.</t>
+          <t xml:space="preserve">Start</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve">● ตรวจพบคน/สัตว์</t>
+          <t xml:space="preserve">Start</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">disinfection_not_detected</t>
+          <t xml:space="preserve">action_stop</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">● No people/pets detected.</t>
+          <t xml:space="preserve">STOP MAKING</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 人や動物は検知されていません</t>
+          <t xml:space="preserve">停止</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 未检测到人/宠物。</t>
+          <t xml:space="preserve">停止冲奶</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 未檢測到人/寵物。</t>
+          <t xml:space="preserve">停止沖奶</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">● 사람/반려동물이 감지되지 않았습니다.</t>
+          <t xml:space="preserve">STOP MAKING</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">● ไม่พบคน/สัตว์เลี้ยง</t>
+          <t xml:space="preserve">STOP MAKING</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">mist_title</t>
+          <t xml:space="preserve">row_high_temp_clean</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mist level</t>
+          <t xml:space="preserve">High-Temp Clean</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミスト設定</t>
+          <t xml:space="preserve">高温洗浄</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">喷雾量设置</t>
+          <t xml:space="preserve">高温清洁</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">噴霧量設定</t>
+          <t xml:space="preserve">高溫清潔</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">미스트 단계</t>
+          <t xml:space="preserve">High-Temp Clean</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve">ระดับละอองน้ำ</t>
+          <t xml:space="preserve">High-Temp Clean</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">mist_nozzle_1</t>
+          <t xml:space="preserve">high_temp_cleaning</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nozzle 1</t>
+          <t xml:space="preserve">High-Temp Cleaning...</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミスト1</t>
+          <t xml:space="preserve">高温洗浄中...</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">喷嘴1</t>
+          <t xml:space="preserve">高温清洁中...</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">噴嘴1</t>
+          <t xml:space="preserve">高溫清潔中...</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">노즐 1</t>
+          <t xml:space="preserve">High-Temp Cleaning...</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">หัวพ่น 1</t>
+          <t xml:space="preserve">High-Temp Cleaning...</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">mist_nozzle_2</t>
+          <t xml:space="preserve">clean_milk_on_hold</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nozzle 2</t>
+          <t xml:space="preserve">Milk mixing is on hold for now!</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミスト2</t>
+          <t xml:space="preserve">調乳は一時停止中です。</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">喷嘴2</t>
+          <t xml:space="preserve">冲奶已暂时暂停。</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">噴嘴2</t>
+          <t xml:space="preserve">沖奶已暫時暫停。</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">노즐 2</t>
+          <t xml:space="preserve">Milk mixing is on hold for now!</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve">หัวพ่น 2</t>
+          <t xml:space="preserve">Milk mixing is on hold for now!</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">fan_title</t>
+          <t xml:space="preserve">row_child_lock</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fan level</t>
+          <t xml:space="preserve">Child Lock</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">風量設定</t>
+          <t xml:space="preserve">チャイルドロック</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">风量设置</t>
+          <t xml:space="preserve">童锁</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">風量設定</t>
+          <t xml:space="preserve">童鎖</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">팬 단계</t>
+          <t xml:space="preserve">Child Lock</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">ระดับพัดลม</t>
+          <t xml:space="preserve">Child Lock</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">cooling_title</t>
+          <t xml:space="preserve">child_lock_on</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cooling mode</t>
+          <t xml:space="preserve">On</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">冷房モード</t>
+          <t xml:space="preserve">オン</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">制冷模式</t>
+          <t xml:space="preserve">开</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">製冷模式</t>
+          <t xml:space="preserve">開</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">냉각 모드</t>
+          <t xml:space="preserve">On</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t xml:space="preserve">โหมดทำความเย็น</t>
+          <t xml:space="preserve">On</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">cooling_mode_intermittent</t>
+          <t xml:space="preserve">child_lock_off</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Intermittent</t>
+          <t xml:space="preserve">Off</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">クーリングモード断続</t>
+          <t xml:space="preserve">オフ</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">间歇</t>
+          <t xml:space="preserve">关</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">間歇</t>
+          <t xml:space="preserve">關</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t xml:space="preserve">간헐</t>
+          <t xml:space="preserve">Off</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">เป็นช่วง</t>
+          <t xml:space="preserve">Off</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">cooling_mode_continuous</t>
+          <t xml:space="preserve">making_progress</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Continuous</t>
+          <t xml:space="preserve">Making in {0} mode...</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">クーリングモード継続</t>
+          <t xml:space="preserve">{0}モードで調乳中...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">持续</t>
+          <t xml:space="preserve">正在{0}模式冲奶...</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">持續</t>
+          <t xml:space="preserve">正在{0}模式沖奶...</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">연속</t>
+          <t xml:space="preserve">Making in {0} mode...</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t xml:space="preserve">ต่อเนื่อง</t>
+          <t xml:space="preserve">Making in {0} mode...</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">power_hint_off</t>
+          <t xml:space="preserve">making_leave_hint</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">≪ Power off</t>
+          <t xml:space="preserve">Making magic! Please leave the bottle be!</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">≪ 電源を切る</t>
+          <t xml:space="preserve">調乳中です。哺乳瓶に触れないでください。</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">≪ 关闭电源</t>
+          <t xml:space="preserve">正在冲奶，请勿移动奶瓶。</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">≪ 關閉電源</t>
+          <t xml:space="preserve">正在沖奶，請勿移動奶瓶。</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">≪ 전원 끄기</t>
+          <t xml:space="preserve">Making magic! Please leave the bottle be!</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t xml:space="preserve">≪ ปิดเครื่อง</t>
+          <t xml:space="preserve">Making magic! Please leave the bottle be!</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">power_hint_on</t>
+          <t xml:space="preserve">action_stop_making</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Power on ≫</t>
+          <t xml:space="preserve">Stop Making</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">電源を入れる ≫</t>
+          <t xml:space="preserve">停止</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">开启电源 ≫</t>
+          <t xml:space="preserve">停止冲奶</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">開啟電源 ≫</t>
+          <t xml:space="preserve">停止沖奶</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve">전원 켜기 ≫</t>
+          <t xml:space="preserve">Stop Making</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t xml:space="preserve">เปิดเครื่อง ≫</t>
+          <t xml:space="preserve">Stop Making</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bottle_made</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bottle Made!</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">調乳完了！</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">冲奶完成！</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">沖奶完成！</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bottle Made!</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bottle Made!</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">water_temperature_label</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temperature</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">温度</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">温度</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">溫度</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temperature</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temperature</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">water_dispensing</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dispensing Water...</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">給水中...</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">出水中...</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">出水中...</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dispensing Water...</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dispensing Water...</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">action_stop_water</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop Water</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">給水停止</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">停止出水</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">停止出水</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop Water</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop Water</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">water_dispensed</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water Dispensed</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">給水完了</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">出水完成</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">出水完成</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water Dispensed</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water Dispensed</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_dispensing</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dispensing Powder...</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">出粉中...</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">出粉中...</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">出粉中...</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dispensing Powder...</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dispensing Powder...</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">action_stop_powder</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop Powder</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">出粉停止</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">停止出粉</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">停止出粉</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop Powder</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop Powder</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_dispensed</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Powder Dispensed</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">出粉完了</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">出粉完成</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">出粉完成</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Powder Dispensed</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Powder Dispensed</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_dispense_caution</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Caution: Do not open the formula container during powder dispensing.</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注意：出粉中はフォーミュラ容器を開けないでください。</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注意：出粉过程中请勿打开奶粉罐。</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注意：出粉過程中請勿打開奶粉罐。</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Caution: Do not open the formula container during powder dispensing.</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Caution: Do not open the formula container during powder dispensing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">snackbar_diary</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feeding record added to Baby Diary.</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">授乳記録をベビーダイアリーに追加しました</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">喂养记录已添加到宝宝日记</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">餵養記錄已新增至寶寶日記</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feeding record added to Baby Diary.</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feeding record added to Baby Diary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">baby_diary_pid_missing</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baby Diary product ID is not configured. Set BABY_DIARY_VIRTUAL_PID.</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ベビーダイアリーの製品 ID が未設定です。BABY_DIARY_VIRTUAL_PID を設定してください。</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未配置宝宝日记产品 ID，请设置 BABY_DIARY_VIRTUAL_PID。</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未設定寶寶日記產品 ID，請設定 BABY_DIARY_VIRTUAL_PID。</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baby Diary product ID is not configured. Set BABY_DIARY_VIRTUAL_PID.</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baby Diary product ID is not configured. Set BABY_DIARY_VIRTUAL_PID.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">baby_diary_open_failed</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Could not open Baby Diary.</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ベビーダイアリーを開けませんでした。</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">无法打开宝宝日记。</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">無法開啟寶寶日記。</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Could not open Baby Diary.</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Could not open Baby Diary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">volume_modal_title</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water amount</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水量設定</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水量设置</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水量設定</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water amount</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">temp_modal_title</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temperature</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">温度設定</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">温度设置</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">溫度設定</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temperature</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temperature</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feed_request_title</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baby may be hungry</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">お腹がすいているかもしれません</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">宝宝可能饿了</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">寶寶可能餓了</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baby may be hungry</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baby may be hungry</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feed_request_body</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A feeding scene was detected. Confirm parameters and start making?</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">授乳シーンを検知しました。パラメータを確認して調乳を開始しますか？</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">检测到喂养场景，请确认参数并开始冲奶？</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">偵測到餵養場景，請確認參數並開始沖奶？</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A feeding scene was detected. Confirm parameters and start making?</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A feeding scene was detected. Confirm parameters and start making?</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">feed_request_start</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Start making</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">調乳を開始</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">开始冲奶</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">開始沖奶</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Start making</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Start making</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">block_none</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">block_water_tank_missing</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water tank is not installed.</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水箱が装着されていません。</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水箱未安装。</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水箱未安裝。</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water tank is not installed.</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water tank is not installed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">block_low_water</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water level is too low.</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水量が不足しています。</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水量不足。</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水量不足。</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water level is too low.</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water level is too low.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">block_powder_box_missing</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Powder box is not installed.</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">粉ミルクボックスが装着されていません。</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">奶粉盒未安装。</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">奶粉盒未安裝。</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Powder box is not installed.</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Powder box is not installed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">block_funnel_missing</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Funnel is not installed.</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ファネルが装着されていません。</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">漏斗未安装。</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">漏斗未安裝。</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Funnel is not installed.</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Funnel is not installed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">block_bottle_missing</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bottle is not in place.</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">哺乳瓶がセットされていません。</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">奶瓶未就位。</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">奶瓶未就位。</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bottle is not in place.</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bottle is not in place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">block_hot_alert</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Device is too hot. Please wait.</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">本体が高温です。しばらくお待ちください。</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">设备温度过高，请稍候。</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">設備溫度過高，請稍候。</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Device is too hot. Please wait.</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Device is too hot. Please wait.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">error_none</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">error_hot</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High temperature alert</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High temperature alert</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High temperature alert</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High temperature alert</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High temperature alert</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High temperature alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">error_e01</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error E01</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error E01</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error E01</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error E01</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error E01</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error E01</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">error_e02</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error E02</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error E02</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error E02</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error E02</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error E02</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error E02</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">error_c01</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error C01</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error C01</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error C01</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error C01</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error C01</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error C01</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">error_c02</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error C02</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error C02</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error C02</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error C02</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error C02</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error C02</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">brand_coming_soon</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brand settings will be available in a future update.</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ブランド設定は今後のアップデートで提供予定です。</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品牌设置将在后续版本中提供。</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品牌設定將在後續版本中提供。</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brand settings will be available in a future update.</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brand settings will be available in a future update.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_page_title</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add Milk Powder Brand</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">粉ミルクブランドを追加</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">添加奶粉品牌</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">新增奶粉品牌</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add Milk Powder Brand</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add Milk Powder Brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_edit_page_title</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edit Milk Powder Brand</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">粉ミルクブランドを編集</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">编辑奶粉品牌</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">編輯奶粉品牌</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edit Milk Powder Brand</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edit Milk Powder Brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_custom_ratio_section</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Custom Ratio</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">カスタム比率</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">自定义配比</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">自訂配比</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Custom Ratio</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Custom Ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_page_note</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注意：ブランド・シリーズ・段階を選択すると、対応する粉ミルク濃度を自動取得し、調乳比率を表示します。</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">说明：选择品牌、系列和段数后，将自动获取对应奶粉浓度并计算、展示冲调比例。</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">說明：選擇品牌、系列與段數後，將自動取得對應奶粉濃度並計算、顯示沖調比例。</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_info_title</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Milk Powder Info</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">粉ミルク情報</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">奶粉信息</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">奶粉資訊</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Milk Powder Info</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Milk Powder Info</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_select_brand</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brand</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ブランド</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品牌</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">品牌</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brand</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_select_series</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Series</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">シリーズ</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">系列</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">系列</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Series</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Series</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_select_stage</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stage</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">段階</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">段数</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">段數</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stage</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stage</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_select_placeholder</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Select</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">選択</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">请选择</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">請選擇</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Select</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Select</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_sheet_select_brand</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Select Brand</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ブランドを選択</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">选择品牌</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">選擇品牌</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Select Brand</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Select Brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_sheet_select_series</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Select Series</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">シリーズを選択</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">选择系列</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">選擇系列</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Select Series</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Select Series</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_sheet_select_stage</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Select Stage</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">段階を選択</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">选择段数</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">選擇段數</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Select Stage</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Select Stage</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_search_placeholder</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Search brand...</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ブランドを検索...</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">搜索品牌...</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">搜尋品牌...</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Search brand...</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Search brand...</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_search_empty</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No brands match your search.</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">該当するブランドがありません。</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未找到匹配的品牌。</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">找不到符合的品牌。</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No brands match your search.</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No brands match your search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_not_listed</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brand not listed? </t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ブランドが見つかりませんか？ </t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">没有您的品牌？ </t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">找不到您的品牌？ </t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brand not listed? </t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brand not listed? </t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_customize_ratio</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customize mixing ratio.</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ミックス比率をカスタマイズ</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">自定义配比</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">自訂配比</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customize mixing ratio.</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customize mixing ratio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_custom_label</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Custom</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">カスタム</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">自定义</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">自訂</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Custom</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Custom</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_custom_water_ml</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water (mL)</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水量 (mL)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水量 (mL)</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水量 (mL)</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water (mL)</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water (mL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_custom_powder_g</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Powder (g)</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">粉量 (g)</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">粉量 (g)</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">粉量 (g)</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Powder (g)</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Powder (g)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_custom_apply</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Apply</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">適用</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">应用</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">套用</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Apply</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Apply</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_ratio_title</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recommended Mix Ratio</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">推奨ミックス比率</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">推荐配比</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">建議配比</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recommended Mix Ratio</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recommended Mix Ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_ratio_water</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Water</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_ratio_powder</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Powder</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">粉ミルク</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">奶粉</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">奶粉</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Powder</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Powder</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_settings_title</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Powder Brand Settings</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">粉ミルクブランド設定</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">奶粉品牌设置</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">奶粉品牌設定</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Powder Brand Settings</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Powder Brand Settings</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_add_brand</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add Brand</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ブランドを追加</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">添加品牌</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">新增品牌</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add Brand</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add Brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_empty_message</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No milk powder brands added yet.</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">粉ミルクブランドはまだ追加されていません。</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">尚未添加奶粉品牌。</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">尚未新增奶粉品牌。</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No milk powder brands added yet.</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No milk powder brands added yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_delete</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Batch Delete</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">一括削除</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">批量删除</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">批次刪除</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Batch Delete</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Batch Delete</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_footer_delete</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_confirm_message_one</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm to delete this {0}?</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm to delete this {0}?</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm to delete this {0}?</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm to delete this {0}?</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm to delete this {0}?</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm to delete this {0}?</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_confirm_message_many</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm to delete these {0}?</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm to delete these {0}?</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm to delete these {0}?</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm to delete these {0}?</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm to delete these {0}?</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm to delete these {0}?</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_delete_title</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Selected Brands?</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">選択したブランドを削除しますか？</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">删除所选品牌？</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">刪除所選品牌？</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Selected Brands?</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Selected Brands?</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_delete_body</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{0}件のブランドを削除しますか？元に戻せません。</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将删除 {0} 个品牌，此操作无法撤销。</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">將刪除 {0} 筆品牌，此操作無法復原。</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_delete_title</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Brand?</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ブランドを削除しますか？</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">删除品牌？</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">刪除品牌？</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Brand?</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Brand?</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_delete_body</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This brand will be removed from your list.</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">このブランドはリストから削除されます。</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">此品牌将从列表中移除。</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">此品牌將從列表中移除。</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This brand will be removed from your list.</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This brand will be removed from your list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_delete_confirm_message</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete the brand:
+"{0} / {1} / {2}"?</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ブランドを削除してもよろしいですか：
+"{0} / {1} / {2}"？</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">确定要删除品牌：
+"{0} / {1} / {2}"吗？</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">確定要刪除品牌：
+"{0} / {1} / {2}"嗎？</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete the brand:
+"{0} / {1} / {2}"?</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete the brand:
+"{0} / {1} / {2}"?</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">custom_mix_ratio_page_title</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customize Mixing Ratio</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ミックス比率をカスタマイズ</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">自定义配比</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">自訂配比</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customize Mixing Ratio</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customize Mixing Ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">custom_mix_ratio_note</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Note: Once the mixing ratio is set, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">注：ミックス比率を設定すると、対応する粉ミルク濃度を自動取得し、調乳比率を算出して表示します。</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">说明：设置配比后，系统将自动获取对应奶粉浓度，计算并展示冲调比例。</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">說明：設定配比後，系統將自動取得對應奶粉濃度，計算並顯示沖調比例。</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Note: Once the mixing ratio is set, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Note: Once the mixing ratio is set, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">custom_mix_ratio_panel_title</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mix Ratio</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ミックス比率</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">配比</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">配比</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mix Ratio</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mix Ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">custom_mix_ratio_incomplete</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please enter both water and powder amounts.</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">水量と粉量の両方を入力してください。</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">请填写水量和粉量。</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">請填寫水量與粉量。</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please enter both water and powder amounts.</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please enter both water and powder amounts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">custom_mix_ratio_delete_confirm_message</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete the custom mixing ratio:
+"{0}ml / {1}g"?</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">カスタムミックス比率を削除してもよろしいですか：
+"{0}ml / {1}g"？</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">确定要删除自定义配比：
+"{0}ml / {1}g"吗？</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">確定要刪除自訂配比：
+"{0}ml / {1}g"嗎？</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete the custom mixing ratio:
+"{0}ml / {1}g"?</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete the custom mixing ratio:
+"{0}ml / {1}g"?</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dp_command_failed</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Could not send the command. Check device connection.</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">コマンドを送信できませんでした。接続を確認してください。</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">无法发送指令，请检查设备连接。</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">無法傳送指令，請檢查裝置連線。</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Could not send the command. Check device connection.</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Could not send the command. Check device connection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">device_power_off</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Device is powered off. Tap the power button to turn on.</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">電源がオフです。電源ボタンをタップしてオンにしてください。</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">设备已关机，请点击电源键开机。</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">裝置已關機，請點擊電源鍵開機。</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Device is powered off. Tap the power button to turn on.</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Device is powered off. Tap the power button to turn on.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: sync device DPs with SmartBottleMaker 07_15 schema
Align dpCodes/schema and app control flows with the latest Excel export:
start/stop via work_mode and working_status, scoop-based formula DPs,
temp value range 20–40, sensor intercepts, and child_lock binding.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/i18n_export.xlsx
+++ b/i18n_export.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G237"/>
+  <dimension ref="A1:G244"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7119,1675 +7119,1934 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_c01</t>
+          <t xml:space="preserve">error_e03</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">Error E03</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">エラー E03</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">错误 E03</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">錯誤 E03</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">Error E03</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">Error E03</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_c02</t>
+          <t xml:space="preserve">error_c01</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t xml:space="preserve">brand_coming_soon</t>
+          <t xml:space="preserve">error_c02</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand settings will be available in a future update.</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランド設定は今後のアップデートで提供予定です。</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t xml:space="preserve">品牌设置将在后续版本中提供。</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t xml:space="preserve">品牌設定將在後續版本中提供。</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand settings will be available in a future update.</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand settings will be available in a future update.</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_page_title</t>
+          <t xml:space="preserve">error_c03</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Milk Powder Brand</t>
+          <t xml:space="preserve">Error C03</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルクブランドを追加</t>
+          <t xml:space="preserve">エラー C03</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t xml:space="preserve">添加奶粉品牌</t>
+          <t xml:space="preserve">错误 C03</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t xml:space="preserve">新增奶粉品牌</t>
+          <t xml:space="preserve">錯誤 C03</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Milk Powder Brand</t>
+          <t xml:space="preserve">Error C03</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Milk Powder Brand</t>
+          <t xml:space="preserve">Error C03</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_edit_page_title</t>
+          <t xml:space="preserve">error_c04</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edit Milk Powder Brand</t>
+          <t xml:space="preserve">Error C04</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルクブランドを編集</t>
+          <t xml:space="preserve">エラー C04</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t xml:space="preserve">编辑奶粉品牌</t>
+          <t xml:space="preserve">错误 C04</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t xml:space="preserve">編輯奶粉品牌</t>
+          <t xml:space="preserve">錯誤 C04</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edit Milk Powder Brand</t>
+          <t xml:space="preserve">Error C04</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edit Milk Powder Brand</t>
+          <t xml:space="preserve">Error C04</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_custom_ratio_section</t>
+          <t xml:space="preserve">sensor_milkbox_missing</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Ratio</t>
+          <t xml:space="preserve">Powder box is not installed.</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t xml:space="preserve">カスタム比率</t>
+          <t xml:space="preserve">粉ミルクボックスが装着されていません。</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t xml:space="preserve">自定义配比</t>
+          <t xml:space="preserve">奶粉盒未安装。</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t xml:space="preserve">自訂配比</t>
+          <t xml:space="preserve">奶粉盒未安裝。</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Ratio</t>
+          <t xml:space="preserve">Powder box is not installed.</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Ratio</t>
+          <t xml:space="preserve">Powder box is not installed.</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_page_note</t>
+          <t xml:space="preserve">sensor_funnel_missing</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
+          <t xml:space="preserve">Funnel is not installed.</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t xml:space="preserve">注意：ブランド・シリーズ・段階を選択すると、対応する粉ミルク濃度を自動取得し、調乳比率を表示します。</t>
+          <t xml:space="preserve">ファネルが装着されていません。</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t xml:space="preserve">说明：选择品牌、系列和段数后，将自动获取对应奶粉浓度并计算、展示冲调比例。</t>
+          <t xml:space="preserve">漏斗未安装。</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t xml:space="preserve">說明：選擇品牌、系列與段數後，將自動取得對應奶粉濃度並計算、顯示沖調比例。</t>
+          <t xml:space="preserve">漏斗未安裝。</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
+          <t xml:space="preserve">Funnel is not installed.</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
+          <t xml:space="preserve">Funnel is not installed.</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_info_title</t>
+          <t xml:space="preserve">sensor_bottle_missing</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk Powder Info</t>
+          <t xml:space="preserve">Bottle is not in place.</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルク情報</t>
+          <t xml:space="preserve">哺乳瓶がセットされていません。</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉信息</t>
+          <t xml:space="preserve">奶瓶未就位。</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉資訊</t>
+          <t xml:space="preserve">奶瓶未就位。</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk Powder Info</t>
+          <t xml:space="preserve">Bottle is not in place.</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk Powder Info</t>
+          <t xml:space="preserve">Bottle is not in place.</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_select_brand</t>
+          <t xml:space="preserve">sensor_watertank_missing</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand</t>
+          <t xml:space="preserve">Water tank is missing or water level is too low.</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランド</t>
+          <t xml:space="preserve">水箱が未装着、または水量不足です。</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t xml:space="preserve">品牌</t>
+          <t xml:space="preserve">水箱未安装或水量不足。</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t xml:space="preserve">品牌</t>
+          <t xml:space="preserve">水箱未安裝或水量不足。</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand</t>
+          <t xml:space="preserve">Water tank is missing or water level is too low.</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand</t>
+          <t xml:space="preserve">Water tank is missing or water level is too low.</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_select_series</t>
+          <t xml:space="preserve">brand_coming_soon</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Brand settings will be available in a future update.</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t xml:space="preserve">シリーズ</t>
+          <t xml:space="preserve">ブランド設定は今後のアップデートで提供予定です。</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t xml:space="preserve">系列</t>
+          <t xml:space="preserve">品牌设置将在后续版本中提供。</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t xml:space="preserve">系列</t>
+          <t xml:space="preserve">品牌設定將在後續版本中提供。</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Brand settings will be available in a future update.</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Brand settings will be available in a future update.</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_select_stage</t>
+          <t xml:space="preserve">powder_brand_page_title</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage</t>
+          <t xml:space="preserve">Add Milk Powder Brand</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t xml:space="preserve">段階</t>
+          <t xml:space="preserve">粉ミルクブランドを追加</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t xml:space="preserve">段数</t>
+          <t xml:space="preserve">添加奶粉品牌</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t xml:space="preserve">段數</t>
+          <t xml:space="preserve">新增奶粉品牌</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage</t>
+          <t xml:space="preserve">Add Milk Powder Brand</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage</t>
+          <t xml:space="preserve">Add Milk Powder Brand</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_select_placeholder</t>
+          <t xml:space="preserve">powder_brand_edit_page_title</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select</t>
+          <t xml:space="preserve">Edit Milk Powder Brand</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t xml:space="preserve">選択</t>
+          <t xml:space="preserve">粉ミルクブランドを編集</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t xml:space="preserve">请选择</t>
+          <t xml:space="preserve">编辑奶粉品牌</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t xml:space="preserve">請選擇</t>
+          <t xml:space="preserve">編輯奶粉品牌</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select</t>
+          <t xml:space="preserve">Edit Milk Powder Brand</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select</t>
+          <t xml:space="preserve">Edit Milk Powder Brand</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_sheet_select_brand</t>
+          <t xml:space="preserve">powder_brand_custom_ratio_section</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Brand</t>
+          <t xml:space="preserve">Custom Ratio</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランドを選択</t>
+          <t xml:space="preserve">カスタム比率</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t xml:space="preserve">选择品牌</t>
+          <t xml:space="preserve">自定义配比</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t xml:space="preserve">選擇品牌</t>
+          <t xml:space="preserve">自訂配比</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Brand</t>
+          <t xml:space="preserve">Custom Ratio</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Brand</t>
+          <t xml:space="preserve">Custom Ratio</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_sheet_select_series</t>
+          <t xml:space="preserve">powder_brand_page_note</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Series</t>
+          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t xml:space="preserve">シリーズを選択</t>
+          <t xml:space="preserve">注意：ブランド・シリーズ・段階を選択すると、対応する粉ミルク濃度を自動取得し、調乳比率を表示します。</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t xml:space="preserve">选择系列</t>
+          <t xml:space="preserve">说明：选择品牌、系列和段数后，将自动获取对应奶粉浓度并计算、展示冲调比例。</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t xml:space="preserve">選擇系列</t>
+          <t xml:space="preserve">說明：選擇品牌、系列與段數後，將自動取得對應奶粉濃度並計算、顯示沖調比例。</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Series</t>
+          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Series</t>
+          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_sheet_select_stage</t>
+          <t xml:space="preserve">powder_brand_info_title</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Stage</t>
+          <t xml:space="preserve">Milk Powder Info</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t xml:space="preserve">段階を選択</t>
+          <t xml:space="preserve">粉ミルク情報</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t xml:space="preserve">选择段数</t>
+          <t xml:space="preserve">奶粉信息</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t xml:space="preserve">選擇段數</t>
+          <t xml:space="preserve">奶粉資訊</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Stage</t>
+          <t xml:space="preserve">Milk Powder Info</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Stage</t>
+          <t xml:space="preserve">Milk Powder Info</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_search_placeholder</t>
+          <t xml:space="preserve">powder_brand_select_brand</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t xml:space="preserve">Search brand...</t>
+          <t xml:space="preserve">Brand</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランドを検索...</t>
+          <t xml:space="preserve">ブランド</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t xml:space="preserve">搜索品牌...</t>
+          <t xml:space="preserve">品牌</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t xml:space="preserve">搜尋品牌...</t>
+          <t xml:space="preserve">品牌</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t xml:space="preserve">Search brand...</t>
+          <t xml:space="preserve">Brand</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t xml:space="preserve">Search brand...</t>
+          <t xml:space="preserve">Brand</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_search_empty</t>
+          <t xml:space="preserve">powder_brand_select_series</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t xml:space="preserve">No brands match your search.</t>
+          <t xml:space="preserve">Series</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t xml:space="preserve">該当するブランドがありません。</t>
+          <t xml:space="preserve">シリーズ</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t xml:space="preserve">未找到匹配的品牌。</t>
+          <t xml:space="preserve">系列</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t xml:space="preserve">找不到符合的品牌。</t>
+          <t xml:space="preserve">系列</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t xml:space="preserve">No brands match your search.</t>
+          <t xml:space="preserve">Series</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t xml:space="preserve">No brands match your search.</t>
+          <t xml:space="preserve">Series</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_not_listed</t>
+          <t xml:space="preserve">powder_brand_select_stage</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand not listed? </t>
+          <t xml:space="preserve">Stage</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランドが見つかりませんか？ </t>
+          <t xml:space="preserve">段階</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t xml:space="preserve">没有您的品牌？ </t>
+          <t xml:space="preserve">段数</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t xml:space="preserve">找不到您的品牌？ </t>
+          <t xml:space="preserve">段數</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand not listed? </t>
+          <t xml:space="preserve">Stage</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand not listed? </t>
+          <t xml:space="preserve">Stage</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_customize_ratio</t>
+          <t xml:space="preserve">powder_brand_select_placeholder</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t xml:space="preserve">Customize mixing ratio.</t>
+          <t xml:space="preserve">Select</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミックス比率をカスタマイズ</t>
+          <t xml:space="preserve">選択</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t xml:space="preserve">自定义配比</t>
+          <t xml:space="preserve">请选择</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t xml:space="preserve">自訂配比</t>
+          <t xml:space="preserve">請選擇</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t xml:space="preserve">Customize mixing ratio.</t>
+          <t xml:space="preserve">Select</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t xml:space="preserve">Customize mixing ratio.</t>
+          <t xml:space="preserve">Select</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_custom_label</t>
+          <t xml:space="preserve">powder_brand_sheet_select_brand</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom</t>
+          <t xml:space="preserve">Select Brand</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t xml:space="preserve">カスタム</t>
+          <t xml:space="preserve">ブランドを選択</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t xml:space="preserve">自定义</t>
+          <t xml:space="preserve">选择品牌</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t xml:space="preserve">自訂</t>
+          <t xml:space="preserve">選擇品牌</t>
         </is>
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom</t>
+          <t xml:space="preserve">Select Brand</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom</t>
+          <t xml:space="preserve">Select Brand</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_custom_water_ml</t>
+          <t xml:space="preserve">powder_brand_sheet_select_series</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water (mL)</t>
+          <t xml:space="preserve">Select Series</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量 (mL)</t>
+          <t xml:space="preserve">シリーズを選択</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量 (mL)</t>
+          <t xml:space="preserve">选择系列</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量 (mL)</t>
+          <t xml:space="preserve">選擇系列</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water (mL)</t>
+          <t xml:space="preserve">Select Series</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water (mL)</t>
+          <t xml:space="preserve">Select Series</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_custom_powder_g</t>
+          <t xml:space="preserve">powder_brand_sheet_select_stage</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder (g)</t>
+          <t xml:space="preserve">Select Stage</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉量 (g)</t>
+          <t xml:space="preserve">段階を選択</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉量 (g)</t>
+          <t xml:space="preserve">选择段数</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉量 (g)</t>
+          <t xml:space="preserve">選擇段數</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder (g)</t>
+          <t xml:space="preserve">Select Stage</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder (g)</t>
+          <t xml:space="preserve">Select Stage</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_custom_apply</t>
+          <t xml:space="preserve">powder_brand_search_placeholder</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apply</t>
+          <t xml:space="preserve">Search brand...</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t xml:space="preserve">適用</t>
+          <t xml:space="preserve">ブランドを検索...</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t xml:space="preserve">应用</t>
+          <t xml:space="preserve">搜索品牌...</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t xml:space="preserve">套用</t>
+          <t xml:space="preserve">搜尋品牌...</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apply</t>
+          <t xml:space="preserve">Search brand...</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apply</t>
+          <t xml:space="preserve">Search brand...</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_ratio_title</t>
+          <t xml:space="preserve">powder_brand_search_empty</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recommended Mix Ratio</t>
+          <t xml:space="preserve">No brands match your search.</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t xml:space="preserve">推奨ミックス比率</t>
+          <t xml:space="preserve">該当するブランドがありません。</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t xml:space="preserve">推荐配比</t>
+          <t xml:space="preserve">未找到匹配的品牌。</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t xml:space="preserve">建議配比</t>
+          <t xml:space="preserve">找不到符合的品牌。</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recommended Mix Ratio</t>
+          <t xml:space="preserve">No brands match your search.</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recommended Mix Ratio</t>
+          <t xml:space="preserve">No brands match your search.</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_ratio_water</t>
+          <t xml:space="preserve">powder_brand_not_listed</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water</t>
+          <t xml:space="preserve">Brand not listed? </t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t xml:space="preserve">水</t>
+          <t xml:space="preserve">ブランドが見つかりませんか？ </t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t xml:space="preserve">水</t>
+          <t xml:space="preserve">没有您的品牌？ </t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t xml:space="preserve">水</t>
+          <t xml:space="preserve">找不到您的品牌？ </t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water</t>
+          <t xml:space="preserve">Brand not listed? </t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water</t>
+          <t xml:space="preserve">Brand not listed? </t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_ratio_powder</t>
+          <t xml:space="preserve">powder_brand_customize_ratio</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder</t>
+          <t xml:space="preserve">Customize mixing ratio.</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルク</t>
+          <t xml:space="preserve">ミックス比率をカスタマイズ</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉</t>
+          <t xml:space="preserve">自定义配比</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉</t>
+          <t xml:space="preserve">自訂配比</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder</t>
+          <t xml:space="preserve">Customize mixing ratio.</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder</t>
+          <t xml:space="preserve">Customize mixing ratio.</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_settings_title</t>
+          <t xml:space="preserve">powder_brand_custom_label</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder Brand Settings</t>
+          <t xml:space="preserve">Custom</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルクブランド設定</t>
+          <t xml:space="preserve">カスタム</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉品牌设置</t>
+          <t xml:space="preserve">自定义</t>
         </is>
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉品牌設定</t>
+          <t xml:space="preserve">自訂</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder Brand Settings</t>
+          <t xml:space="preserve">Custom</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder Brand Settings</t>
+          <t xml:space="preserve">Custom</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_add_brand</t>
+          <t xml:space="preserve">powder_brand_custom_water_ml</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Brand</t>
+          <t xml:space="preserve">Water (mL)</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランドを追加</t>
+          <t xml:space="preserve">水量 (mL)</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t xml:space="preserve">添加品牌</t>
+          <t xml:space="preserve">水量 (mL)</t>
         </is>
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t xml:space="preserve">新增品牌</t>
+          <t xml:space="preserve">水量 (mL)</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Brand</t>
+          <t xml:space="preserve">Water (mL)</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Brand</t>
+          <t xml:space="preserve">Water (mL)</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_empty_message</t>
+          <t xml:space="preserve">powder_brand_custom_powder_g</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t xml:space="preserve">No milk powder brands added yet.</t>
+          <t xml:space="preserve">Powder (g)</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルクブランドはまだ追加されていません。</t>
+          <t xml:space="preserve">粉量 (g)</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t xml:space="preserve">尚未添加奶粉品牌。</t>
+          <t xml:space="preserve">粉量 (g)</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t xml:space="preserve">尚未新增奶粉品牌。</t>
+          <t xml:space="preserve">粉量 (g)</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t xml:space="preserve">No milk powder brands added yet.</t>
+          <t xml:space="preserve">Powder (g)</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t xml:space="preserve">No milk powder brands added yet.</t>
+          <t xml:space="preserve">Powder (g)</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_batch_delete</t>
+          <t xml:space="preserve">powder_brand_custom_apply</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t xml:space="preserve">Batch Delete</t>
+          <t xml:space="preserve">Apply</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t xml:space="preserve">一括削除</t>
+          <t xml:space="preserve">適用</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t xml:space="preserve">批量删除</t>
+          <t xml:space="preserve">应用</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t xml:space="preserve">批次刪除</t>
+          <t xml:space="preserve">套用</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t xml:space="preserve">Batch Delete</t>
+          <t xml:space="preserve">Apply</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t xml:space="preserve">Batch Delete</t>
+          <t xml:space="preserve">Apply</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_batch_footer_delete</t>
+          <t xml:space="preserve">powder_brand_ratio_title</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete ({0})</t>
+          <t xml:space="preserve">Recommended Mix Ratio</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete ({0})</t>
+          <t xml:space="preserve">推奨ミックス比率</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete ({0})</t>
+          <t xml:space="preserve">推荐配比</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete ({0})</t>
+          <t xml:space="preserve">建議配比</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete ({0})</t>
+          <t xml:space="preserve">Recommended Mix Ratio</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete ({0})</t>
+          <t xml:space="preserve">Recommended Mix Ratio</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_batch_confirm_message_one</t>
+          <t xml:space="preserve">powder_brand_ratio_water</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+          <t xml:space="preserve">Water</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+          <t xml:space="preserve">水</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+          <t xml:space="preserve">水</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+          <t xml:space="preserve">水</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+          <t xml:space="preserve">Water</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+          <t xml:space="preserve">Water</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_batch_confirm_message_many</t>
+          <t xml:space="preserve">powder_brand_ratio_powder</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+          <t xml:space="preserve">Powder</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+          <t xml:space="preserve">粉ミルク</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+          <t xml:space="preserve">奶粉</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+          <t xml:space="preserve">奶粉</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+          <t xml:space="preserve">Powder</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+          <t xml:space="preserve">Powder</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_batch_delete_title</t>
+          <t xml:space="preserve">powder_brand_settings_title</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete Selected Brands?</t>
+          <t xml:space="preserve">Powder Brand Settings</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t xml:space="preserve">選択したブランドを削除しますか？</t>
+          <t xml:space="preserve">粉ミルクブランド設定</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t xml:space="preserve">删除所选品牌？</t>
+          <t xml:space="preserve">奶粉品牌设置</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t xml:space="preserve">刪除所選品牌？</t>
+          <t xml:space="preserve">奶粉品牌設定</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete Selected Brands?</t>
+          <t xml:space="preserve">Powder Brand Settings</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete Selected Brands?</t>
+          <t xml:space="preserve">Powder Brand Settings</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_batch_delete_body</t>
+          <t xml:space="preserve">powder_brand_add_brand</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
+          <t xml:space="preserve">Add Brand</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t xml:space="preserve">{0}件のブランドを削除しますか？元に戻せません。</t>
+          <t xml:space="preserve">ブランドを追加</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t xml:space="preserve">将删除 {0} 个品牌，此操作无法撤销。</t>
+          <t xml:space="preserve">添加品牌</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t xml:space="preserve">將刪除 {0} 筆品牌，此操作無法復原。</t>
+          <t xml:space="preserve">新增品牌</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
+          <t xml:space="preserve">Add Brand</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
+          <t xml:space="preserve">Add Brand</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_delete_title</t>
+          <t xml:space="preserve">powder_brand_empty_message</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete Brand?</t>
+          <t xml:space="preserve">No milk powder brands added yet.</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランドを削除しますか？</t>
+          <t xml:space="preserve">粉ミルクブランドはまだ追加されていません。</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t xml:space="preserve">删除品牌？</t>
+          <t xml:space="preserve">尚未添加奶粉品牌。</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t xml:space="preserve">刪除品牌？</t>
+          <t xml:space="preserve">尚未新增奶粉品牌。</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete Brand?</t>
+          <t xml:space="preserve">No milk powder brands added yet.</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete Brand?</t>
+          <t xml:space="preserve">No milk powder brands added yet.</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_delete_body</t>
+          <t xml:space="preserve">powder_brand_batch_delete</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t xml:space="preserve">This brand will be removed from your list.</t>
+          <t xml:space="preserve">Batch Delete</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t xml:space="preserve">このブランドはリストから削除されます。</t>
+          <t xml:space="preserve">一括削除</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t xml:space="preserve">此品牌将从列表中移除。</t>
+          <t xml:space="preserve">批量删除</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t xml:space="preserve">此品牌將從列表中移除。</t>
+          <t xml:space="preserve">批次刪除</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t xml:space="preserve">This brand will be removed from your list.</t>
+          <t xml:space="preserve">Batch Delete</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t xml:space="preserve">This brand will be removed from your list.</t>
+          <t xml:space="preserve">Batch Delete</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
+          <t xml:space="preserve">powder_brand_batch_footer_delete</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_confirm_message_one</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_confirm_message_many</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_delete_title</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Selected Brands?</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">選択したブランドを削除しますか？</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">删除所选品牌？</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">刪除所選品牌？</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Selected Brands?</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Selected Brands?</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_delete_body</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{0}件のブランドを削除しますか？元に戻せません。</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将删除 {0} 个品牌，此操作无法撤销。</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">將刪除 {0} 筆品牌，此操作無法復原。</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_delete_title</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Brand?</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ブランドを削除しますか？</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">删除品牌？</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">刪除品牌？</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Brand?</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Brand?</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_delete_body</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This brand will be removed from your list.</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">このブランドはリストから削除されます。</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">此品牌将从列表中移除。</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">此品牌將從列表中移除。</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This brand will be removed from your list.</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This brand will be removed from your list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
           <t xml:space="preserve">powder_brand_delete_confirm_message</t>
         </is>
       </c>
-      <c r="B230" t="inlineStr">
+      <c r="B237" t="inlineStr">
         <is>
           <t xml:space="preserve">Are you sure you want to delete the brand:
 "{0} / {1} / {2}"?</t>
         </is>
       </c>
-      <c r="C230" t="inlineStr">
+      <c r="C237" t="inlineStr">
         <is>
           <t xml:space="preserve">ブランドを削除してもよろしいですか：
 "{0} / {1} / {2}"？</t>
         </is>
       </c>
-      <c r="D230" t="inlineStr">
+      <c r="D237" t="inlineStr">
         <is>
           <t xml:space="preserve">确定要删除品牌：
 "{0} / {1} / {2}"吗？</t>
         </is>
       </c>
-      <c r="E230" t="inlineStr">
+      <c r="E237" t="inlineStr">
         <is>
           <t xml:space="preserve">確定要刪除品牌：
 "{0} / {1} / {2}"嗎？</t>
         </is>
       </c>
-      <c r="F230" t="inlineStr">
+      <c r="F237" t="inlineStr">
         <is>
           <t xml:space="preserve">Are you sure you want to delete the brand:
 "{0} / {1} / {2}"?</t>
         </is>
       </c>
-      <c r="G230" t="inlineStr">
+      <c r="G237" t="inlineStr">
         <is>
           <t xml:space="preserve">Are you sure you want to delete the brand:
 "{0} / {1} / {2}"?</t>
         </is>
       </c>
     </row>
-    <row r="231">
-      <c r="A231" t="inlineStr">
+    <row r="238">
+      <c r="A238" t="inlineStr">
         <is>
           <t xml:space="preserve">custom_mix_ratio_page_title</t>
         </is>
       </c>
-      <c r="B231" t="inlineStr">
+      <c r="B238" t="inlineStr">
         <is>
           <t xml:space="preserve">Customize Mixing Ratio</t>
         </is>
       </c>
-      <c r="C231" t="inlineStr">
+      <c r="C238" t="inlineStr">
         <is>
           <t xml:space="preserve">ミックス比率をカスタマイズ</t>
         </is>
       </c>
-      <c r="D231" t="inlineStr">
+      <c r="D238" t="inlineStr">
         <is>
           <t xml:space="preserve">自定义配比</t>
         </is>
       </c>
-      <c r="E231" t="inlineStr">
+      <c r="E238" t="inlineStr">
         <is>
           <t xml:space="preserve">自訂配比</t>
         </is>
       </c>
-      <c r="F231" t="inlineStr">
+      <c r="F238" t="inlineStr">
         <is>
           <t xml:space="preserve">Customize Mixing Ratio</t>
         </is>
       </c>
-      <c r="G231" t="inlineStr">
+      <c r="G238" t="inlineStr">
         <is>
           <t xml:space="preserve">Customize Mixing Ratio</t>
         </is>
       </c>
     </row>
-    <row r="232">
-      <c r="A232" t="inlineStr">
+    <row r="239">
+      <c r="A239" t="inlineStr">
         <is>
           <t xml:space="preserve">custom_mix_ratio_note</t>
         </is>
       </c>
-      <c r="B232" t="inlineStr">
+      <c r="B239" t="inlineStr">
         <is>
           <t xml:space="preserve">Note: Once the mixing ratio is set, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
-      <c r="C232" t="inlineStr">
+      <c r="C239" t="inlineStr">
         <is>
           <t xml:space="preserve">注：ミックス比率を設定すると、対応する粉ミルク濃度を自動取得し、調乳比率を算出して表示します。</t>
         </is>
       </c>
-      <c r="D232" t="inlineStr">
+      <c r="D239" t="inlineStr">
         <is>
           <t xml:space="preserve">说明：设置配比后，系统将自动获取对应奶粉浓度，计算并展示冲调比例。</t>
         </is>
       </c>
-      <c r="E232" t="inlineStr">
+      <c r="E239" t="inlineStr">
         <is>
           <t xml:space="preserve">說明：設定配比後，系統將自動取得對應奶粉濃度，計算並顯示沖調比例。</t>
         </is>
       </c>
-      <c r="F232" t="inlineStr">
+      <c r="F239" t="inlineStr">
         <is>
           <t xml:space="preserve">Note: Once the mixing ratio is set, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
-      <c r="G232" t="inlineStr">
+      <c r="G239" t="inlineStr">
         <is>
           <t xml:space="preserve">Note: Once the mixing ratio is set, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
     </row>
-    <row r="233">
-      <c r="A233" t="inlineStr">
+    <row r="240">
+      <c r="A240" t="inlineStr">
         <is>
           <t xml:space="preserve">custom_mix_ratio_panel_title</t>
         </is>
       </c>
-      <c r="B233" t="inlineStr">
+      <c r="B240" t="inlineStr">
         <is>
           <t xml:space="preserve">Mix Ratio</t>
         </is>
       </c>
-      <c r="C233" t="inlineStr">
+      <c r="C240" t="inlineStr">
         <is>
           <t xml:space="preserve">ミックス比率</t>
         </is>
       </c>
-      <c r="D233" t="inlineStr">
+      <c r="D240" t="inlineStr">
         <is>
           <t xml:space="preserve">配比</t>
         </is>
       </c>
-      <c r="E233" t="inlineStr">
+      <c r="E240" t="inlineStr">
         <is>
           <t xml:space="preserve">配比</t>
         </is>
       </c>
-      <c r="F233" t="inlineStr">
+      <c r="F240" t="inlineStr">
         <is>
           <t xml:space="preserve">Mix Ratio</t>
         </is>
       </c>
-      <c r="G233" t="inlineStr">
+      <c r="G240" t="inlineStr">
         <is>
           <t xml:space="preserve">Mix Ratio</t>
         </is>
       </c>
     </row>
-    <row r="234">
-      <c r="A234" t="inlineStr">
+    <row r="241">
+      <c r="A241" t="inlineStr">
         <is>
           <t xml:space="preserve">custom_mix_ratio_incomplete</t>
         </is>
       </c>
-      <c r="B234" t="inlineStr">
+      <c r="B241" t="inlineStr">
         <is>
           <t xml:space="preserve">Please enter both water and powder amounts.</t>
         </is>
       </c>
-      <c r="C234" t="inlineStr">
+      <c r="C241" t="inlineStr">
         <is>
           <t xml:space="preserve">水量と粉量の両方を入力してください。</t>
         </is>
       </c>
-      <c r="D234" t="inlineStr">
+      <c r="D241" t="inlineStr">
         <is>
           <t xml:space="preserve">请填写水量和粉量。</t>
         </is>
       </c>
-      <c r="E234" t="inlineStr">
+      <c r="E241" t="inlineStr">
         <is>
           <t xml:space="preserve">請填寫水量與粉量。</t>
         </is>
       </c>
-      <c r="F234" t="inlineStr">
+      <c r="F241" t="inlineStr">
         <is>
           <t xml:space="preserve">Please enter both water and powder amounts.</t>
         </is>
       </c>
-      <c r="G234" t="inlineStr">
+      <c r="G241" t="inlineStr">
         <is>
           <t xml:space="preserve">Please enter both water and powder amounts.</t>
         </is>
       </c>
     </row>
-    <row r="235">
-      <c r="A235" t="inlineStr">
+    <row r="242">
+      <c r="A242" t="inlineStr">
         <is>
           <t xml:space="preserve">custom_mix_ratio_delete_confirm_message</t>
         </is>
       </c>
-      <c r="B235" t="inlineStr">
+      <c r="B242" t="inlineStr">
         <is>
           <t xml:space="preserve">Are you sure you want to delete the custom mixing ratio:
 "{0}ml / {1}g"?</t>
         </is>
       </c>
-      <c r="C235" t="inlineStr">
+      <c r="C242" t="inlineStr">
         <is>
           <t xml:space="preserve">カスタムミックス比率を削除してもよろしいですか：
 "{0}ml / {1}g"？</t>
         </is>
       </c>
-      <c r="D235" t="inlineStr">
+      <c r="D242" t="inlineStr">
         <is>
           <t xml:space="preserve">确定要删除自定义配比：
 "{0}ml / {1}g"吗？</t>
         </is>
       </c>
-      <c r="E235" t="inlineStr">
+      <c r="E242" t="inlineStr">
         <is>
           <t xml:space="preserve">確定要刪除自訂配比：
 "{0}ml / {1}g"嗎？</t>
         </is>
       </c>
-      <c r="F235" t="inlineStr">
+      <c r="F242" t="inlineStr">
         <is>
           <t xml:space="preserve">Are you sure you want to delete the custom mixing ratio:
 "{0}ml / {1}g"?</t>
         </is>
       </c>
-      <c r="G235" t="inlineStr">
+      <c r="G242" t="inlineStr">
         <is>
           <t xml:space="preserve">Are you sure you want to delete the custom mixing ratio:
 "{0}ml / {1}g"?</t>
         </is>
       </c>
     </row>
-    <row r="236">
-      <c r="A236" t="inlineStr">
+    <row r="243">
+      <c r="A243" t="inlineStr">
         <is>
           <t xml:space="preserve">dp_command_failed</t>
         </is>
       </c>
-      <c r="B236" t="inlineStr">
+      <c r="B243" t="inlineStr">
         <is>
           <t xml:space="preserve">Could not send the command. Check device connection.</t>
         </is>
       </c>
-      <c r="C236" t="inlineStr">
+      <c r="C243" t="inlineStr">
         <is>
           <t xml:space="preserve">コマンドを送信できませんでした。接続を確認してください。</t>
         </is>
       </c>
-      <c r="D236" t="inlineStr">
+      <c r="D243" t="inlineStr">
         <is>
           <t xml:space="preserve">无法发送指令，请检查设备连接。</t>
         </is>
       </c>
-      <c r="E236" t="inlineStr">
+      <c r="E243" t="inlineStr">
         <is>
           <t xml:space="preserve">無法傳送指令，請檢查裝置連線。</t>
         </is>
       </c>
-      <c r="F236" t="inlineStr">
+      <c r="F243" t="inlineStr">
         <is>
           <t xml:space="preserve">Could not send the command. Check device connection.</t>
         </is>
       </c>
-      <c r="G236" t="inlineStr">
+      <c r="G243" t="inlineStr">
         <is>
           <t xml:space="preserve">Could not send the command. Check device connection.</t>
         </is>
       </c>
     </row>
-    <row r="237">
-      <c r="A237" t="inlineStr">
+    <row r="244">
+      <c r="A244" t="inlineStr">
         <is>
           <t xml:space="preserve">device_power_off</t>
         </is>
       </c>
-      <c r="B237" t="inlineStr">
+      <c r="B244" t="inlineStr">
         <is>
           <t xml:space="preserve">Device is powered off. Tap the power button to turn on.</t>
         </is>
       </c>
-      <c r="C237" t="inlineStr">
+      <c r="C244" t="inlineStr">
         <is>
           <t xml:space="preserve">電源がオフです。電源ボタンをタップしてオンにしてください。</t>
         </is>
       </c>
-      <c r="D237" t="inlineStr">
+      <c r="D244" t="inlineStr">
         <is>
           <t xml:space="preserve">设备已关机，请点击电源键开机。</t>
         </is>
       </c>
-      <c r="E237" t="inlineStr">
+      <c r="E244" t="inlineStr">
         <is>
           <t xml:space="preserve">裝置已關機，請點擊電源鍵開機。</t>
         </is>
       </c>
-      <c r="F237" t="inlineStr">
+      <c r="F244" t="inlineStr">
         <is>
           <t xml:space="preserve">Device is powered off. Tap the power button to turn on.</t>
         </is>
       </c>
-      <c r="G237" t="inlineStr">
+      <c r="G244" t="inlineStr">
         <is>
           <t xml:space="preserve">Device is powered off. Tap the power button to turn on.</t>
         </is>

</xml_diff>

<commit_message>
feat: add feeding record confirmation flow
</commit_message>
<xml_diff>
--- a/i18n_export.xlsx
+++ b/i18n_export.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G293"/>
+  <dimension ref="A1:G302"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7970,2896 +7970,3229 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t xml:space="preserve">block_none</t>
+          <t xml:space="preserve">feeding_confirmation_title</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Milk Feeding Record Confirmation!</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Milk Feeding Record Confirmation!</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">确认奶瓶喂养记录</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Milk Feeding Record Confirmation!</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Milk Feeding Record Confirmation!</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Milk Feeding Record Confirmation!</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t xml:space="preserve">block_water_tank_missing</t>
+          <t xml:space="preserve">feeding_confirmation_body</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank is not installed.</t>
+          <t xml:space="preserve">Please confirm how much of the prepared milk your baby finished.</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱が装着されていません。</t>
+          <t xml:space="preserve">Please confirm how much of the prepared milk your baby finished.</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱未安装。</t>
+          <t xml:space="preserve">请确认宝宝喝完了多少已冲调的奶。</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱未安裝。</t>
+          <t xml:space="preserve">Please confirm how much of the prepared milk your baby finished.</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank is not installed.</t>
+          <t xml:space="preserve">Please confirm how much of the prepared milk your baby finished.</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank is not installed.</t>
+          <t xml:space="preserve">Please confirm how much of the prepared milk your baby finished.</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t xml:space="preserve">block_low_water</t>
+          <t xml:space="preserve">feeding_confirmation_remaining</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water level is too low.</t>
+          <t xml:space="preserve">Remaining milk</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量が不足しています。</t>
+          <t xml:space="preserve">Remaining milk</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量不足。</t>
+          <t xml:space="preserve">剩余奶量</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量不足。</t>
+          <t xml:space="preserve">Remaining milk</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water level is too low.</t>
+          <t xml:space="preserve">Remaining milk</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water level is too low.</t>
+          <t xml:space="preserve">Remaining milk</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t xml:space="preserve">block_powder_box_missing</t>
+          <t xml:space="preserve">feeding_confirmation_updated</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder box is not installed.</t>
+          <t xml:space="preserve">Feeding record updated</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルクボックスが装着されていません。</t>
+          <t xml:space="preserve">Feeding record updated</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉盒未安装。</t>
+          <t xml:space="preserve">喂养记录已更新</t>
         </is>
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉盒未安裝。</t>
+          <t xml:space="preserve">Feeding record updated</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder box is not installed.</t>
+          <t xml:space="preserve">Feeding record updated</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder box is not installed.</t>
+          <t xml:space="preserve">Feeding record updated</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t xml:space="preserve">block_funnel_missing</t>
+          <t xml:space="preserve">feeding_confirmation_unavailable</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Funnel is not installed.</t>
+          <t xml:space="preserve">This feeding record is unavailable.</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t xml:space="preserve">ファネルが装着されていません。</t>
+          <t xml:space="preserve">This feeding record is unavailable.</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t xml:space="preserve">漏斗未安装。</t>
+          <t xml:space="preserve">无法读取这条喂养记录。</t>
         </is>
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t xml:space="preserve">漏斗未安裝。</t>
+          <t xml:space="preserve">This feeding record is unavailable.</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Funnel is not installed.</t>
+          <t xml:space="preserve">This feeding record is unavailable.</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Funnel is not installed.</t>
+          <t xml:space="preserve">This feeding record is unavailable.</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t xml:space="preserve">block_bottle_missing</t>
+          <t xml:space="preserve">feeding_confirmation_update_failed</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle is not in place.</t>
+          <t xml:space="preserve">Couldn’t update the feeding record. Try again.</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t xml:space="preserve">哺乳瓶がセットされていません。</t>
+          <t xml:space="preserve">Couldn’t update the feeding record. Try again.</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶瓶未就位。</t>
+          <t xml:space="preserve">无法更新喂养记录，请重试。</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶瓶未就位。</t>
+          <t xml:space="preserve">Couldn’t update the feeding record. Try again.</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle is not in place.</t>
+          <t xml:space="preserve">Couldn’t update the feeding record. Try again.</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle is not in place.</t>
+          <t xml:space="preserve">Couldn’t update the feeding record. Try again.</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t xml:space="preserve">block_hot_alert</t>
+          <t xml:space="preserve">feeding_confirmation_clear_failed</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t xml:space="preserve">Device is too hot. Please wait.</t>
+          <t xml:space="preserve">The record was updated, but the reminder could not be cleared.</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t xml:space="preserve">本体が高温です。しばらくお待ちください。</t>
+          <t xml:space="preserve">The record was updated, but the reminder could not be cleared.</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t xml:space="preserve">设备温度过高，请稍候。</t>
+          <t xml:space="preserve">记录已更新，但无法清除提醒。</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t xml:space="preserve">設備溫度過高，請稍候。</t>
+          <t xml:space="preserve">The record was updated, but the reminder could not be cleared.</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t xml:space="preserve">Device is too hot. Please wait.</t>
+          <t xml:space="preserve">The record was updated, but the reminder could not be cleared.</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t xml:space="preserve">Device is too hot. Please wait.</t>
+          <t xml:space="preserve">The record was updated, but the reminder could not be cleared.</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_none</t>
+          <t xml:space="preserve">feeding_confirmation_offline</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Connect the device to confirm this record.</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Connect the device to confirm this record.</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">连接设备后再确认这条记录。</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Connect the device to confirm this record.</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Connect the device to confirm this record.</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Connect the device to confirm this record.</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_hot</t>
+          <t xml:space="preserve">feeding_confirmation_saving</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t xml:space="preserve">High temperature alert</t>
+          <t xml:space="preserve">Saving…</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t xml:space="preserve">High temperature alert</t>
+          <t xml:space="preserve">Saving…</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t xml:space="preserve">High temperature alert</t>
+          <t xml:space="preserve">保存中…</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t xml:space="preserve">High temperature alert</t>
+          <t xml:space="preserve">Saving…</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t xml:space="preserve">High temperature alert</t>
+          <t xml:space="preserve">Saving…</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t xml:space="preserve">High temperature alert</t>
+          <t xml:space="preserve">Saving…</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_e01</t>
+          <t xml:space="preserve">block_none</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E01</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E01</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E01</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E01</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E01</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E01</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_e02</t>
+          <t xml:space="preserve">block_water_tank_missing</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E02</t>
+          <t xml:space="preserve">Water tank is not installed.</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E02</t>
+          <t xml:space="preserve">水箱が装着されていません。</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E02</t>
+          <t xml:space="preserve">水箱未安装。</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E02</t>
+          <t xml:space="preserve">水箱未安裝。</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E02</t>
+          <t xml:space="preserve">Water tank is not installed.</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E02</t>
+          <t xml:space="preserve">Water tank is not installed.</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_e03</t>
+          <t xml:space="preserve">block_low_water</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E03</t>
+          <t xml:space="preserve">Water level is too low.</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t xml:space="preserve">エラー E03</t>
+          <t xml:space="preserve">水量が不足しています。</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t xml:space="preserve">错误 E03</t>
+          <t xml:space="preserve">水量不足。</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t xml:space="preserve">錯誤 E03</t>
+          <t xml:space="preserve">水量不足。</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E03</t>
+          <t xml:space="preserve">Water level is too low.</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E03</t>
+          <t xml:space="preserve">Water level is too low.</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_c01</t>
+          <t xml:space="preserve">block_powder_box_missing</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">Powder box is not installed.</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">粉ミルクボックスが装着されていません。</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">奶粉盒未安装。</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">奶粉盒未安裝。</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">Powder box is not installed.</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">Powder box is not installed.</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_c02</t>
+          <t xml:space="preserve">block_funnel_missing</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">Funnel is not installed.</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">ファネルが装着されていません。</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">漏斗未安装。</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">漏斗未安裝。</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">Funnel is not installed.</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">Funnel is not installed.</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_c03</t>
+          <t xml:space="preserve">block_bottle_missing</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C03</t>
+          <t xml:space="preserve">Bottle is not in place.</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t xml:space="preserve">エラー C03</t>
+          <t xml:space="preserve">哺乳瓶がセットされていません。</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t xml:space="preserve">错误 C03</t>
+          <t xml:space="preserve">奶瓶未就位。</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t xml:space="preserve">錯誤 C03</t>
+          <t xml:space="preserve">奶瓶未就位。</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C03</t>
+          <t xml:space="preserve">Bottle is not in place.</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C03</t>
+          <t xml:space="preserve">Bottle is not in place.</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_c04</t>
+          <t xml:space="preserve">block_hot_alert</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C04</t>
+          <t xml:space="preserve">Device is too hot. Please wait.</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t xml:space="preserve">エラー C04</t>
+          <t xml:space="preserve">本体が高温です。しばらくお待ちください。</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t xml:space="preserve">错误 C04</t>
+          <t xml:space="preserve">设备温度过高，请稍候。</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t xml:space="preserve">錯誤 C04</t>
+          <t xml:space="preserve">設備溫度過高，請稍候。</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C04</t>
+          <t xml:space="preserve">Device is too hot. Please wait.</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C04</t>
+          <t xml:space="preserve">Device is too hot. Please wait.</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t xml:space="preserve">sensor_milkbox_missing</t>
+          <t xml:space="preserve">error_none</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder box is not installed.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルクボックスが装着されていません。</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉盒未安装。</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉盒未安裝。</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder box is not installed.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder box is not installed.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t xml:space="preserve">sensor_funnel_missing</t>
+          <t xml:space="preserve">error_hot</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Funnel is not installed.</t>
+          <t xml:space="preserve">High temperature alert</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t xml:space="preserve">ファネルが装着されていません。</t>
+          <t xml:space="preserve">High temperature alert</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t xml:space="preserve">漏斗未安装。</t>
+          <t xml:space="preserve">High temperature alert</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t xml:space="preserve">漏斗未安裝。</t>
+          <t xml:space="preserve">High temperature alert</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Funnel is not installed.</t>
+          <t xml:space="preserve">High temperature alert</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Funnel is not installed.</t>
+          <t xml:space="preserve">High temperature alert</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t xml:space="preserve">sensor_bottle_missing</t>
+          <t xml:space="preserve">error_e01</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle is not in place.</t>
+          <t xml:space="preserve">Error E01</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t xml:space="preserve">哺乳瓶がセットされていません。</t>
+          <t xml:space="preserve">Error E01</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶瓶未就位。</t>
+          <t xml:space="preserve">Error E01</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶瓶未就位。</t>
+          <t xml:space="preserve">Error E01</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle is not in place.</t>
+          <t xml:space="preserve">Error E01</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle is not in place.</t>
+          <t xml:space="preserve">Error E01</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t xml:space="preserve">sensor_watertank_missing</t>
+          <t xml:space="preserve">error_e02</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank is missing or water level is too low.</t>
+          <t xml:space="preserve">Error E02</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱が未装着、または水量不足です。</t>
+          <t xml:space="preserve">Error E02</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱未安装或水量不足。</t>
+          <t xml:space="preserve">Error E02</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱未安裝或水量不足。</t>
+          <t xml:space="preserve">Error E02</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank is missing or water level is too low.</t>
+          <t xml:space="preserve">Error E02</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank is missing or water level is too low.</t>
+          <t xml:space="preserve">Error E02</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_check_toast</t>
+          <t xml:space="preserve">error_e03</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before brewing.</t>
+          <t xml:space="preserve">Error E03</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t xml:space="preserve">調乳前にデバイス状態を確認してください。</t>
+          <t xml:space="preserve">エラー E03</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t xml:space="preserve">冲奶前请先检查设备状态。</t>
+          <t xml:space="preserve">错误 E03</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t xml:space="preserve">沖奶前請先檢查設備狀態。</t>
+          <t xml:space="preserve">錯誤 E03</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before brewing.</t>
+          <t xml:space="preserve">Error E03</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before brewing.</t>
+          <t xml:space="preserve">Error E03</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_check_toast_water</t>
+          <t xml:space="preserve">error_c01</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before water dispensing.</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t xml:space="preserve">出水前にデバイス状態を確認してください。</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t xml:space="preserve">出水前请先检查设备状态。</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t xml:space="preserve">出水前請先檢查設備狀態。</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before water dispensing.</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before water dispensing.</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_check_toast_powder</t>
+          <t xml:space="preserve">error_c02</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before formula dispensing.</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t xml:space="preserve">出粉前にデバイス状態を確認してください。</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t xml:space="preserve">出粉前请先检查设备状态。</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t xml:space="preserve">出粉前請先檢查設備狀態。</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before formula dispensing.</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before formula dispensing.</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_panel_title</t>
+          <t xml:space="preserve">error_c03</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t xml:space="preserve">Formula brewing is unavailable.</t>
+          <t xml:space="preserve">Error C03</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t xml:space="preserve">調乳を開始できません。</t>
+          <t xml:space="preserve">エラー C03</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t xml:space="preserve">无法开始冲奶。</t>
+          <t xml:space="preserve">错误 C03</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t xml:space="preserve">無法開始沖奶。</t>
+          <t xml:space="preserve">錯誤 C03</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t xml:space="preserve">Formula brewing is unavailable.</t>
+          <t xml:space="preserve">Error C03</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t xml:space="preserve">Formula brewing is unavailable.</t>
+          <t xml:space="preserve">Error C03</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_panel_subtitle</t>
+          <t xml:space="preserve">error_c04</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t xml:space="preserve">Please make sure all the following device assemblies are fully prepared.</t>
+          <t xml:space="preserve">Error C04</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t xml:space="preserve">以下の装置がすべて正しく準備されていることを確認してください。</t>
+          <t xml:space="preserve">エラー C04</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t xml:space="preserve">请确认以下装置均已正确准备就绪。</t>
+          <t xml:space="preserve">错误 C04</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t xml:space="preserve">請確認以下裝置均已正確準備就緒。</t>
+          <t xml:space="preserve">錯誤 C04</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t xml:space="preserve">Please make sure all the following device assemblies are fully prepared.</t>
+          <t xml:space="preserve">Error C04</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t xml:space="preserve">Please make sure all the following device assemblies are fully prepared.</t>
+          <t xml:space="preserve">Error C04</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_mixing_chamber</t>
+          <t xml:space="preserve">sensor_milkbox_missing</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixing chamber installed</t>
+          <t xml:space="preserve">Powder box is not installed.</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミキシングチャンバー装着済み</t>
+          <t xml:space="preserve">粉ミルクボックスが装着されていません。</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t xml:space="preserve">混合舱已安装</t>
+          <t xml:space="preserve">奶粉盒未安装。</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t xml:space="preserve">混合艙已安裝</t>
+          <t xml:space="preserve">奶粉盒未安裝。</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixing chamber installed</t>
+          <t xml:space="preserve">Powder box is not installed.</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixing chamber installed</t>
+          <t xml:space="preserve">Powder box is not installed.</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_water_tank</t>
+          <t xml:space="preserve">sensor_funnel_missing</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank installed</t>
+          <t xml:space="preserve">Funnel is not installed.</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱装着済み</t>
+          <t xml:space="preserve">ファネルが装着されていません。</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱已安装</t>
+          <t xml:space="preserve">漏斗未安装。</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱已安裝</t>
+          <t xml:space="preserve">漏斗未安裝。</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank installed</t>
+          <t xml:space="preserve">Funnel is not installed.</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank installed</t>
+          <t xml:space="preserve">Funnel is not installed.</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_water_level</t>
+          <t xml:space="preserve">sensor_bottle_missing</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sufficient water level</t>
+          <t xml:space="preserve">Bottle is not in place.</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量十分</t>
+          <t xml:space="preserve">哺乳瓶がセットされていません。</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量充足</t>
+          <t xml:space="preserve">奶瓶未就位。</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量充足</t>
+          <t xml:space="preserve">奶瓶未就位。</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sufficient water level</t>
+          <t xml:space="preserve">Bottle is not in place.</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sufficient water level</t>
+          <t xml:space="preserve">Bottle is not in place.</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_milk_powder</t>
+          <t xml:space="preserve">sensor_watertank_missing</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk powder container installed</t>
+          <t xml:space="preserve">Water tank is missing or water level is too low.</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルク容器装着済み</t>
+          <t xml:space="preserve">水箱が未装着、または水量不足です。</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉盒已安装</t>
+          <t xml:space="preserve">水箱未安装或水量不足。</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉盒已安裝</t>
+          <t xml:space="preserve">水箱未安裝或水量不足。</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk powder container installed</t>
+          <t xml:space="preserve">Water tank is missing or water level is too low.</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk powder container installed</t>
+          <t xml:space="preserve">Water tank is missing or water level is too low.</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_bottle</t>
+          <t xml:space="preserve">device_status_check_toast</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle in place</t>
+          <t xml:space="preserve">Check device status before brewing.</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t xml:space="preserve">哺乳瓶セット済み</t>
+          <t xml:space="preserve">調乳前にデバイス状態を確認してください。</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶瓶已就位</t>
+          <t xml:space="preserve">冲奶前请先检查设备状态。</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶瓶已就位</t>
+          <t xml:space="preserve">沖奶前請先檢查設備狀態。</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle in place</t>
+          <t xml:space="preserve">Check device status before brewing.</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle in place</t>
+          <t xml:space="preserve">Check device status before brewing.</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_no_blockage</t>
+          <t xml:space="preserve">device_status_check_toast_water</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t xml:space="preserve">No blockage detected</t>
+          <t xml:space="preserve">Check device status before water dispensing.</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t xml:space="preserve">詰まりなし</t>
+          <t xml:space="preserve">出水前にデバイス状態を確認してください。</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t xml:space="preserve">未检测到堵塞</t>
+          <t xml:space="preserve">出水前请先检查设备状态。</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t xml:space="preserve">未偵測到堵塞</t>
+          <t xml:space="preserve">出水前請先檢查設備狀態。</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t xml:space="preserve">No blockage detected</t>
+          <t xml:space="preserve">Check device status before water dispensing.</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t xml:space="preserve">No blockage detected</t>
+          <t xml:space="preserve">Check device status before water dispensing.</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_water_low_toast</t>
+          <t xml:space="preserve">device_status_check_toast_powder</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank low, please refill promptly!</t>
+          <t xml:space="preserve">Check device status before formula dispensing.</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱の水量が不足しています。すぐに補充してください。</t>
+          <t xml:space="preserve">出粉前にデバイス状態を確認してください。</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱水量不足，请尽快加水。</t>
+          <t xml:space="preserve">出粉前请先检查设备状态。</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱水量不足，請盡快加水。</t>
+          <t xml:space="preserve">出粉前請先檢查設備狀態。</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank low, please refill promptly!</t>
+          <t xml:space="preserve">Check device status before formula dispensing.</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank low, please refill promptly!</t>
+          <t xml:space="preserve">Check device status before formula dispensing.</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_temp_unavailable_toast</t>
+          <t xml:space="preserve">device_status_panel_title</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t xml:space="preserve">Temperature setting unavailable! Please wait for temperature recovery or adjust tank temp to retry.</t>
+          <t xml:space="preserve">Formula brewing is unavailable.</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t xml:space="preserve">温度設定が利用できません。温度が回復するまでお待ちいただくか、水箱の温度を調整してから再試行してください。</t>
+          <t xml:space="preserve">調乳を開始できません。</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t xml:space="preserve">温度设定不可用！请等待温度恢复或调整水箱温度后重试。</t>
+          <t xml:space="preserve">无法开始冲奶。</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t xml:space="preserve">溫度設定不可用！請等待溫度恢復或調整水箱溫度後重試。</t>
+          <t xml:space="preserve">無法開始沖奶。</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t xml:space="preserve">Temperature setting unavailable! Please wait for temperature recovery or adjust tank temp to retry.</t>
+          <t xml:space="preserve">Formula brewing is unavailable.</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t xml:space="preserve">Temperature setting unavailable! Please wait for temperature recovery or adjust tank temp to retry.</t>
+          <t xml:space="preserve">Formula brewing is unavailable.</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t xml:space="preserve">brand_coming_soon</t>
+          <t xml:space="preserve">device_status_panel_subtitle</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand settings will be available in a future update.</t>
+          <t xml:space="preserve">Please make sure all the following device assemblies are fully prepared.</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランド設定は今後のアップデートで提供予定です。</t>
+          <t xml:space="preserve">以下の装置がすべて正しく準備されていることを確認してください。</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t xml:space="preserve">品牌设置将在后续版本中提供。</t>
+          <t xml:space="preserve">请确认以下装置均已正确准备就绪。</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t xml:space="preserve">品牌設定將在後續版本中提供。</t>
+          <t xml:space="preserve">請確認以下裝置均已正確準備就緒。</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand settings will be available in a future update.</t>
+          <t xml:space="preserve">Please make sure all the following device assemblies are fully prepared.</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand settings will be available in a future update.</t>
+          <t xml:space="preserve">Please make sure all the following device assemblies are fully prepared.</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_page_title</t>
+          <t xml:space="preserve">device_status_mixing_chamber</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Milk Powder Brand</t>
+          <t xml:space="preserve">Mixing chamber installed</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルクブランドを追加</t>
+          <t xml:space="preserve">ミキシングチャンバー装着済み</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t xml:space="preserve">添加奶粉品牌</t>
+          <t xml:space="preserve">混合舱已安装</t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t xml:space="preserve">新增奶粉品牌</t>
+          <t xml:space="preserve">混合艙已安裝</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Milk Powder Brand</t>
+          <t xml:space="preserve">Mixing chamber installed</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Milk Powder Brand</t>
+          <t xml:space="preserve">Mixing chamber installed</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_edit_page_title</t>
+          <t xml:space="preserve">device_status_water_tank</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edit Milk Powder Brand</t>
+          <t xml:space="preserve">Water tank installed</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルクブランドを編集</t>
+          <t xml:space="preserve">水箱装着済み</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t xml:space="preserve">编辑奶粉品牌</t>
+          <t xml:space="preserve">水箱已安装</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t xml:space="preserve">編輯奶粉品牌</t>
+          <t xml:space="preserve">水箱已安裝</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edit Milk Powder Brand</t>
+          <t xml:space="preserve">Water tank installed</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edit Milk Powder Brand</t>
+          <t xml:space="preserve">Water tank installed</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_custom_ratio_section</t>
+          <t xml:space="preserve">device_status_water_level</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Ratio</t>
+          <t xml:space="preserve">Sufficient water level</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t xml:space="preserve">カスタム比率</t>
+          <t xml:space="preserve">水量十分</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t xml:space="preserve">自定义配比</t>
+          <t xml:space="preserve">水量充足</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t xml:space="preserve">自訂配比</t>
+          <t xml:space="preserve">水量充足</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Ratio</t>
+          <t xml:space="preserve">Sufficient water level</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Ratio</t>
+          <t xml:space="preserve">Sufficient water level</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_page_note</t>
+          <t xml:space="preserve">device_status_milk_powder</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
+          <t xml:space="preserve">Milk powder container installed</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t xml:space="preserve">注意：ブランド・シリーズ・段階を選択すると、対応する粉ミルク濃度を自動取得し、調乳比率を表示します。</t>
+          <t xml:space="preserve">粉ミルク容器装着済み</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t xml:space="preserve">说明：选择品牌、系列和段数后，将自动获取对应奶粉浓度并计算、展示冲调比例。</t>
+          <t xml:space="preserve">奶粉盒已安装</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t xml:space="preserve">說明：選擇品牌、系列與段數後，將自動取得對應奶粉濃度並計算、顯示沖調比例。</t>
+          <t xml:space="preserve">奶粉盒已安裝</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
+          <t xml:space="preserve">Milk powder container installed</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
+          <t xml:space="preserve">Milk powder container installed</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_info_title</t>
+          <t xml:space="preserve">device_status_bottle</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk Powder Info</t>
+          <t xml:space="preserve">Bottle in place</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルク情報</t>
+          <t xml:space="preserve">哺乳瓶セット済み</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉信息</t>
+          <t xml:space="preserve">奶瓶已就位</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉資訊</t>
+          <t xml:space="preserve">奶瓶已就位</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk Powder Info</t>
+          <t xml:space="preserve">Bottle in place</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk Powder Info</t>
+          <t xml:space="preserve">Bottle in place</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_select_brand</t>
+          <t xml:space="preserve">device_status_no_blockage</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand</t>
+          <t xml:space="preserve">No blockage detected</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランド</t>
+          <t xml:space="preserve">詰まりなし</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t xml:space="preserve">品牌</t>
+          <t xml:space="preserve">未检测到堵塞</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t xml:space="preserve">品牌</t>
+          <t xml:space="preserve">未偵測到堵塞</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand</t>
+          <t xml:space="preserve">No blockage detected</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand</t>
+          <t xml:space="preserve">No blockage detected</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_select_series</t>
+          <t xml:space="preserve">device_status_water_low_toast</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Water tank low, please refill promptly!</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t xml:space="preserve">シリーズ</t>
+          <t xml:space="preserve">水箱の水量が不足しています。すぐに補充してください。</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t xml:space="preserve">系列</t>
+          <t xml:space="preserve">水箱水量不足，请尽快加水。</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t xml:space="preserve">系列</t>
+          <t xml:space="preserve">水箱水量不足，請盡快加水。</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Water tank low, please refill promptly!</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Water tank low, please refill promptly!</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_select_stage</t>
+          <t xml:space="preserve">device_status_temp_unavailable_toast</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage</t>
+          <t xml:space="preserve">Temperature setting unavailable! Please wait for temperature recovery or adjust tank temp to retry.</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t xml:space="preserve">段階</t>
+          <t xml:space="preserve">温度設定が利用できません。温度が回復するまでお待ちいただくか、水箱の温度を調整してから再試行してください。</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t xml:space="preserve">段数</t>
+          <t xml:space="preserve">温度设定不可用！请等待温度恢复或调整水箱温度后重试。</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t xml:space="preserve">段數</t>
+          <t xml:space="preserve">溫度設定不可用！請等待溫度恢復或調整水箱溫度後重試。</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage</t>
+          <t xml:space="preserve">Temperature setting unavailable! Please wait for temperature recovery or adjust tank temp to retry.</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage</t>
+          <t xml:space="preserve">Temperature setting unavailable! Please wait for temperature recovery or adjust tank temp to retry.</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_select_placeholder</t>
+          <t xml:space="preserve">brand_coming_soon</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select</t>
+          <t xml:space="preserve">Brand settings will be available in a future update.</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t xml:space="preserve">選択</t>
+          <t xml:space="preserve">ブランド設定は今後のアップデートで提供予定です。</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t xml:space="preserve">请选择</t>
+          <t xml:space="preserve">品牌设置将在后续版本中提供。</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t xml:space="preserve">請選擇</t>
+          <t xml:space="preserve">品牌設定將在後續版本中提供。</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select</t>
+          <t xml:space="preserve">Brand settings will be available in a future update.</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select</t>
+          <t xml:space="preserve">Brand settings will be available in a future update.</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_sheet_select_brand</t>
+          <t xml:space="preserve">powder_brand_page_title</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Brand</t>
+          <t xml:space="preserve">Add Milk Powder Brand</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランドを選択</t>
+          <t xml:space="preserve">粉ミルクブランドを追加</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t xml:space="preserve">选择品牌</t>
+          <t xml:space="preserve">添加奶粉品牌</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t xml:space="preserve">選擇品牌</t>
+          <t xml:space="preserve">新增奶粉品牌</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Brand</t>
+          <t xml:space="preserve">Add Milk Powder Brand</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Brand</t>
+          <t xml:space="preserve">Add Milk Powder Brand</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_sheet_select_series</t>
+          <t xml:space="preserve">powder_brand_edit_page_title</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Series</t>
+          <t xml:space="preserve">Edit Milk Powder Brand</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t xml:space="preserve">シリーズを選択</t>
+          <t xml:space="preserve">粉ミルクブランドを編集</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t xml:space="preserve">选择系列</t>
+          <t xml:space="preserve">编辑奶粉品牌</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t xml:space="preserve">選擇系列</t>
+          <t xml:space="preserve">編輯奶粉品牌</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Series</t>
+          <t xml:space="preserve">Edit Milk Powder Brand</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Series</t>
+          <t xml:space="preserve">Edit Milk Powder Brand</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_sheet_select_stage</t>
+          <t xml:space="preserve">powder_brand_custom_ratio_section</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Stage</t>
+          <t xml:space="preserve">Custom Ratio</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t xml:space="preserve">段階を選択</t>
+          <t xml:space="preserve">カスタム比率</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t xml:space="preserve">选择段数</t>
+          <t xml:space="preserve">自定义配比</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t xml:space="preserve">選擇段數</t>
+          <t xml:space="preserve">自訂配比</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Stage</t>
+          <t xml:space="preserve">Custom Ratio</t>
         </is>
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Stage</t>
+          <t xml:space="preserve">Custom Ratio</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_search_placeholder</t>
+          <t xml:space="preserve">powder_brand_page_note</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t xml:space="preserve">Search brand...</t>
+          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランドを検索...</t>
+          <t xml:space="preserve">注意：ブランド・シリーズ・段階を選択すると、対応する粉ミルク濃度を自動取得し、調乳比率を表示します。</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t xml:space="preserve">搜索品牌...</t>
+          <t xml:space="preserve">说明：选择品牌、系列和段数后，将自动获取对应奶粉浓度并计算、展示冲调比例。</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t xml:space="preserve">搜尋品牌...</t>
+          <t xml:space="preserve">說明：選擇品牌、系列與段數後，將自動取得對應奶粉濃度並計算、顯示沖調比例。</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t xml:space="preserve">Search brand...</t>
+          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t xml:space="preserve">Search brand...</t>
+          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_search_empty</t>
+          <t xml:space="preserve">powder_brand_info_title</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t xml:space="preserve">No brands match your search.</t>
+          <t xml:space="preserve">Milk Powder Info</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t xml:space="preserve">該当するブランドがありません。</t>
+          <t xml:space="preserve">粉ミルク情報</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t xml:space="preserve">未找到匹配的品牌。</t>
+          <t xml:space="preserve">奶粉信息</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t xml:space="preserve">找不到符合的品牌。</t>
+          <t xml:space="preserve">奶粉資訊</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t xml:space="preserve">No brands match your search.</t>
+          <t xml:space="preserve">Milk Powder Info</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t xml:space="preserve">No brands match your search.</t>
+          <t xml:space="preserve">Milk Powder Info</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_not_listed</t>
+          <t xml:space="preserve">powder_brand_select_brand</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand not listed? </t>
+          <t xml:space="preserve">Brand</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランドが見つかりませんか？ </t>
+          <t xml:space="preserve">ブランド</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t xml:space="preserve">没有您的品牌？ </t>
+          <t xml:space="preserve">品牌</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t xml:space="preserve">找不到您的品牌？ </t>
+          <t xml:space="preserve">品牌</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand not listed? </t>
+          <t xml:space="preserve">Brand</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand not listed? </t>
+          <t xml:space="preserve">Brand</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_customize_ratio</t>
+          <t xml:space="preserve">powder_brand_select_series</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t xml:space="preserve">Customize mixing ratio.</t>
+          <t xml:space="preserve">Series</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミックス比率をカスタマイズ</t>
+          <t xml:space="preserve">シリーズ</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t xml:space="preserve">自定义配比</t>
+          <t xml:space="preserve">系列</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t xml:space="preserve">自訂配比</t>
+          <t xml:space="preserve">系列</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t xml:space="preserve">Customize mixing ratio.</t>
+          <t xml:space="preserve">Series</t>
         </is>
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t xml:space="preserve">Customize mixing ratio.</t>
+          <t xml:space="preserve">Series</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_custom_label</t>
+          <t xml:space="preserve">powder_brand_select_stage</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom</t>
+          <t xml:space="preserve">Stage</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t xml:space="preserve">カスタム</t>
+          <t xml:space="preserve">段階</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t xml:space="preserve">自定义</t>
+          <t xml:space="preserve">段数</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t xml:space="preserve">自訂</t>
+          <t xml:space="preserve">段數</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom</t>
+          <t xml:space="preserve">Stage</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom</t>
+          <t xml:space="preserve">Stage</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_custom_water_ml</t>
+          <t xml:space="preserve">powder_brand_select_placeholder</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water (mL)</t>
+          <t xml:space="preserve">Select</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量 (mL)</t>
+          <t xml:space="preserve">選択</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量 (mL)</t>
+          <t xml:space="preserve">请选择</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量 (mL)</t>
+          <t xml:space="preserve">請選擇</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water (mL)</t>
+          <t xml:space="preserve">Select</t>
         </is>
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water (mL)</t>
+          <t xml:space="preserve">Select</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_custom_powder_g</t>
+          <t xml:space="preserve">powder_brand_sheet_select_brand</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder (g)</t>
+          <t xml:space="preserve">Select Brand</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉量 (g)</t>
+          <t xml:space="preserve">ブランドを選択</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉量 (g)</t>
+          <t xml:space="preserve">选择品牌</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉量 (g)</t>
+          <t xml:space="preserve">選擇品牌</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder (g)</t>
+          <t xml:space="preserve">Select Brand</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder (g)</t>
+          <t xml:space="preserve">Select Brand</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_custom_apply</t>
+          <t xml:space="preserve">powder_brand_sheet_select_series</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apply</t>
+          <t xml:space="preserve">Select Series</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t xml:space="preserve">適用</t>
+          <t xml:space="preserve">シリーズを選択</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t xml:space="preserve">应用</t>
+          <t xml:space="preserve">选择系列</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t xml:space="preserve">套用</t>
+          <t xml:space="preserve">選擇系列</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apply</t>
+          <t xml:space="preserve">Select Series</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apply</t>
+          <t xml:space="preserve">Select Series</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_ratio_title</t>
+          <t xml:space="preserve">powder_brand_sheet_select_stage</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recommended Mix Ratio</t>
+          <t xml:space="preserve">Select Stage</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t xml:space="preserve">推奨ミックス比率</t>
+          <t xml:space="preserve">段階を選択</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t xml:space="preserve">推荐配比</t>
+          <t xml:space="preserve">选择段数</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t xml:space="preserve">建議配比</t>
+          <t xml:space="preserve">選擇段數</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recommended Mix Ratio</t>
+          <t xml:space="preserve">Select Stage</t>
         </is>
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recommended Mix Ratio</t>
+          <t xml:space="preserve">Select Stage</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_ratio_water</t>
+          <t xml:space="preserve">powder_brand_search_placeholder</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water</t>
+          <t xml:space="preserve">Search brand...</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t xml:space="preserve">水</t>
+          <t xml:space="preserve">ブランドを検索...</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t xml:space="preserve">水</t>
+          <t xml:space="preserve">搜索品牌...</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t xml:space="preserve">水</t>
+          <t xml:space="preserve">搜尋品牌...</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water</t>
+          <t xml:space="preserve">Search brand...</t>
         </is>
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water</t>
+          <t xml:space="preserve">Search brand...</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_ratio_powder</t>
+          <t xml:space="preserve">powder_brand_search_empty</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder</t>
+          <t xml:space="preserve">No brands match your search.</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルク</t>
+          <t xml:space="preserve">該当するブランドがありません。</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉</t>
+          <t xml:space="preserve">未找到匹配的品牌。</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉</t>
+          <t xml:space="preserve">找不到符合的品牌。</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder</t>
+          <t xml:space="preserve">No brands match your search.</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder</t>
+          <t xml:space="preserve">No brands match your search.</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_settings_title</t>
+          <t xml:space="preserve">powder_brand_not_listed</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder Brand Settings</t>
+          <t xml:space="preserve">Brand not listed? </t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルクブランド設定</t>
+          <t xml:space="preserve">ブランドが見つかりませんか？ </t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉品牌设置</t>
+          <t xml:space="preserve">没有您的品牌？ </t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉品牌設定</t>
+          <t xml:space="preserve">找不到您的品牌？ </t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder Brand Settings</t>
+          <t xml:space="preserve">Brand not listed? </t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder Brand Settings</t>
+          <t xml:space="preserve">Brand not listed? </t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_add_brand</t>
+          <t xml:space="preserve">powder_brand_customize_ratio</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Brand</t>
+          <t xml:space="preserve">Customize mixing ratio.</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランドを追加</t>
+          <t xml:space="preserve">ミックス比率をカスタマイズ</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t xml:space="preserve">添加品牌</t>
+          <t xml:space="preserve">自定义配比</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t xml:space="preserve">新增品牌</t>
+          <t xml:space="preserve">自訂配比</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Brand</t>
+          <t xml:space="preserve">Customize mixing ratio.</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Brand</t>
+          <t xml:space="preserve">Customize mixing ratio.</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_empty_message</t>
+          <t xml:space="preserve">powder_brand_custom_label</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t xml:space="preserve">No milk powder brands added yet.</t>
+          <t xml:space="preserve">Custom</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルクブランドはまだ追加されていません。</t>
+          <t xml:space="preserve">カスタム</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t xml:space="preserve">尚未添加奶粉品牌。</t>
+          <t xml:space="preserve">自定义</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t xml:space="preserve">尚未新增奶粉品牌。</t>
+          <t xml:space="preserve">自訂</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t xml:space="preserve">No milk powder brands added yet.</t>
+          <t xml:space="preserve">Custom</t>
         </is>
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t xml:space="preserve">No milk powder brands added yet.</t>
+          <t xml:space="preserve">Custom</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_batch_delete</t>
+          <t xml:space="preserve">powder_brand_custom_water_ml</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t xml:space="preserve">Batch Delete</t>
+          <t xml:space="preserve">Water (mL)</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t xml:space="preserve">一括削除</t>
+          <t xml:space="preserve">水量 (mL)</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t xml:space="preserve">批量删除</t>
+          <t xml:space="preserve">水量 (mL)</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t xml:space="preserve">批次刪除</t>
+          <t xml:space="preserve">水量 (mL)</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t xml:space="preserve">Batch Delete</t>
+          <t xml:space="preserve">Water (mL)</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t xml:space="preserve">Batch Delete</t>
+          <t xml:space="preserve">Water (mL)</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_batch_footer_delete</t>
+          <t xml:space="preserve">powder_brand_custom_powder_g</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete ({0})</t>
+          <t xml:space="preserve">Powder (g)</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete ({0})</t>
+          <t xml:space="preserve">粉量 (g)</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete ({0})</t>
+          <t xml:space="preserve">粉量 (g)</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete ({0})</t>
+          <t xml:space="preserve">粉量 (g)</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete ({0})</t>
+          <t xml:space="preserve">Powder (g)</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete ({0})</t>
+          <t xml:space="preserve">Powder (g)</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_batch_confirm_message_one</t>
+          <t xml:space="preserve">powder_brand_custom_apply</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+          <t xml:space="preserve">Apply</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+          <t xml:space="preserve">適用</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+          <t xml:space="preserve">应用</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+          <t xml:space="preserve">套用</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+          <t xml:space="preserve">Apply</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+          <t xml:space="preserve">Apply</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_batch_confirm_message_many</t>
+          <t xml:space="preserve">powder_brand_ratio_title</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+          <t xml:space="preserve">Recommended Mix Ratio</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+          <t xml:space="preserve">推奨ミックス比率</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+          <t xml:space="preserve">推荐配比</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+          <t xml:space="preserve">建議配比</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+          <t xml:space="preserve">Recommended Mix Ratio</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+          <t xml:space="preserve">Recommended Mix Ratio</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_batch_delete_title</t>
+          <t xml:space="preserve">powder_brand_ratio_water</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete Selected Brands?</t>
+          <t xml:space="preserve">Water</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t xml:space="preserve">選択したブランドを削除しますか？</t>
+          <t xml:space="preserve">水</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t xml:space="preserve">删除所选品牌？</t>
+          <t xml:space="preserve">水</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t xml:space="preserve">刪除所選品牌？</t>
+          <t xml:space="preserve">水</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete Selected Brands?</t>
+          <t xml:space="preserve">Water</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete Selected Brands?</t>
+          <t xml:space="preserve">Water</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_batch_delete_body</t>
+          <t xml:space="preserve">powder_brand_ratio_powder</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
+          <t xml:space="preserve">Powder</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t xml:space="preserve">{0}件のブランドを削除しますか？元に戻せません。</t>
+          <t xml:space="preserve">粉ミルク</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t xml:space="preserve">将删除 {0} 个品牌，此操作无法撤销。</t>
+          <t xml:space="preserve">奶粉</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t xml:space="preserve">將刪除 {0} 筆品牌，此操作無法復原。</t>
+          <t xml:space="preserve">奶粉</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
+          <t xml:space="preserve">Powder</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
+          <t xml:space="preserve">Powder</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_delete_title</t>
+          <t xml:space="preserve">powder_brand_settings_title</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete Brand?</t>
+          <t xml:space="preserve">Powder Brand Settings</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランドを削除しますか？</t>
+          <t xml:space="preserve">粉ミルクブランド設定</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t xml:space="preserve">删除品牌？</t>
+          <t xml:space="preserve">奶粉品牌设置</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t xml:space="preserve">刪除品牌？</t>
+          <t xml:space="preserve">奶粉品牌設定</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete Brand?</t>
+          <t xml:space="preserve">Powder Brand Settings</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t xml:space="preserve">Delete Brand?</t>
+          <t xml:space="preserve">Powder Brand Settings</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_delete_body</t>
+          <t xml:space="preserve">powder_brand_add_brand</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t xml:space="preserve">This brand will be removed from your list.</t>
+          <t xml:space="preserve">Add Brand</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t xml:space="preserve">このブランドはリストから削除されます。</t>
+          <t xml:space="preserve">ブランドを追加</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t xml:space="preserve">此品牌将从列表中移除。</t>
+          <t xml:space="preserve">添加品牌</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t xml:space="preserve">此品牌將從列表中移除。</t>
+          <t xml:space="preserve">新增品牌</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t xml:space="preserve">This brand will be removed from your list.</t>
+          <t xml:space="preserve">Add Brand</t>
         </is>
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t xml:space="preserve">This brand will be removed from your list.</t>
+          <t xml:space="preserve">Add Brand</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
+          <t xml:space="preserve">powder_brand_empty_message</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No milk powder brands added yet.</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t xml:space="preserve">粉ミルクブランドはまだ追加されていません。</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t xml:space="preserve">尚未添加奶粉品牌。</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t xml:space="preserve">尚未新增奶粉品牌。</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No milk powder brands added yet.</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No milk powder brands added yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_delete</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Batch Delete</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">一括削除</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">批量删除</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">批次刪除</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Batch Delete</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Batch Delete</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_footer_delete</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete ({0})</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_confirm_message_one</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_confirm_message_many</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_delete_title</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Selected Brands?</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">選択したブランドを削除しますか？</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">删除所选品牌？</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">刪除所選品牌？</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Selected Brands?</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Selected Brands?</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_batch_delete_body</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{0}件のブランドを削除しますか？元に戻せません。</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t xml:space="preserve">将删除 {0} 个品牌，此操作无法撤销。</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t xml:space="preserve">將刪除 {0} 筆品牌，此操作無法復原。</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_delete_title</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Brand?</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ブランドを削除しますか？</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">删除品牌？</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">刪除品牌？</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Brand?</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Brand?</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">powder_brand_delete_body</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This brand will be removed from your list.</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">このブランドはリストから削除されます。</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">此品牌将从列表中移除。</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">此品牌將從列表中移除。</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This brand will be removed from your list.</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This brand will be removed from your list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
           <t xml:space="preserve">powder_brand_delete_confirm_message</t>
         </is>
       </c>
-      <c r="B284" t="inlineStr">
+      <c r="B293" t="inlineStr">
         <is>
           <t xml:space="preserve">Are you sure you want to delete the brand:
 "{0} / {1} / {2}"?</t>
         </is>
       </c>
-      <c r="C284" t="inlineStr">
+      <c r="C293" t="inlineStr">
         <is>
           <t xml:space="preserve">ブランドを削除してもよろしいですか：
 "{0} / {1} / {2}"？</t>
         </is>
       </c>
-      <c r="D284" t="inlineStr">
+      <c r="D293" t="inlineStr">
         <is>
           <t xml:space="preserve">确定要删除品牌：
 "{0} / {1} / {2}"吗？</t>
         </is>
       </c>
-      <c r="E284" t="inlineStr">
+      <c r="E293" t="inlineStr">
         <is>
           <t xml:space="preserve">確定要刪除品牌：
 "{0} / {1} / {2}"嗎？</t>
         </is>
       </c>
-      <c r="F284" t="inlineStr">
+      <c r="F293" t="inlineStr">
         <is>
           <t xml:space="preserve">Are you sure you want to delete the brand:
 "{0} / {1} / {2}"?</t>
         </is>
       </c>
-      <c r="G284" t="inlineStr">
+      <c r="G293" t="inlineStr">
         <is>
           <t xml:space="preserve">Are you sure you want to delete the brand:
 "{0} / {1} / {2}"?</t>
         </is>
       </c>
     </row>
-    <row r="285">
-      <c r="A285" t="inlineStr">
+    <row r="294">
+      <c r="A294" t="inlineStr">
         <is>
           <t xml:space="preserve">custom_mix_ratio_page_title</t>
         </is>
       </c>
-      <c r="B285" t="inlineStr">
+      <c r="B294" t="inlineStr">
         <is>
           <t xml:space="preserve">Customize Mixing Ratio</t>
         </is>
       </c>
-      <c r="C285" t="inlineStr">
+      <c r="C294" t="inlineStr">
         <is>
           <t xml:space="preserve">ミックス比率をカスタマイズ</t>
         </is>
       </c>
-      <c r="D285" t="inlineStr">
+      <c r="D294" t="inlineStr">
         <is>
           <t xml:space="preserve">自定义配比</t>
         </is>
       </c>
-      <c r="E285" t="inlineStr">
+      <c r="E294" t="inlineStr">
         <is>
           <t xml:space="preserve">自訂配比</t>
         </is>
       </c>
-      <c r="F285" t="inlineStr">
+      <c r="F294" t="inlineStr">
         <is>
           <t xml:space="preserve">Customize Mixing Ratio</t>
         </is>
       </c>
-      <c r="G285" t="inlineStr">
+      <c r="G294" t="inlineStr">
         <is>
           <t xml:space="preserve">Customize Mixing Ratio</t>
         </is>
       </c>
     </row>
-    <row r="286">
-      <c r="A286" t="inlineStr">
+    <row r="295">
+      <c r="A295" t="inlineStr">
         <is>
           <t xml:space="preserve">custom_mix_ratio_note</t>
         </is>
       </c>
-      <c r="B286" t="inlineStr">
+      <c r="B295" t="inlineStr">
         <is>
           <t xml:space="preserve">Note: Once the mixing ratio is set, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
-      <c r="C286" t="inlineStr">
+      <c r="C295" t="inlineStr">
         <is>
           <t xml:space="preserve">注：ミックス比率を設定すると、対応する粉ミルク濃度を自動取得し、調乳比率を算出して表示します。</t>
         </is>
       </c>
-      <c r="D286" t="inlineStr">
+      <c r="D295" t="inlineStr">
         <is>
           <t xml:space="preserve">说明：设置配比后，系统将自动获取对应奶粉浓度，计算并展示冲调比例。</t>
         </is>
       </c>
-      <c r="E286" t="inlineStr">
+      <c r="E295" t="inlineStr">
         <is>
           <t xml:space="preserve">說明：設定配比後，系統將自動取得對應奶粉濃度，計算並顯示沖調比例。</t>
         </is>
       </c>
-      <c r="F286" t="inlineStr">
+      <c r="F295" t="inlineStr">
         <is>
           <t xml:space="preserve">Note: Once the mixing ratio is set, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
-      <c r="G286" t="inlineStr">
+      <c r="G295" t="inlineStr">
         <is>
           <t xml:space="preserve">Note: Once the mixing ratio is set, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
     </row>
-    <row r="287">
-      <c r="A287" t="inlineStr">
+    <row r="296">
+      <c r="A296" t="inlineStr">
         <is>
           <t xml:space="preserve">custom_mix_ratio_panel_title</t>
         </is>
       </c>
-      <c r="B287" t="inlineStr">
+      <c r="B296" t="inlineStr">
         <is>
           <t xml:space="preserve">Mix Ratio</t>
         </is>
       </c>
-      <c r="C287" t="inlineStr">
+      <c r="C296" t="inlineStr">
         <is>
           <t xml:space="preserve">ミックス比率</t>
         </is>
       </c>
-      <c r="D287" t="inlineStr">
+      <c r="D296" t="inlineStr">
         <is>
           <t xml:space="preserve">配比</t>
         </is>
       </c>
-      <c r="E287" t="inlineStr">
+      <c r="E296" t="inlineStr">
         <is>
           <t xml:space="preserve">配比</t>
         </is>
       </c>
-      <c r="F287" t="inlineStr">
+      <c r="F296" t="inlineStr">
         <is>
           <t xml:space="preserve">Mix Ratio</t>
         </is>
       </c>
-      <c r="G287" t="inlineStr">
+      <c r="G296" t="inlineStr">
         <is>
           <t xml:space="preserve">Mix Ratio</t>
         </is>
       </c>
     </row>
-    <row r="288">
-      <c r="A288" t="inlineStr">
+    <row r="297">
+      <c r="A297" t="inlineStr">
         <is>
           <t xml:space="preserve">custom_mix_ratio_incomplete</t>
         </is>
       </c>
-      <c r="B288" t="inlineStr">
+      <c r="B297" t="inlineStr">
         <is>
           <t xml:space="preserve">Please enter both water and powder amounts.</t>
         </is>
       </c>
-      <c r="C288" t="inlineStr">
+      <c r="C297" t="inlineStr">
         <is>
           <t xml:space="preserve">水量と粉量の両方を入力してください。</t>
         </is>
       </c>
-      <c r="D288" t="inlineStr">
+      <c r="D297" t="inlineStr">
         <is>
           <t xml:space="preserve">请填写水量和粉量。</t>
         </is>
       </c>
-      <c r="E288" t="inlineStr">
+      <c r="E297" t="inlineStr">
         <is>
           <t xml:space="preserve">請填寫水量與粉量。</t>
         </is>
       </c>
-      <c r="F288" t="inlineStr">
+      <c r="F297" t="inlineStr">
         <is>
           <t xml:space="preserve">Please enter both water and powder amounts.</t>
         </is>
       </c>
-      <c r="G288" t="inlineStr">
+      <c r="G297" t="inlineStr">
         <is>
           <t xml:space="preserve">Please enter both water and powder amounts.</t>
         </is>
       </c>
     </row>
-    <row r="289">
-      <c r="A289" t="inlineStr">
+    <row r="298">
+      <c r="A298" t="inlineStr">
         <is>
           <t xml:space="preserve">custom_mix_ratio_delete_confirm_message</t>
         </is>
       </c>
-      <c r="B289" t="inlineStr">
+      <c r="B298" t="inlineStr">
         <is>
           <t xml:space="preserve">Are you sure you want to delete the custom mixing ratio:
 "{0}ml / {1}g"?</t>
         </is>
       </c>
-      <c r="C289" t="inlineStr">
+      <c r="C298" t="inlineStr">
         <is>
           <t xml:space="preserve">カスタムミックス比率を削除してもよろしいですか：
 "{0}ml / {1}g"？</t>
         </is>
       </c>
-      <c r="D289" t="inlineStr">
+      <c r="D298" t="inlineStr">
         <is>
           <t xml:space="preserve">确定要删除自定义配比：
 "{0}ml / {1}g"吗？</t>
         </is>
       </c>
-      <c r="E289" t="inlineStr">
+      <c r="E298" t="inlineStr">
         <is>
           <t xml:space="preserve">確定要刪除自訂配比：
 "{0}ml / {1}g"嗎？</t>
         </is>
       </c>
-      <c r="F289" t="inlineStr">
+      <c r="F298" t="inlineStr">
         <is>
           <t xml:space="preserve">Are you sure you want to delete the custom mixing ratio:
 "{0}ml / {1}g"?</t>
         </is>
       </c>
-      <c r="G289" t="inlineStr">
+      <c r="G298" t="inlineStr">
         <is>
           <t xml:space="preserve">Are you sure you want to delete the custom mixing ratio:
 "{0}ml / {1}g"?</t>
         </is>
       </c>
     </row>
-    <row r="290">
-      <c r="A290" t="inlineStr">
+    <row r="299">
+      <c r="A299" t="inlineStr">
         <is>
           <t xml:space="preserve">dp_command_failed</t>
         </is>
       </c>
-      <c r="B290" t="inlineStr">
+      <c r="B299" t="inlineStr">
         <is>
           <t xml:space="preserve">Could not send the command. Check device connection.</t>
         </is>
       </c>
-      <c r="C290" t="inlineStr">
+      <c r="C299" t="inlineStr">
         <is>
           <t xml:space="preserve">コマンドを送信できませんでした。接続を確認してください。</t>
         </is>
       </c>
-      <c r="D290" t="inlineStr">
+      <c r="D299" t="inlineStr">
         <is>
           <t xml:space="preserve">无法发送指令，请检查设备连接。</t>
         </is>
       </c>
-      <c r="E290" t="inlineStr">
+      <c r="E299" t="inlineStr">
         <is>
           <t xml:space="preserve">無法傳送指令，請檢查裝置連線。</t>
         </is>
       </c>
-      <c r="F290" t="inlineStr">
+      <c r="F299" t="inlineStr">
         <is>
           <t xml:space="preserve">Could not send the command. Check device connection.</t>
         </is>
       </c>
-      <c r="G290" t="inlineStr">
+      <c r="G299" t="inlineStr">
         <is>
           <t xml:space="preserve">Could not send the command. Check device connection.</t>
         </is>
       </c>
     </row>
-    <row r="291">
-      <c r="A291" t="inlineStr">
+    <row r="300">
+      <c r="A300" t="inlineStr">
         <is>
           <t xml:space="preserve">device_power_off</t>
         </is>
       </c>
-      <c r="B291" t="inlineStr">
+      <c r="B300" t="inlineStr">
         <is>
           <t xml:space="preserve">Device is powered off. Tap the power button to turn on.</t>
         </is>
       </c>
-      <c r="C291" t="inlineStr">
+      <c r="C300" t="inlineStr">
         <is>
           <t xml:space="preserve">電源がオフです。電源ボタンをタップしてオンにしてください。</t>
         </is>
       </c>
-      <c r="D291" t="inlineStr">
+      <c r="D300" t="inlineStr">
         <is>
           <t xml:space="preserve">设备已关机，请点击电源键开机。</t>
         </is>
       </c>
-      <c r="E291" t="inlineStr">
+      <c r="E300" t="inlineStr">
         <is>
           <t xml:space="preserve">裝置已關機，請點擊電源鍵開機。</t>
         </is>
       </c>
-      <c r="F291" t="inlineStr">
+      <c r="F300" t="inlineStr">
         <is>
           <t xml:space="preserve">Device is powered off. Tap the power button to turn on.</t>
         </is>
       </c>
-      <c r="G291" t="inlineStr">
+      <c r="G300" t="inlineStr">
         <is>
           <t xml:space="preserve">Device is powered off. Tap the power button to turn on.</t>
         </is>
       </c>
     </row>
-    <row r="292">
-      <c r="A292" t="inlineStr">
+    <row r="301">
+      <c r="A301" t="inlineStr">
         <is>
           <t xml:space="preserve">device_settings_unavailable</t>
         </is>
       </c>
-      <c r="B292" t="inlineStr">
+      <c r="B301" t="inlineStr">
         <is>
           <t xml:space="preserve">Device settings are unavailable.</t>
         </is>
       </c>
-      <c r="C292" t="inlineStr">
+      <c r="C301" t="inlineStr">
         <is>
           <t xml:space="preserve">デバイス設定を開けません。</t>
         </is>
       </c>
-      <c r="D292" t="inlineStr">
+      <c r="D301" t="inlineStr">
         <is>
           <t xml:space="preserve">无法打开设备设置。</t>
         </is>
       </c>
-      <c r="E292" t="inlineStr">
+      <c r="E301" t="inlineStr">
         <is>
           <t xml:space="preserve">無法開啟裝置設定。</t>
         </is>
       </c>
-      <c r="F292" t="inlineStr">
+      <c r="F301" t="inlineStr">
         <is>
           <t xml:space="preserve">Device settings are unavailable.</t>
         </is>
       </c>
-      <c r="G292" t="inlineStr">
+      <c r="G301" t="inlineStr">
         <is>
           <t xml:space="preserve">Device settings are unavailable.</t>
         </is>
       </c>
     </row>
-    <row r="293">
-      <c r="A293" t="inlineStr">
+    <row r="302">
+      <c r="A302" t="inlineStr">
         <is>
           <t xml:space="preserve">device_settings_open_failed</t>
         </is>
       </c>
-      <c r="B293" t="inlineStr">
+      <c r="B302" t="inlineStr">
         <is>
           <t xml:space="preserve">Could not open device settings.</t>
         </is>
       </c>
-      <c r="C293" t="inlineStr">
+      <c r="C302" t="inlineStr">
         <is>
           <t xml:space="preserve">デバイス設定を開けませんでした。</t>
         </is>
       </c>
-      <c r="D293" t="inlineStr">
+      <c r="D302" t="inlineStr">
         <is>
           <t xml:space="preserve">无法打开设备设置页。</t>
         </is>
       </c>
-      <c r="E293" t="inlineStr">
+      <c r="E302" t="inlineStr">
         <is>
           <t xml:space="preserve">無法開啟裝置設定頁。</t>
         </is>
       </c>
-      <c r="F293" t="inlineStr">
+      <c r="F302" t="inlineStr">
         <is>
           <t xml:space="preserve">Could not open device settings.</t>
         </is>
       </c>
-      <c r="G293" t="inlineStr">
+      <c r="G302" t="inlineStr">
         <is>
           <t xml:space="preserve">Could not open device settings.</t>
         </is>

</xml_diff>

<commit_message>
refactor: clean home IA and stabilize panel boot
Move feeding record to the nav bottle icon and Smart Prep setup to a
dismissible snackbar, remove leftover pet/fan/guide assets, rebrand to
Smart Bottle Maker, and fix nav hit area plus React hook/lifecycle issues
on IDE boot.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/i18n_export.xlsx
+++ b/i18n_export.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G293"/>
+  <dimension ref="A1:G259"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6564,4302 +6564,3044 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t xml:space="preserve">volume_modal_title</t>
+          <t xml:space="preserve">feed_request_title</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water amount</t>
+          <t xml:space="preserve">Baby may be hungry!</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量設定</t>
+          <t xml:space="preserve">お腹がすいているかもしれません</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量设置</t>
+          <t xml:space="preserve">宝宝可能饿了</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量設定</t>
+          <t xml:space="preserve">寶寶可能餓了</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water amount</t>
+          <t xml:space="preserve">Baby may be hungry!</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water amount</t>
+          <t xml:space="preserve">Baby may be hungry!</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t xml:space="preserve">temp_modal_title</t>
+          <t xml:space="preserve">feed_request_subtitle</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t xml:space="preserve">Temperature</t>
+          <t xml:space="preserve">CryAssist detected your baby may be hungry. Start preparing a bottle with these settings, or adjust them first.</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t xml:space="preserve">温度設定</t>
+          <t xml:space="preserve">CryAssist が赤ちゃんの空腹を検知しました。この設定で調乳を開始するか、先に調整してください。</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t xml:space="preserve">温度设置</t>
+          <t xml:space="preserve">CryAssist 检测到宝宝可能饿了。可用以下设置开始冲奶，或先自行调整。</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t xml:space="preserve">溫度設定</t>
+          <t xml:space="preserve">哭聲翻譯偵測到寶寶可能飢餓。可用以下設定開始沖奶，或先自行調整。</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t xml:space="preserve">Temperature</t>
+          <t xml:space="preserve">CryAssist detected your baby may be hungry. Start preparing a bottle with these settings, or adjust them first.</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t xml:space="preserve">Temperature</t>
+          <t xml:space="preserve">CryAssist detected your baby may be hungry. Start preparing a bottle with these settings, or adjust them first.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t xml:space="preserve">feed_request_title</t>
+          <t xml:space="preserve">feed_request_start</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baby may be hungry!</t>
+          <t xml:space="preserve">Start Making</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t xml:space="preserve">お腹がすいているかもしれません</t>
+          <t xml:space="preserve">調乳を開始</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t xml:space="preserve">宝宝可能饿了</t>
+          <t xml:space="preserve">开始冲奶</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t xml:space="preserve">寶寶可能餓了</t>
+          <t xml:space="preserve">開始沖奶</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baby may be hungry!</t>
+          <t xml:space="preserve">Start Making</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baby may be hungry!</t>
+          <t xml:space="preserve">Start Making</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t xml:space="preserve">feed_request_subtitle</t>
+          <t xml:space="preserve">smart_prep_snackbar_setup</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t xml:space="preserve">CryAssist detected your baby may be hungry. Start preparing a bottle with these settings, or adjust them first.</t>
+          <t xml:space="preserve">Finish Smart Prep setup</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t xml:space="preserve">CryAssist が赤ちゃんの空腹を検知しました。この設定で調乳を開始するか、先に調整してください。</t>
+          <t xml:space="preserve">Smart Prep の設定を完了</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t xml:space="preserve">CryAssist 检测到宝宝可能饿了。可用以下设置开始冲奶，或先自行调整。</t>
+          <t xml:space="preserve">请完成 Smart Prep 设置</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t xml:space="preserve">哭聲翻譯偵測到寶寶可能飢餓。可用以下設定開始沖奶，或先自行調整。</t>
+          <t xml:space="preserve">請完成 Smart Prep 設定</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t xml:space="preserve">CryAssist detected your baby may be hungry. Start preparing a bottle with these settings, or adjust them first.</t>
+          <t xml:space="preserve">Finish Smart Prep setup</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t xml:space="preserve">CryAssist detected your baby may be hungry. Start preparing a bottle with these settings, or adjust them first.</t>
+          <t xml:space="preserve">Finish Smart Prep setup</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t xml:space="preserve">feed_request_body</t>
+          <t xml:space="preserve">block_none</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Maxi-Cosi CryAssist device reported Hungry. Confirm water, powder, and temperature on Smart Bottle Maker, then start making.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maxi-Cosi CryAssist 対応デバイスが Hungry を報告しました。Smart Bottle Maker で水量・粉量・温度を確認してから調乳を開始してください。</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maxi-Cosi CryAssist 设备回报 Hungry。请在 Smart Bottle Maker 确认水量、粉量和温度后开始冲奶。</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maxi-Cosi 哭聲翻譯設備回報飢餓。請在 Smart Bottle Maker 確認水量、粉量與溫度後開始沖奶。</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Maxi-Cosi CryAssist device reported Hungry. Confirm water, powder, and temperature on Smart Bottle Maker, then start making.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Maxi-Cosi CryAssist device reported Hungry. Confirm water, powder, and temperature on Smart Bottle Maker, then start making.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t xml:space="preserve">feed_request_start</t>
+          <t xml:space="preserve">block_water_tank_missing</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t xml:space="preserve">Start Making</t>
+          <t xml:space="preserve">Water tank is not installed.</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t xml:space="preserve">調乳を開始</t>
+          <t xml:space="preserve">水箱が装着されていません。</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t xml:space="preserve">开始冲奶</t>
+          <t xml:space="preserve">水箱未安装。</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t xml:space="preserve">開始沖奶</t>
+          <t xml:space="preserve">水箱未安裝。</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t xml:space="preserve">Start Making</t>
+          <t xml:space="preserve">Water tank is not installed.</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t xml:space="preserve">Start Making</t>
+          <t xml:space="preserve">Water tank is not installed.</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_activate_title</t>
+          <t xml:space="preserve">block_low_water</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enable Smart Prep reminder</t>
+          <t xml:space="preserve">Water level is too low.</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Prep リマインダーを有効にする</t>
+          <t xml:space="preserve">水量が不足しています。</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t xml:space="preserve">开启 Smart Prep 提醒</t>
+          <t xml:space="preserve">水量不足。</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t xml:space="preserve">啟用 Smart Prep 提醒</t>
+          <t xml:space="preserve">水量不足。</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enable Smart Prep reminder</t>
+          <t xml:space="preserve">Water level is too low.</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enable Smart Prep reminder</t>
+          <t xml:space="preserve">Water level is too low.</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_activate_body</t>
+          <t xml:space="preserve">block_powder_box_missing</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t xml:space="preserve">When a Maxi-Cosi CryAssist device detects your baby may be hungry, Smart Bottle Maker can remind you to prepare a bottle.</t>
+          <t xml:space="preserve">Powder box is not installed.</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maxi-Cosi CryAssist 対応デバイスが赤ちゃんの空腹を検知したとき、Smart Bottle Maker が調乳をお知らせできます。</t>
+          <t xml:space="preserve">粉ミルクボックスが装着されていません。</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t xml:space="preserve">当 Maxi-Cosi CryAssist 设备检测到宝宝可能饿了时，Smart Bottle Maker 可提醒您准备奶瓶。</t>
+          <t xml:space="preserve">奶粉盒未安装。</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t xml:space="preserve">當 Maxi-Cosi 哭聲翻譯設備偵測到寶寶可能飢餓時，Smart Bottle Maker 可提醒您準備奶瓶。</t>
+          <t xml:space="preserve">奶粉盒未安裝。</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t xml:space="preserve">When a Maxi-Cosi CryAssist device detects your baby may be hungry, Smart Bottle Maker can remind you to prepare a bottle.</t>
+          <t xml:space="preserve">Powder box is not installed.</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t xml:space="preserve">When a Maxi-Cosi CryAssist device detects your baby may be hungry, Smart Bottle Maker can remind you to prepare a bottle.</t>
+          <t xml:space="preserve">Powder box is not installed.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_enable_reminder</t>
+          <t xml:space="preserve">block_funnel_missing</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enable Reminder</t>
+          <t xml:space="preserve">Funnel is not installed.</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t xml:space="preserve">リマインダーを有効にする</t>
+          <t xml:space="preserve">ファネルが装着されていません。</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t xml:space="preserve">开启提醒</t>
+          <t xml:space="preserve">漏斗未安装。</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t xml:space="preserve">啟用提醒</t>
+          <t xml:space="preserve">漏斗未安裝。</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enable Reminder</t>
+          <t xml:space="preserve">Funnel is not installed.</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enable Reminder</t>
+          <t xml:space="preserve">Funnel is not installed.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_cry_detected_title</t>
+          <t xml:space="preserve">block_bottle_missing</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t xml:space="preserve">CryAssist device detected</t>
+          <t xml:space="preserve">Bottle is not in place.</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t xml:space="preserve">CryAssist デバイスを検出しました</t>
+          <t xml:space="preserve">哺乳瓶がセットされていません。</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t xml:space="preserve">检测到 CryAssist 设备</t>
+          <t xml:space="preserve">奶瓶未就位。</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t xml:space="preserve">偵測到哭聲翻譯設備</t>
+          <t xml:space="preserve">奶瓶未就位。</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t xml:space="preserve">CryAssist device detected</t>
+          <t xml:space="preserve">Bottle is not in place.</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t xml:space="preserve">CryAssist device detected</t>
+          <t xml:space="preserve">Bottle is not in place.</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_cry_detected_body</t>
+          <t xml:space="preserve">block_hot_alert</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Maxi-Cosi CryAssist device was found. Remind you to prepare a bottle when CryAssist Result is Hungry. Enable now?</t>
+          <t xml:space="preserve">Device is too hot. Please wait.</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maxi-Cosi CryAssist 対応デバイスが見つかりました。CryAssist Result が Hungry のときに調乳をお知らせします。今すぐ有効にしますか？</t>
+          <t xml:space="preserve">本体が高温です。しばらくお待ちください。</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t xml:space="preserve">已找到 Maxi-Cosi CryAssist 设备。当 CryAssist Result 为 Hungry 时可提醒冲奶。是否现在开启？</t>
+          <t xml:space="preserve">设备温度过高，请稍候。</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t xml:space="preserve">已找到 Maxi-Cosi 哭聲翻譯設備。當哭聲翻譯結果為飢餓時可提醒沖奶。是否現在開啟？</t>
+          <t xml:space="preserve">設備溫度過高，請稍候。</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Maxi-Cosi CryAssist device was found. Remind you to prepare a bottle when CryAssist Result is Hungry. Enable now?</t>
+          <t xml:space="preserve">Device is too hot. Please wait.</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t xml:space="preserve">A Maxi-Cosi CryAssist device was found. Remind you to prepare a bottle when CryAssist Result is Hungry. Enable now?</t>
+          <t xml:space="preserve">Device is too hot. Please wait.</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_enable_now</t>
+          <t xml:space="preserve">error_none</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enable</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t xml:space="preserve">有効にする</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t xml:space="preserve">开启</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t xml:space="preserve">開啟</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enable</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enable</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_later</t>
+          <t xml:space="preserve">error_hot</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t xml:space="preserve">Later</t>
+          <t xml:space="preserve">High temperature alert</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t xml:space="preserve">後で</t>
+          <t xml:space="preserve">High temperature alert</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t xml:space="preserve">稍后</t>
+          <t xml:space="preserve">High temperature alert</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t xml:space="preserve">稍後</t>
+          <t xml:space="preserve">High temperature alert</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t xml:space="preserve">Later</t>
+          <t xml:space="preserve">High temperature alert</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t xml:space="preserve">Later</t>
+          <t xml:space="preserve">High temperature alert</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_no_cry_device_title</t>
+          <t xml:space="preserve">error_e01</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t xml:space="preserve">No CryAssist device found</t>
+          <t xml:space="preserve">Error E01</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t xml:space="preserve">CryAssist デバイスが見つかりません</t>
+          <t xml:space="preserve">Error E01</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t xml:space="preserve">未找到 CryAssist 设备</t>
+          <t xml:space="preserve">Error E01</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t xml:space="preserve">未找到哭聲翻譯設備</t>
+          <t xml:space="preserve">Error E01</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t xml:space="preserve">No CryAssist device found</t>
+          <t xml:space="preserve">Error E01</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t xml:space="preserve">No CryAssist device found</t>
+          <t xml:space="preserve">Error E01</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_no_cry_device</t>
+          <t xml:space="preserve">error_e02</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Maxi-Cosi CryAssist device found in this home. You can set this up later in Routines.</t>
+          <t xml:space="preserve">Error E02</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t xml:space="preserve">このホームに Maxi-Cosi CryAssist 対応デバイスが見つかりません。後でルーティンから設定できます。</t>
+          <t xml:space="preserve">Error E02</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t xml:space="preserve">当前家庭未找到 Maxi-Cosi CryAssist 设备，可稍后在智能场景中设置。</t>
+          <t xml:space="preserve">Error E02</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t xml:space="preserve">目前家庭未找到 Maxi-Cosi 哭聲翻譯設備，可稍後在智慧場景中設定。</t>
+          <t xml:space="preserve">Error E02</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Maxi-Cosi CryAssist device found in this home. You can set this up later in Routines.</t>
+          <t xml:space="preserve">Error E02</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Maxi-Cosi CryAssist device found in this home. You can set this up later in Routines.</t>
+          <t xml:space="preserve">Error E02</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_setup_page_title</t>
+          <t xml:space="preserve">error_e03</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recommend Routine</t>
+          <t xml:space="preserve">Error E03</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t xml:space="preserve">おすすめルーティン</t>
+          <t xml:space="preserve">エラー E03</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t xml:space="preserve">推荐场景</t>
+          <t xml:space="preserve">错误 E03</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t xml:space="preserve">推薦場景</t>
+          <t xml:space="preserve">錯誤 E03</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recommend Routine</t>
+          <t xml:space="preserve">Error E03</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recommend Routine</t>
+          <t xml:space="preserve">Error E03</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_setup_title</t>
+          <t xml:space="preserve">error_c01</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Turn on Smart Prep reminder</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Prep リマインダーをオンにする</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t xml:space="preserve">开启 Smart Prep 提醒</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t xml:space="preserve">開啟 Smart Prep 提醒</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Turn on Smart Prep reminder</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Turn on Smart Prep reminder</t>
+          <t xml:space="preserve">Error C01</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_setup_desc</t>
+          <t xml:space="preserve">error_c02</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t xml:space="preserve">When a Maxi-Cosi CryAssist device reports Hungry, Smart Bottle Maker can remind you to prepare a bottle.</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maxi-Cosi CryAssist 対応デバイスが Hungry を報告すると、Smart Bottle Maker が調乳をお知らせできます。</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t xml:space="preserve">当 Maxi-Cosi CryAssist 设备回报 Hungry 时，Smart Bottle Maker 可提醒您准备奶瓶。</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t xml:space="preserve">當 Maxi-Cosi 哭聲翻譯設備回報飢餓時，Smart Bottle Maker 可提醒您準備奶瓶。</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t xml:space="preserve">When a Maxi-Cosi CryAssist device reports Hungry, Smart Bottle Maker can remind you to prepare a bottle.</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t xml:space="preserve">When a Maxi-Cosi CryAssist device reports Hungry, Smart Bottle Maker can remind you to prepare a bottle.</t>
+          <t xml:space="preserve">Error C02</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_setup_if_label</t>
+          <t xml:space="preserve">error_c03</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t xml:space="preserve">If</t>
+          <t xml:space="preserve">Error C03</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t xml:space="preserve">条件</t>
+          <t xml:space="preserve">エラー C03</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t xml:space="preserve">如果</t>
+          <t xml:space="preserve">错误 C03</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t xml:space="preserve">如果</t>
+          <t xml:space="preserve">錯誤 C03</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t xml:space="preserve">If</t>
+          <t xml:space="preserve">Error C03</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t xml:space="preserve">If</t>
+          <t xml:space="preserve">Error C03</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_setup_then_label</t>
+          <t xml:space="preserve">error_c04</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t xml:space="preserve">Then</t>
+          <t xml:space="preserve">Error C04</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t xml:space="preserve">実行</t>
+          <t xml:space="preserve">エラー C04</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t xml:space="preserve">那么</t>
+          <t xml:space="preserve">错误 C04</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t xml:space="preserve">執行</t>
+          <t xml:space="preserve">錯誤 C04</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t xml:space="preserve">Then</t>
+          <t xml:space="preserve">Error C04</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t xml:space="preserve">Then</t>
+          <t xml:space="preserve">Error C04</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_setup_if_detail</t>
+          <t xml:space="preserve">sensor_milkbox_missing</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maxi-Cosi CryAssist device</t>
+          <t xml:space="preserve">Powder box is not installed.</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maxi-Cosi CryAssist 対応デバイス</t>
+          <t xml:space="preserve">粉ミルクボックスが装着されていません。</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maxi-Cosi CryAssist 设备</t>
+          <t xml:space="preserve">奶粉盒未安装。</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maxi-Cosi 哭聲翻譯設備</t>
+          <t xml:space="preserve">奶粉盒未安裝。</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maxi-Cosi CryAssist device</t>
+          <t xml:space="preserve">Powder box is not installed.</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maxi-Cosi CryAssist device</t>
+          <t xml:space="preserve">Powder box is not installed.</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_setup_if_sub</t>
+          <t xml:space="preserve">sensor_funnel_missing</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t xml:space="preserve">CryAssist Result: Hungry</t>
+          <t xml:space="preserve">Funnel is not installed.</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t xml:space="preserve">CryAssist Result: Hungry</t>
+          <t xml:space="preserve">ファネルが装着されていません。</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t xml:space="preserve">CryAssist Result: Hungry</t>
+          <t xml:space="preserve">漏斗未安装。</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t xml:space="preserve">哭聲翻譯結果：飢餓</t>
+          <t xml:space="preserve">漏斗未安裝。</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t xml:space="preserve">CryAssist Result: Hungry</t>
+          <t xml:space="preserve">Funnel is not installed.</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t xml:space="preserve">CryAssist Result: Hungry</t>
+          <t xml:space="preserve">Funnel is not installed.</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_setup_then_detail</t>
+          <t xml:space="preserve">sensor_bottle_missing</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Bottle Maker</t>
+          <t xml:space="preserve">Bottle is not in place.</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Bottle Maker</t>
+          <t xml:space="preserve">哺乳瓶がセットされていません。</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Bottle Maker</t>
+          <t xml:space="preserve">奶瓶未就位。</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Bottle Maker</t>
+          <t xml:space="preserve">奶瓶未就位。</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Bottle Maker</t>
+          <t xml:space="preserve">Bottle is not in place.</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Bottle Maker</t>
+          <t xml:space="preserve">Bottle is not in place.</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_setup_then_sub</t>
+          <t xml:space="preserve">sensor_watertank_missing</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk prep reminder</t>
+          <t xml:space="preserve">Water tank is missing or water level is too low.</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t xml:space="preserve">調乳リマインダー</t>
+          <t xml:space="preserve">水箱が未装着、または水量不足です。</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t xml:space="preserve">冲奶提醒</t>
+          <t xml:space="preserve">水箱未安装或水量不足。</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t xml:space="preserve">沖奶提醒</t>
+          <t xml:space="preserve">水箱未安裝或水量不足。</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk prep reminder</t>
+          <t xml:space="preserve">Water tank is missing or water level is too low.</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk prep reminder</t>
+          <t xml:space="preserve">Water tank is missing or water level is too low.</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_setup_add</t>
+          <t xml:space="preserve">device_status_check_toast</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add</t>
+          <t xml:space="preserve">Check device status before brewing.</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t xml:space="preserve">追加</t>
+          <t xml:space="preserve">調乳前にデバイス状態を確認してください。</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t xml:space="preserve">添加</t>
+          <t xml:space="preserve">冲奶前请先检查设备状态。</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t xml:space="preserve">新增</t>
+          <t xml:space="preserve">沖奶前請先檢查設備狀態。</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add</t>
+          <t xml:space="preserve">Check device status before brewing.</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add</t>
+          <t xml:space="preserve">Check device status before brewing.</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_setup_added</t>
+          <t xml:space="preserve">device_status_check_toast_water</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Prep reminder enabled</t>
+          <t xml:space="preserve">Check device status before water dispensing.</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Prep リマインダーを有効にしました</t>
+          <t xml:space="preserve">出水前にデバイス状態を確認してください。</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Prep 提醒已开启</t>
+          <t xml:space="preserve">出水前请先检查设备状态。</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Prep 提醒已啟用</t>
+          <t xml:space="preserve">出水前請先檢查設備狀態。</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Prep reminder enabled</t>
+          <t xml:space="preserve">Check device status before water dispensing.</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Prep reminder enabled</t>
+          <t xml:space="preserve">Check device status before water dispensing.</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_opened_routines</t>
+          <t xml:space="preserve">device_status_check_toast_powder</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opened Routines. Follow the steps to finish setup.</t>
+          <t xml:space="preserve">Check device status before formula dispensing.</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t xml:space="preserve">ルーティンを開きました。手順に沿って設定を完了してください。</t>
+          <t xml:space="preserve">出粉前にデバイス状態を確認してください。</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t xml:space="preserve">已打开智能场景，请按步骤完成设置。</t>
+          <t xml:space="preserve">出粉前请先检查设备状态。</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t xml:space="preserve">已開啟智慧場景，請依步驟完成設定。</t>
+          <t xml:space="preserve">出粉前請先檢查設備狀態。</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opened Routines. Follow the steps to finish setup.</t>
+          <t xml:space="preserve">Check device status before formula dispensing.</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opened Routines. Follow the steps to finish setup.</t>
+          <t xml:space="preserve">Check device status before formula dispensing.</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_setup_failed</t>
+          <t xml:space="preserve">device_status_panel_title</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t xml:space="preserve">Could not open Routines. Try again from the App.</t>
+          <t xml:space="preserve">Formula brewing is unavailable.</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t xml:space="preserve">ルーティンを開けませんでした。App から再試行してください。</t>
+          <t xml:space="preserve">調乳を開始できません。</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t xml:space="preserve">无法打开智能场景，请从 App 重试。</t>
+          <t xml:space="preserve">无法开始冲奶。</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t xml:space="preserve">無法開啟智慧場景，請從 App 重試。</t>
+          <t xml:space="preserve">無法開始沖奶。</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t xml:space="preserve">Could not open Routines. Try again from the App.</t>
+          <t xml:space="preserve">Formula brewing is unavailable.</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t xml:space="preserve">Could not open Routines. Try again from the App.</t>
+          <t xml:space="preserve">Formula brewing is unavailable.</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_tutorial_title</t>
+          <t xml:space="preserve">device_status_panel_subtitle</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t xml:space="preserve">Set up Smart Prep Routine</t>
+          <t xml:space="preserve">Please make sure all the following device assemblies are fully prepared.</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Prep ルーティンを設定</t>
+          <t xml:space="preserve">以下の装置がすべて正しく準備されていることを確認してください。</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t xml:space="preserve">设置 Smart Prep 智能场景</t>
+          <t xml:space="preserve">请确认以下装置均已正确准备就绪。</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t xml:space="preserve">設定 Smart Prep 智慧場景</t>
+          <t xml:space="preserve">請確認以下裝置均已正確準備就緒。</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t xml:space="preserve">Set up Smart Prep Routine</t>
+          <t xml:space="preserve">Please make sure all the following device assemblies are fully prepared.</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t xml:space="preserve">Set up Smart Prep Routine</t>
+          <t xml:space="preserve">Please make sure all the following device assemblies are fully prepared.</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_tutorial_intro</t>
+          <t xml:space="preserve">device_status_mixing_chamber</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t xml:space="preserve">Create this Routine once in the App. Use these exact steps:</t>
+          <t xml:space="preserve">Mixing chamber installed</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t xml:space="preserve">App のルーティンで一度だけ設定します。次の手順に従ってください：</t>
+          <t xml:space="preserve">ミキシングチャンバー装着済み</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t xml:space="preserve">请在 App 的智能场景中完成一次设置，步骤如下：</t>
+          <t xml:space="preserve">混合舱已安装</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t xml:space="preserve">請在 App 的智慧場景中完成一次設定，步驟如下：</t>
+          <t xml:space="preserve">混合艙已安裝</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t xml:space="preserve">Create this Routine once in the App. Use these exact steps:</t>
+          <t xml:space="preserve">Mixing chamber installed</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t xml:space="preserve">Create this Routine once in the App. Use these exact steps:</t>
+          <t xml:space="preserve">Mixing chamber installed</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_tutorial_step_1</t>
+          <t xml:space="preserve">device_status_water_tank</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Create Routine → When device status changes</t>
+          <t xml:space="preserve">Water tank installed</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Create Routine → When device status changes</t>
+          <t xml:space="preserve">水箱装着済み</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. 创建智能场景 → 当设备状态变化时</t>
+          <t xml:space="preserve">水箱已安装</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. 建立智慧場景 → 當設備狀態改變時</t>
+          <t xml:space="preserve">水箱已安裝</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Create Routine → When device status changes</t>
+          <t xml:space="preserve">Water tank installed</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Create Routine → When device status changes</t>
+          <t xml:space="preserve">Water tank installed</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_tutorial_step_2</t>
+          <t xml:space="preserve">device_status_water_level</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. If: Maxi-Cosi CryAssist device → CryAssist Result → Hungry</t>
+          <t xml:space="preserve">Sufficient water level</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. If: Maxi-Cosi CryAssist device → CryAssist Result → Hungry</t>
+          <t xml:space="preserve">水量十分</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. 如果：Maxi-Cosi CryAssist 设备 → CryAssist 结果 → 饿了</t>
+          <t xml:space="preserve">水量充足</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. 如果：Maxi-Cosi 哭聲翻譯設備 → 哭聲翻譯結果 → 飢餓</t>
+          <t xml:space="preserve">水量充足</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. If: Maxi-Cosi CryAssist device → CryAssist Result → Hungry</t>
+          <t xml:space="preserve">Sufficient water level</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. If: Maxi-Cosi CryAssist device → CryAssist Result → Hungry</t>
+          <t xml:space="preserve">Sufficient water level</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_tutorial_step_3</t>
+          <t xml:space="preserve">device_status_milk_powder</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t xml:space="preserve">3. Then: Smart Bottle Maker → scene_feed_request → hungry_pending</t>
+          <t xml:space="preserve">Milk powder container installed</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t xml:space="preserve">3. Then: Smart Bottle Maker → scene_feed_request → hungry_pending</t>
+          <t xml:space="preserve">粉ミルク容器装着済み</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t xml:space="preserve">3. 那么：Smart Bottle Maker → scene_feed_request → hungry_pending</t>
+          <t xml:space="preserve">奶粉盒已安装</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t xml:space="preserve">3. 執行：Smart Bottle Maker → scene_feed_request → hungry_pending</t>
+          <t xml:space="preserve">奶粉盒已安裝</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t xml:space="preserve">3. Then: Smart Bottle Maker → scene_feed_request → hungry_pending</t>
+          <t xml:space="preserve">Milk powder container installed</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t xml:space="preserve">3. Then: Smart Bottle Maker → scene_feed_request → hungry_pending</t>
+          <t xml:space="preserve">Milk powder container installed</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_tutorial_step_4</t>
+          <t xml:space="preserve">device_status_bottle</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t xml:space="preserve">4. Name: Milk Prep Reminder → Save</t>
+          <t xml:space="preserve">Bottle in place</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t xml:space="preserve">4. Name: Milk Prep Reminder → Save</t>
+          <t xml:space="preserve">哺乳瓶セット済み</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t xml:space="preserve">4. 名称：Milk Prep Reminder → 保存</t>
+          <t xml:space="preserve">奶瓶已就位</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t xml:space="preserve">4. 名稱：Milk Prep Reminder → 儲存</t>
+          <t xml:space="preserve">奶瓶已就位</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t xml:space="preserve">4. Name: Milk Prep Reminder → Save</t>
+          <t xml:space="preserve">Bottle in place</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t xml:space="preserve">4. Name: Milk Prep Reminder → Save</t>
+          <t xml:space="preserve">Bottle in place</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_tutorial_done</t>
+          <t xml:space="preserve">device_status_no_blockage</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t xml:space="preserve">I've finished setup</t>
+          <t xml:space="preserve">No blockage detected</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t xml:space="preserve">設定済みにする</t>
+          <t xml:space="preserve">詰まりなし</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t xml:space="preserve">我已完成设置</t>
+          <t xml:space="preserve">未检测到堵塞</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t xml:space="preserve">我已完成設定</t>
+          <t xml:space="preserve">未偵測到堵塞</t>
         </is>
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t xml:space="preserve">I've finished setup</t>
+          <t xml:space="preserve">No blockage detected</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t xml:space="preserve">I've finished setup</t>
+          <t xml:space="preserve">No blockage detected</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_open_routines</t>
+          <t xml:space="preserve">device_status_water_low_toast</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open Routines</t>
+          <t xml:space="preserve">Water tank low, please refill promptly!</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t xml:space="preserve">ルーティンを開く</t>
+          <t xml:space="preserve">水箱の水量が不足しています。すぐに補充してください。</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t xml:space="preserve">打开智能场景</t>
+          <t xml:space="preserve">水箱水量不足，请尽快加水。</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t xml:space="preserve">開啟智慧場景</t>
+          <t xml:space="preserve">水箱水量不足，請盡快加水。</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open Routines</t>
+          <t xml:space="preserve">Water tank low, please refill promptly!</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open Routines</t>
+          <t xml:space="preserve">Water tank low, please refill promptly!</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_snackbar_setup</t>
+          <t xml:space="preserve">device_status_temp_unavailable_toast</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t xml:space="preserve">Finish Smart Prep setup</t>
+          <t xml:space="preserve">Temperature setting unavailable! Please wait for temperature recovery or adjust tank temp to retry.</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Prep の設定を完了</t>
+          <t xml:space="preserve">温度設定が利用できません。温度が回復するまでお待ちいただくか、水箱の温度を調整してから再試行してください。</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t xml:space="preserve">请完成 Smart Prep 设置</t>
+          <t xml:space="preserve">温度设定不可用！请等待温度恢复或调整水箱温度后重试。</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t xml:space="preserve">請完成 Smart Prep 設定</t>
+          <t xml:space="preserve">溫度設定不可用！請等待溫度恢復或調整水箱溫度後重試。</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t xml:space="preserve">Finish Smart Prep setup</t>
+          <t xml:space="preserve">Temperature setting unavailable! Please wait for temperature recovery or adjust tank temp to retry.</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t xml:space="preserve">Finish Smart Prep setup</t>
+          <t xml:space="preserve">Temperature setting unavailable! Please wait for temperature recovery or adjust tank temp to retry.</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t xml:space="preserve">smart_prep_marked_done</t>
+          <t xml:space="preserve">brand_coming_soon</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Prep reminder marked as set up</t>
+          <t xml:space="preserve">Brand settings will be available in a future update.</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Prep リマインダーを設定済みにしました</t>
+          <t xml:space="preserve">ブランド設定は今後のアップデートで提供予定です。</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t xml:space="preserve">已标记 Smart Prep 提醒设置完成</t>
+          <t xml:space="preserve">品牌设置将在后续版本中提供。</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t xml:space="preserve">已標記 Smart Prep 提醒設定完成</t>
+          <t xml:space="preserve">品牌設定將在後續版本中提供。</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Prep reminder marked as set up</t>
+          <t xml:space="preserve">Brand settings will be available in a future update.</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Prep reminder marked as set up</t>
+          <t xml:space="preserve">Brand settings will be available in a future update.</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t xml:space="preserve">block_none</t>
+          <t xml:space="preserve">powder_brand_page_title</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Add Milk Powder Brand</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">粉ミルクブランドを追加</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">添加奶粉品牌</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">新增奶粉品牌</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Add Milk Powder Brand</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Add Milk Powder Brand</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t xml:space="preserve">block_water_tank_missing</t>
+          <t xml:space="preserve">powder_brand_edit_page_title</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank is not installed.</t>
+          <t xml:space="preserve">Edit Milk Powder Brand</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱が装着されていません。</t>
+          <t xml:space="preserve">粉ミルクブランドを編集</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱未安装。</t>
+          <t xml:space="preserve">编辑奶粉品牌</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱未安裝。</t>
+          <t xml:space="preserve">編輯奶粉品牌</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank is not installed.</t>
+          <t xml:space="preserve">Edit Milk Powder Brand</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank is not installed.</t>
+          <t xml:space="preserve">Edit Milk Powder Brand</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t xml:space="preserve">block_low_water</t>
+          <t xml:space="preserve">powder_brand_custom_ratio_section</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water level is too low.</t>
+          <t xml:space="preserve">Custom Ratio</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量が不足しています。</t>
+          <t xml:space="preserve">カスタム比率</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量不足。</t>
+          <t xml:space="preserve">自定义配比</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量不足。</t>
+          <t xml:space="preserve">自訂配比</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water level is too low.</t>
+          <t xml:space="preserve">Custom Ratio</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water level is too low.</t>
+          <t xml:space="preserve">Custom Ratio</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t xml:space="preserve">block_powder_box_missing</t>
+          <t xml:space="preserve">powder_brand_page_note</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder box is not installed.</t>
+          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルクボックスが装着されていません。</t>
+          <t xml:space="preserve">注意：ブランド・シリーズ・段階を選択すると、対応する粉ミルク濃度を自動取得し、調乳比率を表示します。</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉盒未安装。</t>
+          <t xml:space="preserve">说明：选择品牌、系列和段数后，将自动获取对应奶粉浓度并计算、展示冲调比例。</t>
         </is>
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉盒未安裝。</t>
+          <t xml:space="preserve">說明：選擇品牌、系列與段數後，將自動取得對應奶粉濃度並計算、顯示沖調比例。</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder box is not installed.</t>
+          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder box is not installed.</t>
+          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t xml:space="preserve">block_funnel_missing</t>
+          <t xml:space="preserve">powder_brand_info_title</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Funnel is not installed.</t>
+          <t xml:space="preserve">Milk Powder Info</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t xml:space="preserve">ファネルが装着されていません。</t>
+          <t xml:space="preserve">粉ミルク情報</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t xml:space="preserve">漏斗未安装。</t>
+          <t xml:space="preserve">奶粉信息</t>
         </is>
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t xml:space="preserve">漏斗未安裝。</t>
+          <t xml:space="preserve">奶粉資訊</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Funnel is not installed.</t>
+          <t xml:space="preserve">Milk Powder Info</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Funnel is not installed.</t>
+          <t xml:space="preserve">Milk Powder Info</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t xml:space="preserve">block_bottle_missing</t>
+          <t xml:space="preserve">powder_brand_select_brand</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle is not in place.</t>
+          <t xml:space="preserve">Brand</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t xml:space="preserve">哺乳瓶がセットされていません。</t>
+          <t xml:space="preserve">ブランド</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶瓶未就位。</t>
+          <t xml:space="preserve">品牌</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶瓶未就位。</t>
+          <t xml:space="preserve">品牌</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle is not in place.</t>
+          <t xml:space="preserve">Brand</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle is not in place.</t>
+          <t xml:space="preserve">Brand</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t xml:space="preserve">block_hot_alert</t>
+          <t xml:space="preserve">powder_brand_select_series</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t xml:space="preserve">Device is too hot. Please wait.</t>
+          <t xml:space="preserve">Series</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t xml:space="preserve">本体が高温です。しばらくお待ちください。</t>
+          <t xml:space="preserve">シリーズ</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t xml:space="preserve">设备温度过高，请稍候。</t>
+          <t xml:space="preserve">系列</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t xml:space="preserve">設備溫度過高，請稍候。</t>
+          <t xml:space="preserve">系列</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t xml:space="preserve">Device is too hot. Please wait.</t>
+          <t xml:space="preserve">Series</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t xml:space="preserve">Device is too hot. Please wait.</t>
+          <t xml:space="preserve">Series</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_none</t>
+          <t xml:space="preserve">powder_brand_select_stage</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Stage</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">段階</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">段数</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">段數</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Stage</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Stage</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_hot</t>
+          <t xml:space="preserve">powder_brand_select_placeholder</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t xml:space="preserve">High temperature alert</t>
+          <t xml:space="preserve">Select</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t xml:space="preserve">High temperature alert</t>
+          <t xml:space="preserve">選択</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t xml:space="preserve">High temperature alert</t>
+          <t xml:space="preserve">请选择</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t xml:space="preserve">High temperature alert</t>
+          <t xml:space="preserve">請選擇</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t xml:space="preserve">High temperature alert</t>
+          <t xml:space="preserve">Select</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t xml:space="preserve">High temperature alert</t>
+          <t xml:space="preserve">Select</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_e01</t>
+          <t xml:space="preserve">powder_brand_sheet_select_brand</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E01</t>
+          <t xml:space="preserve">Select Brand</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E01</t>
+          <t xml:space="preserve">ブランドを選択</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E01</t>
+          <t xml:space="preserve">选择品牌</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E01</t>
+          <t xml:space="preserve">選擇品牌</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E01</t>
+          <t xml:space="preserve">Select Brand</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E01</t>
+          <t xml:space="preserve">Select Brand</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_e02</t>
+          <t xml:space="preserve">powder_brand_sheet_select_series</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E02</t>
+          <t xml:space="preserve">Select Series</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E02</t>
+          <t xml:space="preserve">シリーズを選択</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E02</t>
+          <t xml:space="preserve">选择系列</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E02</t>
+          <t xml:space="preserve">選擇系列</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E02</t>
+          <t xml:space="preserve">Select Series</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E02</t>
+          <t xml:space="preserve">Select Series</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_e03</t>
+          <t xml:space="preserve">powder_brand_sheet_select_stage</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E03</t>
+          <t xml:space="preserve">Select Stage</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t xml:space="preserve">エラー E03</t>
+          <t xml:space="preserve">段階を選択</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t xml:space="preserve">错误 E03</t>
+          <t xml:space="preserve">选择段数</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t xml:space="preserve">錯誤 E03</t>
+          <t xml:space="preserve">選擇段數</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E03</t>
+          <t xml:space="preserve">Select Stage</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error E03</t>
+          <t xml:space="preserve">Select Stage</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_c01</t>
+          <t xml:space="preserve">powder_brand_search_placeholder</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">Search brand...</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">ブランドを検索...</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">搜索品牌...</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">搜尋品牌...</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">Search brand...</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C01</t>
+          <t xml:space="preserve">Search brand...</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_c02</t>
+          <t xml:space="preserve">powder_brand_search_empty</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">No brands match your search.</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">該当するブランドがありません。</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">未找到匹配的品牌。</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">找不到符合的品牌。</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">No brands match your search.</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C02</t>
+          <t xml:space="preserve">No brands match your search.</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_c03</t>
+          <t xml:space="preserve">powder_brand_not_listed</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C03</t>
+          <t xml:space="preserve">Brand not listed? </t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t xml:space="preserve">エラー C03</t>
+          <t xml:space="preserve">ブランドが見つかりませんか？ </t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t xml:space="preserve">错误 C03</t>
+          <t xml:space="preserve">没有您的品牌？ </t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t xml:space="preserve">錯誤 C03</t>
+          <t xml:space="preserve">找不到您的品牌？ </t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C03</t>
+          <t xml:space="preserve">Brand not listed? </t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C03</t>
+          <t xml:space="preserve">Brand not listed? </t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t xml:space="preserve">error_c04</t>
+          <t xml:space="preserve">powder_brand_customize_ratio</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C04</t>
+          <t xml:space="preserve">Customize mixing ratio.</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t xml:space="preserve">エラー C04</t>
+          <t xml:space="preserve">ミックス比率をカスタマイズ</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t xml:space="preserve">错误 C04</t>
+          <t xml:space="preserve">自定义配比</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t xml:space="preserve">錯誤 C04</t>
+          <t xml:space="preserve">自訂配比</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C04</t>
+          <t xml:space="preserve">Customize mixing ratio.</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error C04</t>
+          <t xml:space="preserve">Customize mixing ratio.</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t xml:space="preserve">sensor_milkbox_missing</t>
+          <t xml:space="preserve">powder_brand_custom_label</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder box is not installed.</t>
+          <t xml:space="preserve">Custom</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルクボックスが装着されていません。</t>
+          <t xml:space="preserve">カスタム</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉盒未安装。</t>
+          <t xml:space="preserve">自定义</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉盒未安裝。</t>
+          <t xml:space="preserve">自訂</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder box is not installed.</t>
+          <t xml:space="preserve">Custom</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powder box is not installed.</t>
+          <t xml:space="preserve">Custom</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t xml:space="preserve">sensor_funnel_missing</t>
+          <t xml:space="preserve">powder_brand_custom_water_ml</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Funnel is not installed.</t>
+          <t xml:space="preserve">Water (mL)</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t xml:space="preserve">ファネルが装着されていません。</t>
+          <t xml:space="preserve">水量 (mL)</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t xml:space="preserve">漏斗未安装。</t>
+          <t xml:space="preserve">水量 (mL)</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t xml:space="preserve">漏斗未安裝。</t>
+          <t xml:space="preserve">水量 (mL)</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Funnel is not installed.</t>
+          <t xml:space="preserve">Water (mL)</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Funnel is not installed.</t>
+          <t xml:space="preserve">Water (mL)</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t xml:space="preserve">sensor_bottle_missing</t>
+          <t xml:space="preserve">powder_brand_custom_powder_g</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle is not in place.</t>
+          <t xml:space="preserve">Powder (g)</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t xml:space="preserve">哺乳瓶がセットされていません。</t>
+          <t xml:space="preserve">粉量 (g)</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶瓶未就位。</t>
+          <t xml:space="preserve">粉量 (g)</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶瓶未就位。</t>
+          <t xml:space="preserve">粉量 (g)</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle is not in place.</t>
+          <t xml:space="preserve">Powder (g)</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle is not in place.</t>
+          <t xml:space="preserve">Powder (g)</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t xml:space="preserve">sensor_watertank_missing</t>
+          <t xml:space="preserve">powder_brand_custom_apply</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank is missing or water level is too low.</t>
+          <t xml:space="preserve">Apply</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱が未装着、または水量不足です。</t>
+          <t xml:space="preserve">適用</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱未安装或水量不足。</t>
+          <t xml:space="preserve">应用</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱未安裝或水量不足。</t>
+          <t xml:space="preserve">套用</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank is missing or water level is too low.</t>
+          <t xml:space="preserve">Apply</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank is missing or water level is too low.</t>
+          <t xml:space="preserve">Apply</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_check_toast</t>
+          <t xml:space="preserve">powder_brand_ratio_title</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before brewing.</t>
+          <t xml:space="preserve">Recommended Mix Ratio</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t xml:space="preserve">調乳前にデバイス状態を確認してください。</t>
+          <t xml:space="preserve">推奨ミックス比率</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t xml:space="preserve">冲奶前请先检查设备状态。</t>
+          <t xml:space="preserve">推荐配比</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t xml:space="preserve">沖奶前請先檢查設備狀態。</t>
+          <t xml:space="preserve">建議配比</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before brewing.</t>
+          <t xml:space="preserve">Recommended Mix Ratio</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before brewing.</t>
+          <t xml:space="preserve">Recommended Mix Ratio</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_check_toast_water</t>
+          <t xml:space="preserve">powder_brand_ratio_water</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before water dispensing.</t>
+          <t xml:space="preserve">Water</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t xml:space="preserve">出水前にデバイス状態を確認してください。</t>
+          <t xml:space="preserve">水</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t xml:space="preserve">出水前请先检查设备状态。</t>
+          <t xml:space="preserve">水</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t xml:space="preserve">出水前請先檢查設備狀態。</t>
+          <t xml:space="preserve">水</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before water dispensing.</t>
+          <t xml:space="preserve">Water</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before water dispensing.</t>
+          <t xml:space="preserve">Water</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_check_toast_powder</t>
+          <t xml:space="preserve">powder_brand_ratio_powder</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before formula dispensing.</t>
+          <t xml:space="preserve">Powder</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t xml:space="preserve">出粉前にデバイス状態を確認してください。</t>
+          <t xml:space="preserve">粉ミルク</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t xml:space="preserve">出粉前请先检查设备状态。</t>
+          <t xml:space="preserve">奶粉</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t xml:space="preserve">出粉前請先檢查設備狀態。</t>
+          <t xml:space="preserve">奶粉</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before formula dispensing.</t>
+          <t xml:space="preserve">Powder</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check device status before formula dispensing.</t>
+          <t xml:space="preserve">Powder</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_panel_title</t>
+          <t xml:space="preserve">powder_brand_settings_title</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t xml:space="preserve">Formula brewing is unavailable.</t>
+          <t xml:space="preserve">Powder Brand Settings</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t xml:space="preserve">調乳を開始できません。</t>
+          <t xml:space="preserve">粉ミルクブランド設定</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t xml:space="preserve">无法开始冲奶。</t>
+          <t xml:space="preserve">奶粉品牌设置</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t xml:space="preserve">無法開始沖奶。</t>
+          <t xml:space="preserve">奶粉品牌設定</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t xml:space="preserve">Formula brewing is unavailable.</t>
+          <t xml:space="preserve">Powder Brand Settings</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t xml:space="preserve">Formula brewing is unavailable.</t>
+          <t xml:space="preserve">Powder Brand Settings</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_panel_subtitle</t>
+          <t xml:space="preserve">powder_brand_add_brand</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t xml:space="preserve">Please make sure all the following device assemblies are fully prepared.</t>
+          <t xml:space="preserve">Add Brand</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t xml:space="preserve">以下の装置がすべて正しく準備されていることを確認してください。</t>
+          <t xml:space="preserve">ブランドを追加</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t xml:space="preserve">请确认以下装置均已正确准备就绪。</t>
+          <t xml:space="preserve">添加品牌</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t xml:space="preserve">請確認以下裝置均已正確準備就緒。</t>
+          <t xml:space="preserve">新增品牌</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t xml:space="preserve">Please make sure all the following device assemblies are fully prepared.</t>
+          <t xml:space="preserve">Add Brand</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t xml:space="preserve">Please make sure all the following device assemblies are fully prepared.</t>
+          <t xml:space="preserve">Add Brand</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_mixing_chamber</t>
+          <t xml:space="preserve">powder_brand_empty_message</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixing chamber installed</t>
+          <t xml:space="preserve">No milk powder brands added yet.</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t xml:space="preserve">ミキシングチャンバー装着済み</t>
+          <t xml:space="preserve">粉ミルクブランドはまだ追加されていません。</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t xml:space="preserve">混合舱已安装</t>
+          <t xml:space="preserve">尚未添加奶粉品牌。</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t xml:space="preserve">混合艙已安裝</t>
+          <t xml:space="preserve">尚未新增奶粉品牌。</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixing chamber installed</t>
+          <t xml:space="preserve">No milk powder brands added yet.</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixing chamber installed</t>
+          <t xml:space="preserve">No milk powder brands added yet.</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_water_tank</t>
+          <t xml:space="preserve">powder_brand_batch_delete</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank installed</t>
+          <t xml:space="preserve">Batch Delete</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱装着済み</t>
+          <t xml:space="preserve">一括削除</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱已安装</t>
+          <t xml:space="preserve">批量删除</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱已安裝</t>
+          <t xml:space="preserve">批次刪除</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank installed</t>
+          <t xml:space="preserve">Batch Delete</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank installed</t>
+          <t xml:space="preserve">Batch Delete</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_water_level</t>
+          <t xml:space="preserve">powder_brand_batch_footer_delete</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sufficient water level</t>
+          <t xml:space="preserve">Delete ({0})</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量十分</t>
+          <t xml:space="preserve">Delete ({0})</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量充足</t>
+          <t xml:space="preserve">Delete ({0})</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t xml:space="preserve">水量充足</t>
+          <t xml:space="preserve">Delete ({0})</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sufficient water level</t>
+          <t xml:space="preserve">Delete ({0})</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sufficient water level</t>
+          <t xml:space="preserve">Delete ({0})</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_milk_powder</t>
+          <t xml:space="preserve">powder_brand_batch_confirm_message_one</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk powder container installed</t>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルク容器装着済み</t>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉盒已安装</t>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉盒已安裝</t>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk powder container installed</t>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk powder container installed</t>
+          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_bottle</t>
+          <t xml:space="preserve">powder_brand_batch_confirm_message_many</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle in place</t>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t xml:space="preserve">哺乳瓶セット済み</t>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶瓶已就位</t>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶瓶已就位</t>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle in place</t>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bottle in place</t>
+          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_no_blockage</t>
+          <t xml:space="preserve">powder_brand_batch_delete_title</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t xml:space="preserve">No blockage detected</t>
+          <t xml:space="preserve">Delete Selected Brands?</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t xml:space="preserve">詰まりなし</t>
+          <t xml:space="preserve">選択したブランドを削除しますか？</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t xml:space="preserve">未检测到堵塞</t>
+          <t xml:space="preserve">删除所选品牌？</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t xml:space="preserve">未偵測到堵塞</t>
+          <t xml:space="preserve">刪除所選品牌？</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t xml:space="preserve">No blockage detected</t>
+          <t xml:space="preserve">Delete Selected Brands?</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t xml:space="preserve">No blockage detected</t>
+          <t xml:space="preserve">Delete Selected Brands?</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_water_low_toast</t>
+          <t xml:space="preserve">powder_brand_batch_delete_body</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank low, please refill promptly!</t>
+          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱の水量が不足しています。すぐに補充してください。</t>
+          <t xml:space="preserve">{0}件のブランドを削除しますか？元に戻せません。</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱水量不足，请尽快加水。</t>
+          <t xml:space="preserve">将删除 {0} 个品牌，此操作无法撤销。</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t xml:space="preserve">水箱水量不足，請盡快加水。</t>
+          <t xml:space="preserve">將刪除 {0} 筆品牌，此操作無法復原。</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank low, please refill promptly!</t>
+          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t xml:space="preserve">Water tank low, please refill promptly!</t>
+          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t xml:space="preserve">device_status_temp_unavailable_toast</t>
+          <t xml:space="preserve">powder_brand_delete_title</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t xml:space="preserve">Temperature setting unavailable! Please wait for temperature recovery or adjust tank temp to retry.</t>
+          <t xml:space="preserve">Delete Brand?</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t xml:space="preserve">温度設定が利用できません。温度が回復するまでお待ちいただくか、水箱の温度を調整してから再試行してください。</t>
+          <t xml:space="preserve">ブランドを削除しますか？</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t xml:space="preserve">温度设定不可用！请等待温度恢复或调整水箱温度后重试。</t>
+          <t xml:space="preserve">删除品牌？</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t xml:space="preserve">溫度設定不可用！請等待溫度恢復或調整水箱溫度後重試。</t>
+          <t xml:space="preserve">刪除品牌？</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t xml:space="preserve">Temperature setting unavailable! Please wait for temperature recovery or adjust tank temp to retry.</t>
+          <t xml:space="preserve">Delete Brand?</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t xml:space="preserve">Temperature setting unavailable! Please wait for temperature recovery or adjust tank temp to retry.</t>
+          <t xml:space="preserve">Delete Brand?</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t xml:space="preserve">brand_coming_soon</t>
+          <t xml:space="preserve">powder_brand_delete_body</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand settings will be available in a future update.</t>
+          <t xml:space="preserve">This brand will be removed from your list.</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランド設定は今後のアップデートで提供予定です。</t>
+          <t xml:space="preserve">このブランドはリストから削除されます。</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t xml:space="preserve">品牌设置将在后续版本中提供。</t>
+          <t xml:space="preserve">此品牌将从列表中移除。</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t xml:space="preserve">品牌設定將在後續版本中提供。</t>
+          <t xml:space="preserve">此品牌將從列表中移除。</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand settings will be available in a future update.</t>
+          <t xml:space="preserve">This brand will be removed from your list.</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand settings will be available in a future update.</t>
+          <t xml:space="preserve">This brand will be removed from your list.</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_page_title</t>
+          <t xml:space="preserve">powder_brand_delete_confirm_message</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Milk Powder Brand</t>
+          <t xml:space="preserve">Are you sure you want to delete the brand:
+"{0} / {1} / {2}"?</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルクブランドを追加</t>
+          <t xml:space="preserve">ブランドを削除してもよろしいですか：
+"{0} / {1} / {2}"？</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t xml:space="preserve">添加奶粉品牌</t>
+          <t xml:space="preserve">确定要删除品牌：
+"{0} / {1} / {2}"吗？</t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t xml:space="preserve">新增奶粉品牌</t>
+          <t xml:space="preserve">確定要刪除品牌：
+"{0} / {1} / {2}"嗎？</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Milk Powder Brand</t>
+          <t xml:space="preserve">Are you sure you want to delete the brand:
+"{0} / {1} / {2}"?</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Milk Powder Brand</t>
+          <t xml:space="preserve">Are you sure you want to delete the brand:
+"{0} / {1} / {2}"?</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_edit_page_title</t>
+          <t xml:space="preserve">custom_mix_ratio_page_title</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edit Milk Powder Brand</t>
+          <t xml:space="preserve">Customize Mixing Ratio</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルクブランドを編集</t>
+          <t xml:space="preserve">ミックス比率をカスタマイズ</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t xml:space="preserve">编辑奶粉品牌</t>
+          <t xml:space="preserve">自定义配比</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t xml:space="preserve">編輯奶粉品牌</t>
+          <t xml:space="preserve">自訂配比</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edit Milk Powder Brand</t>
+          <t xml:space="preserve">Customize Mixing Ratio</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edit Milk Powder Brand</t>
+          <t xml:space="preserve">Customize Mixing Ratio</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_custom_ratio_section</t>
+          <t xml:space="preserve">custom_mix_ratio_note</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Ratio</t>
+          <t xml:space="preserve">Note: Once the mixing ratio is set, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t xml:space="preserve">カスタム比率</t>
+          <t xml:space="preserve">注：ミックス比率を設定すると、対応する粉ミルク濃度を自動取得し、調乳比率を算出して表示します。</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t xml:space="preserve">自定义配比</t>
+          <t xml:space="preserve">说明：设置配比后，系统将自动获取对应奶粉浓度，计算并展示冲调比例。</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t xml:space="preserve">自訂配比</t>
+          <t xml:space="preserve">說明：設定配比後，系統將自動取得對應奶粉濃度，計算並顯示沖調比例。</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Ratio</t>
+          <t xml:space="preserve">Note: Once the mixing ratio is set, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Ratio</t>
+          <t xml:space="preserve">Note: Once the mixing ratio is set, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_page_note</t>
+          <t xml:space="preserve">custom_mix_ratio_panel_title</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
+          <t xml:space="preserve">Mix Ratio</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t xml:space="preserve">注意：ブランド・シリーズ・段階を選択すると、対応する粉ミルク濃度を自動取得し、調乳比率を表示します。</t>
+          <t xml:space="preserve">ミックス比率</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t xml:space="preserve">说明：选择品牌、系列和段数后，将自动获取对应奶粉浓度并计算、展示冲调比例。</t>
+          <t xml:space="preserve">配比</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t xml:space="preserve">說明：選擇品牌、系列與段數後，將自動取得對應奶粉濃度並計算、顯示沖調比例。</t>
+          <t xml:space="preserve">配比</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
+          <t xml:space="preserve">Mix Ratio</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t xml:space="preserve">Note: Once the brand, series and stage are chosen, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
+          <t xml:space="preserve">Mix Ratio</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_info_title</t>
+          <t xml:space="preserve">custom_mix_ratio_incomplete</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk Powder Info</t>
+          <t xml:space="preserve">Please enter both water and powder amounts.</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t xml:space="preserve">粉ミルク情報</t>
+          <t xml:space="preserve">水量と粉量の両方を入力してください。</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉信息</t>
+          <t xml:space="preserve">请填写水量和粉量。</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t xml:space="preserve">奶粉資訊</t>
+          <t xml:space="preserve">請填寫水量與粉量。</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk Powder Info</t>
+          <t xml:space="preserve">Please enter both water and powder amounts.</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milk Powder Info</t>
+          <t xml:space="preserve">Please enter both water and powder amounts.</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_select_brand</t>
+          <t xml:space="preserve">custom_mix_ratio_delete_confirm_message</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand</t>
+          <t xml:space="preserve">Are you sure you want to delete the custom mixing ratio:
+"{0}ml / {1}g"?</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランド</t>
+          <t xml:space="preserve">カスタムミックス比率を削除してもよろしいですか：
+"{0}ml / {1}g"？</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t xml:space="preserve">品牌</t>
+          <t xml:space="preserve">确定要删除自定义配比：
+"{0}ml / {1}g"吗？</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t xml:space="preserve">品牌</t>
+          <t xml:space="preserve">確定要刪除自訂配比：
+"{0}ml / {1}g"嗎？</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand</t>
+          <t xml:space="preserve">Are you sure you want to delete the custom mixing ratio:
+"{0}ml / {1}g"?</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brand</t>
+          <t xml:space="preserve">Are you sure you want to delete the custom mixing ratio:
+"{0}ml / {1}g"?</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_select_series</t>
+          <t xml:space="preserve">dp_command_failed</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Could not send the command. Check device connection.</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t xml:space="preserve">シリーズ</t>
+          <t xml:space="preserve">コマンドを送信できませんでした。接続を確認してください。</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t xml:space="preserve">系列</t>
+          <t xml:space="preserve">无法发送指令，请检查设备连接。</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t xml:space="preserve">系列</t>
+          <t xml:space="preserve">無法傳送指令，請檢查裝置連線。</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Could not send the command. Check device connection.</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Series</t>
+          <t xml:space="preserve">Could not send the command. Check device connection.</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_select_stage</t>
+          <t xml:space="preserve">device_power_off</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage</t>
+          <t xml:space="preserve">Device is powered off. Tap the power button to turn on.</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t xml:space="preserve">段階</t>
+          <t xml:space="preserve">電源がオフです。電源ボタンをタップしてオンにしてください。</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t xml:space="preserve">段数</t>
+          <t xml:space="preserve">设备已关机，请点击电源键开机。</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t xml:space="preserve">段數</t>
+          <t xml:space="preserve">裝置已關機，請點擊電源鍵開機。</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage</t>
+          <t xml:space="preserve">Device is powered off. Tap the power button to turn on.</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage</t>
+          <t xml:space="preserve">Device is powered off. Tap the power button to turn on.</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_select_placeholder</t>
+          <t xml:space="preserve">device_settings_unavailable</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select</t>
+          <t xml:space="preserve">Device settings are unavailable.</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t xml:space="preserve">選択</t>
+          <t xml:space="preserve">デバイス設定を開けません。</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t xml:space="preserve">请选择</t>
+          <t xml:space="preserve">无法打开设备设置。</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t xml:space="preserve">請選擇</t>
+          <t xml:space="preserve">無法開啟裝置設定。</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select</t>
+          <t xml:space="preserve">Device settings are unavailable.</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select</t>
+          <t xml:space="preserve">Device settings are unavailable.</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t xml:space="preserve">powder_brand_sheet_select_brand</t>
+          <t xml:space="preserve">device_settings_open_failed</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Brand</t>
+          <t xml:space="preserve">Could not open device settings.</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t xml:space="preserve">ブランドを選択</t>
+          <t xml:space="preserve">デバイス設定を開けませんでした。</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t xml:space="preserve">选择品牌</t>
+          <t xml:space="preserve">无法打开设备设置页。</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t xml:space="preserve">選擇品牌</t>
+          <t xml:space="preserve">無法開啟裝置設定頁。</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select Brand</t>
+          <t xml:space="preserve">Could not open device settings.</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Select Brand</t>
-        </is>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_sheet_select_series</t>
-        </is>
-      </c>
-      <c r="B260" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Select Series</t>
-        </is>
-      </c>
-      <c r="C260" t="inlineStr">
-        <is>
-          <t xml:space="preserve">シリーズを選択</t>
-        </is>
-      </c>
-      <c r="D260" t="inlineStr">
-        <is>
-          <t xml:space="preserve">选择系列</t>
-        </is>
-      </c>
-      <c r="E260" t="inlineStr">
-        <is>
-          <t xml:space="preserve">選擇系列</t>
-        </is>
-      </c>
-      <c r="F260" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Select Series</t>
-        </is>
-      </c>
-      <c r="G260" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Select Series</t>
-        </is>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_sheet_select_stage</t>
-        </is>
-      </c>
-      <c r="B261" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Select Stage</t>
-        </is>
-      </c>
-      <c r="C261" t="inlineStr">
-        <is>
-          <t xml:space="preserve">段階を選択</t>
-        </is>
-      </c>
-      <c r="D261" t="inlineStr">
-        <is>
-          <t xml:space="preserve">选择段数</t>
-        </is>
-      </c>
-      <c r="E261" t="inlineStr">
-        <is>
-          <t xml:space="preserve">選擇段數</t>
-        </is>
-      </c>
-      <c r="F261" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Select Stage</t>
-        </is>
-      </c>
-      <c r="G261" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Select Stage</t>
-        </is>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_search_placeholder</t>
-        </is>
-      </c>
-      <c r="B262" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Search brand...</t>
-        </is>
-      </c>
-      <c r="C262" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ブランドを検索...</t>
-        </is>
-      </c>
-      <c r="D262" t="inlineStr">
-        <is>
-          <t xml:space="preserve">搜索品牌...</t>
-        </is>
-      </c>
-      <c r="E262" t="inlineStr">
-        <is>
-          <t xml:space="preserve">搜尋品牌...</t>
-        </is>
-      </c>
-      <c r="F262" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Search brand...</t>
-        </is>
-      </c>
-      <c r="G262" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Search brand...</t>
-        </is>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_search_empty</t>
-        </is>
-      </c>
-      <c r="B263" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No brands match your search.</t>
-        </is>
-      </c>
-      <c r="C263" t="inlineStr">
-        <is>
-          <t xml:space="preserve">該当するブランドがありません。</t>
-        </is>
-      </c>
-      <c r="D263" t="inlineStr">
-        <is>
-          <t xml:space="preserve">未找到匹配的品牌。</t>
-        </is>
-      </c>
-      <c r="E263" t="inlineStr">
-        <is>
-          <t xml:space="preserve">找不到符合的品牌。</t>
-        </is>
-      </c>
-      <c r="F263" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No brands match your search.</t>
-        </is>
-      </c>
-      <c r="G263" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No brands match your search.</t>
-        </is>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_not_listed</t>
-        </is>
-      </c>
-      <c r="B264" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Brand not listed? </t>
-        </is>
-      </c>
-      <c r="C264" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ブランドが見つかりませんか？ </t>
-        </is>
-      </c>
-      <c r="D264" t="inlineStr">
-        <is>
-          <t xml:space="preserve">没有您的品牌？ </t>
-        </is>
-      </c>
-      <c r="E264" t="inlineStr">
-        <is>
-          <t xml:space="preserve">找不到您的品牌？ </t>
-        </is>
-      </c>
-      <c r="F264" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Brand not listed? </t>
-        </is>
-      </c>
-      <c r="G264" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Brand not listed? </t>
-        </is>
-      </c>
-    </row>
-    <row r="265">
-      <c r="A265" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_customize_ratio</t>
-        </is>
-      </c>
-      <c r="B265" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Customize mixing ratio.</t>
-        </is>
-      </c>
-      <c r="C265" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ミックス比率をカスタマイズ</t>
-        </is>
-      </c>
-      <c r="D265" t="inlineStr">
-        <is>
-          <t xml:space="preserve">自定义配比</t>
-        </is>
-      </c>
-      <c r="E265" t="inlineStr">
-        <is>
-          <t xml:space="preserve">自訂配比</t>
-        </is>
-      </c>
-      <c r="F265" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Customize mixing ratio.</t>
-        </is>
-      </c>
-      <c r="G265" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Customize mixing ratio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="266">
-      <c r="A266" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_custom_label</t>
-        </is>
-      </c>
-      <c r="B266" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Custom</t>
-        </is>
-      </c>
-      <c r="C266" t="inlineStr">
-        <is>
-          <t xml:space="preserve">カスタム</t>
-        </is>
-      </c>
-      <c r="D266" t="inlineStr">
-        <is>
-          <t xml:space="preserve">自定义</t>
-        </is>
-      </c>
-      <c r="E266" t="inlineStr">
-        <is>
-          <t xml:space="preserve">自訂</t>
-        </is>
-      </c>
-      <c r="F266" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Custom</t>
-        </is>
-      </c>
-      <c r="G266" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Custom</t>
-        </is>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_custom_water_ml</t>
-        </is>
-      </c>
-      <c r="B267" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Water (mL)</t>
-        </is>
-      </c>
-      <c r="C267" t="inlineStr">
-        <is>
-          <t xml:space="preserve">水量 (mL)</t>
-        </is>
-      </c>
-      <c r="D267" t="inlineStr">
-        <is>
-          <t xml:space="preserve">水量 (mL)</t>
-        </is>
-      </c>
-      <c r="E267" t="inlineStr">
-        <is>
-          <t xml:space="preserve">水量 (mL)</t>
-        </is>
-      </c>
-      <c r="F267" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Water (mL)</t>
-        </is>
-      </c>
-      <c r="G267" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Water (mL)</t>
-        </is>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_custom_powder_g</t>
-        </is>
-      </c>
-      <c r="B268" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Powder (g)</t>
-        </is>
-      </c>
-      <c r="C268" t="inlineStr">
-        <is>
-          <t xml:space="preserve">粉量 (g)</t>
-        </is>
-      </c>
-      <c r="D268" t="inlineStr">
-        <is>
-          <t xml:space="preserve">粉量 (g)</t>
-        </is>
-      </c>
-      <c r="E268" t="inlineStr">
-        <is>
-          <t xml:space="preserve">粉量 (g)</t>
-        </is>
-      </c>
-      <c r="F268" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Powder (g)</t>
-        </is>
-      </c>
-      <c r="G268" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Powder (g)</t>
-        </is>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_custom_apply</t>
-        </is>
-      </c>
-      <c r="B269" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Apply</t>
-        </is>
-      </c>
-      <c r="C269" t="inlineStr">
-        <is>
-          <t xml:space="preserve">適用</t>
-        </is>
-      </c>
-      <c r="D269" t="inlineStr">
-        <is>
-          <t xml:space="preserve">应用</t>
-        </is>
-      </c>
-      <c r="E269" t="inlineStr">
-        <is>
-          <t xml:space="preserve">套用</t>
-        </is>
-      </c>
-      <c r="F269" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Apply</t>
-        </is>
-      </c>
-      <c r="G269" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Apply</t>
-        </is>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_ratio_title</t>
-        </is>
-      </c>
-      <c r="B270" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Recommended Mix Ratio</t>
-        </is>
-      </c>
-      <c r="C270" t="inlineStr">
-        <is>
-          <t xml:space="preserve">推奨ミックス比率</t>
-        </is>
-      </c>
-      <c r="D270" t="inlineStr">
-        <is>
-          <t xml:space="preserve">推荐配比</t>
-        </is>
-      </c>
-      <c r="E270" t="inlineStr">
-        <is>
-          <t xml:space="preserve">建議配比</t>
-        </is>
-      </c>
-      <c r="F270" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Recommended Mix Ratio</t>
-        </is>
-      </c>
-      <c r="G270" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Recommended Mix Ratio</t>
-        </is>
-      </c>
-    </row>
-    <row r="271">
-      <c r="A271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_ratio_water</t>
-        </is>
-      </c>
-      <c r="B271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Water</t>
-        </is>
-      </c>
-      <c r="C271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">水</t>
-        </is>
-      </c>
-      <c r="D271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">水</t>
-        </is>
-      </c>
-      <c r="E271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">水</t>
-        </is>
-      </c>
-      <c r="F271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Water</t>
-        </is>
-      </c>
-      <c r="G271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Water</t>
-        </is>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_ratio_powder</t>
-        </is>
-      </c>
-      <c r="B272" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Powder</t>
-        </is>
-      </c>
-      <c r="C272" t="inlineStr">
-        <is>
-          <t xml:space="preserve">粉ミルク</t>
-        </is>
-      </c>
-      <c r="D272" t="inlineStr">
-        <is>
-          <t xml:space="preserve">奶粉</t>
-        </is>
-      </c>
-      <c r="E272" t="inlineStr">
-        <is>
-          <t xml:space="preserve">奶粉</t>
-        </is>
-      </c>
-      <c r="F272" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Powder</t>
-        </is>
-      </c>
-      <c r="G272" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Powder</t>
-        </is>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_settings_title</t>
-        </is>
-      </c>
-      <c r="B273" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Powder Brand Settings</t>
-        </is>
-      </c>
-      <c r="C273" t="inlineStr">
-        <is>
-          <t xml:space="preserve">粉ミルクブランド設定</t>
-        </is>
-      </c>
-      <c r="D273" t="inlineStr">
-        <is>
-          <t xml:space="preserve">奶粉品牌设置</t>
-        </is>
-      </c>
-      <c r="E273" t="inlineStr">
-        <is>
-          <t xml:space="preserve">奶粉品牌設定</t>
-        </is>
-      </c>
-      <c r="F273" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Powder Brand Settings</t>
-        </is>
-      </c>
-      <c r="G273" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Powder Brand Settings</t>
-        </is>
-      </c>
-    </row>
-    <row r="274">
-      <c r="A274" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_add_brand</t>
-        </is>
-      </c>
-      <c r="B274" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Add Brand</t>
-        </is>
-      </c>
-      <c r="C274" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ブランドを追加</t>
-        </is>
-      </c>
-      <c r="D274" t="inlineStr">
-        <is>
-          <t xml:space="preserve">添加品牌</t>
-        </is>
-      </c>
-      <c r="E274" t="inlineStr">
-        <is>
-          <t xml:space="preserve">新增品牌</t>
-        </is>
-      </c>
-      <c r="F274" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Add Brand</t>
-        </is>
-      </c>
-      <c r="G274" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Add Brand</t>
-        </is>
-      </c>
-    </row>
-    <row r="275">
-      <c r="A275" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_empty_message</t>
-        </is>
-      </c>
-      <c r="B275" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No milk powder brands added yet.</t>
-        </is>
-      </c>
-      <c r="C275" t="inlineStr">
-        <is>
-          <t xml:space="preserve">粉ミルクブランドはまだ追加されていません。</t>
-        </is>
-      </c>
-      <c r="D275" t="inlineStr">
-        <is>
-          <t xml:space="preserve">尚未添加奶粉品牌。</t>
-        </is>
-      </c>
-      <c r="E275" t="inlineStr">
-        <is>
-          <t xml:space="preserve">尚未新增奶粉品牌。</t>
-        </is>
-      </c>
-      <c r="F275" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No milk powder brands added yet.</t>
-        </is>
-      </c>
-      <c r="G275" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No milk powder brands added yet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="276">
-      <c r="A276" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_batch_delete</t>
-        </is>
-      </c>
-      <c r="B276" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Batch Delete</t>
-        </is>
-      </c>
-      <c r="C276" t="inlineStr">
-        <is>
-          <t xml:space="preserve">一括削除</t>
-        </is>
-      </c>
-      <c r="D276" t="inlineStr">
-        <is>
-          <t xml:space="preserve">批量删除</t>
-        </is>
-      </c>
-      <c r="E276" t="inlineStr">
-        <is>
-          <t xml:space="preserve">批次刪除</t>
-        </is>
-      </c>
-      <c r="F276" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Batch Delete</t>
-        </is>
-      </c>
-      <c r="G276" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Batch Delete</t>
-        </is>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_batch_footer_delete</t>
-        </is>
-      </c>
-      <c r="B277" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Delete ({0})</t>
-        </is>
-      </c>
-      <c r="C277" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Delete ({0})</t>
-        </is>
-      </c>
-      <c r="D277" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Delete ({0})</t>
-        </is>
-      </c>
-      <c r="E277" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Delete ({0})</t>
-        </is>
-      </c>
-      <c r="F277" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Delete ({0})</t>
-        </is>
-      </c>
-      <c r="G277" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Delete ({0})</t>
-        </is>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_batch_confirm_message_one</t>
-        </is>
-      </c>
-      <c r="B278" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
-        </is>
-      </c>
-      <c r="C278" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
-        </is>
-      </c>
-      <c r="D278" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
-        </is>
-      </c>
-      <c r="E278" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
-        </is>
-      </c>
-      <c r="F278" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
-        </is>
-      </c>
-      <c r="G278" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete this formula?</t>
-        </is>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_batch_confirm_message_many</t>
-        </is>
-      </c>
-      <c r="B279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
-        </is>
-      </c>
-      <c r="C279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
-        </is>
-      </c>
-      <c r="D279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
-        </is>
-      </c>
-      <c r="E279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
-        </is>
-      </c>
-      <c r="F279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
-        </is>
-      </c>
-      <c r="G279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete these {0} formulas?</t>
-        </is>
-      </c>
-    </row>
-    <row r="280">
-      <c r="A280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_batch_delete_title</t>
-        </is>
-      </c>
-      <c r="B280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Delete Selected Brands?</t>
-        </is>
-      </c>
-      <c r="C280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">選択したブランドを削除しますか？</t>
-        </is>
-      </c>
-      <c r="D280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">删除所选品牌？</t>
-        </is>
-      </c>
-      <c r="E280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">刪除所選品牌？</t>
-        </is>
-      </c>
-      <c r="F280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Delete Selected Brands?</t>
-        </is>
-      </c>
-      <c r="G280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Delete Selected Brands?</t>
-        </is>
-      </c>
-    </row>
-    <row r="281">
-      <c r="A281" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_batch_delete_body</t>
-        </is>
-      </c>
-      <c r="B281" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
-        </is>
-      </c>
-      <c r="C281" t="inlineStr">
-        <is>
-          <t xml:space="preserve">{0}件のブランドを削除しますか？元に戻せません。</t>
-        </is>
-      </c>
-      <c r="D281" t="inlineStr">
-        <is>
-          <t xml:space="preserve">将删除 {0} 个品牌，此操作无法撤销。</t>
-        </is>
-      </c>
-      <c r="E281" t="inlineStr">
-        <is>
-          <t xml:space="preserve">將刪除 {0} 筆品牌，此操作無法復原。</t>
-        </is>
-      </c>
-      <c r="F281" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
-        </is>
-      </c>
-      <c r="G281" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Delete {0} brand(s)? This cannot be undone.</t>
-        </is>
-      </c>
-    </row>
-    <row r="282">
-      <c r="A282" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_delete_title</t>
-        </is>
-      </c>
-      <c r="B282" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Delete Brand?</t>
-        </is>
-      </c>
-      <c r="C282" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ブランドを削除しますか？</t>
-        </is>
-      </c>
-      <c r="D282" t="inlineStr">
-        <is>
-          <t xml:space="preserve">删除品牌？</t>
-        </is>
-      </c>
-      <c r="E282" t="inlineStr">
-        <is>
-          <t xml:space="preserve">刪除品牌？</t>
-        </is>
-      </c>
-      <c r="F282" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Delete Brand?</t>
-        </is>
-      </c>
-      <c r="G282" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Delete Brand?</t>
-        </is>
-      </c>
-    </row>
-    <row r="283">
-      <c r="A283" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_delete_body</t>
-        </is>
-      </c>
-      <c r="B283" t="inlineStr">
-        <is>
-          <t xml:space="preserve">This brand will be removed from your list.</t>
-        </is>
-      </c>
-      <c r="C283" t="inlineStr">
-        <is>
-          <t xml:space="preserve">このブランドはリストから削除されます。</t>
-        </is>
-      </c>
-      <c r="D283" t="inlineStr">
-        <is>
-          <t xml:space="preserve">此品牌将从列表中移除。</t>
-        </is>
-      </c>
-      <c r="E283" t="inlineStr">
-        <is>
-          <t xml:space="preserve">此品牌將從列表中移除。</t>
-        </is>
-      </c>
-      <c r="F283" t="inlineStr">
-        <is>
-          <t xml:space="preserve">This brand will be removed from your list.</t>
-        </is>
-      </c>
-      <c r="G283" t="inlineStr">
-        <is>
-          <t xml:space="preserve">This brand will be removed from your list.</t>
-        </is>
-      </c>
-    </row>
-    <row r="284">
-      <c r="A284" t="inlineStr">
-        <is>
-          <t xml:space="preserve">powder_brand_delete_confirm_message</t>
-        </is>
-      </c>
-      <c r="B284" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete the brand:
-"{0} / {1} / {2}"?</t>
-        </is>
-      </c>
-      <c r="C284" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ブランドを削除してもよろしいですか：
-"{0} / {1} / {2}"？</t>
-        </is>
-      </c>
-      <c r="D284" t="inlineStr">
-        <is>
-          <t xml:space="preserve">确定要删除品牌：
-"{0} / {1} / {2}"吗？</t>
-        </is>
-      </c>
-      <c r="E284" t="inlineStr">
-        <is>
-          <t xml:space="preserve">確定要刪除品牌：
-"{0} / {1} / {2}"嗎？</t>
-        </is>
-      </c>
-      <c r="F284" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete the brand:
-"{0} / {1} / {2}"?</t>
-        </is>
-      </c>
-      <c r="G284" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete the brand:
-"{0} / {1} / {2}"?</t>
-        </is>
-      </c>
-    </row>
-    <row r="285">
-      <c r="A285" t="inlineStr">
-        <is>
-          <t xml:space="preserve">custom_mix_ratio_page_title</t>
-        </is>
-      </c>
-      <c r="B285" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Customize Mixing Ratio</t>
-        </is>
-      </c>
-      <c r="C285" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ミックス比率をカスタマイズ</t>
-        </is>
-      </c>
-      <c r="D285" t="inlineStr">
-        <is>
-          <t xml:space="preserve">自定义配比</t>
-        </is>
-      </c>
-      <c r="E285" t="inlineStr">
-        <is>
-          <t xml:space="preserve">自訂配比</t>
-        </is>
-      </c>
-      <c r="F285" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Customize Mixing Ratio</t>
-        </is>
-      </c>
-      <c r="G285" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Customize Mixing Ratio</t>
-        </is>
-      </c>
-    </row>
-    <row r="286">
-      <c r="A286" t="inlineStr">
-        <is>
-          <t xml:space="preserve">custom_mix_ratio_note</t>
-        </is>
-      </c>
-      <c r="B286" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Note: Once the mixing ratio is set, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
-        </is>
-      </c>
-      <c r="C286" t="inlineStr">
-        <is>
-          <t xml:space="preserve">注：ミックス比率を設定すると、対応する粉ミルク濃度を自動取得し、調乳比率を算出して表示します。</t>
-        </is>
-      </c>
-      <c r="D286" t="inlineStr">
-        <is>
-          <t xml:space="preserve">说明：设置配比后，系统将自动获取对应奶粉浓度，计算并展示冲调比例。</t>
-        </is>
-      </c>
-      <c r="E286" t="inlineStr">
-        <is>
-          <t xml:space="preserve">說明：設定配比後，系統將自動取得對應奶粉濃度，計算並顯示沖調比例。</t>
-        </is>
-      </c>
-      <c r="F286" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Note: Once the mixing ratio is set, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
-        </is>
-      </c>
-      <c r="G286" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Note: Once the mixing ratio is set, we will automatically retrieve the corresponding milk powder concentration to compute and present the preparation ratio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="287">
-      <c r="A287" t="inlineStr">
-        <is>
-          <t xml:space="preserve">custom_mix_ratio_panel_title</t>
-        </is>
-      </c>
-      <c r="B287" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mix Ratio</t>
-        </is>
-      </c>
-      <c r="C287" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ミックス比率</t>
-        </is>
-      </c>
-      <c r="D287" t="inlineStr">
-        <is>
-          <t xml:space="preserve">配比</t>
-        </is>
-      </c>
-      <c r="E287" t="inlineStr">
-        <is>
-          <t xml:space="preserve">配比</t>
-        </is>
-      </c>
-      <c r="F287" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mix Ratio</t>
-        </is>
-      </c>
-      <c r="G287" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mix Ratio</t>
-        </is>
-      </c>
-    </row>
-    <row r="288">
-      <c r="A288" t="inlineStr">
-        <is>
-          <t xml:space="preserve">custom_mix_ratio_incomplete</t>
-        </is>
-      </c>
-      <c r="B288" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Please enter both water and powder amounts.</t>
-        </is>
-      </c>
-      <c r="C288" t="inlineStr">
-        <is>
-          <t xml:space="preserve">水量と粉量の両方を入力してください。</t>
-        </is>
-      </c>
-      <c r="D288" t="inlineStr">
-        <is>
-          <t xml:space="preserve">请填写水量和粉量。</t>
-        </is>
-      </c>
-      <c r="E288" t="inlineStr">
-        <is>
-          <t xml:space="preserve">請填寫水量與粉量。</t>
-        </is>
-      </c>
-      <c r="F288" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Please enter both water and powder amounts.</t>
-        </is>
-      </c>
-      <c r="G288" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Please enter both water and powder amounts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="289">
-      <c r="A289" t="inlineStr">
-        <is>
-          <t xml:space="preserve">custom_mix_ratio_delete_confirm_message</t>
-        </is>
-      </c>
-      <c r="B289" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete the custom mixing ratio:
-"{0}ml / {1}g"?</t>
-        </is>
-      </c>
-      <c r="C289" t="inlineStr">
-        <is>
-          <t xml:space="preserve">カスタムミックス比率を削除してもよろしいですか：
-"{0}ml / {1}g"？</t>
-        </is>
-      </c>
-      <c r="D289" t="inlineStr">
-        <is>
-          <t xml:space="preserve">确定要删除自定义配比：
-"{0}ml / {1}g"吗？</t>
-        </is>
-      </c>
-      <c r="E289" t="inlineStr">
-        <is>
-          <t xml:space="preserve">確定要刪除自訂配比：
-"{0}ml / {1}g"嗎？</t>
-        </is>
-      </c>
-      <c r="F289" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete the custom mixing ratio:
-"{0}ml / {1}g"?</t>
-        </is>
-      </c>
-      <c r="G289" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Are you sure you want to delete the custom mixing ratio:
-"{0}ml / {1}g"?</t>
-        </is>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dp_command_failed</t>
-        </is>
-      </c>
-      <c r="B290" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Could not send the command. Check device connection.</t>
-        </is>
-      </c>
-      <c r="C290" t="inlineStr">
-        <is>
-          <t xml:space="preserve">コマンドを送信できませんでした。接続を確認してください。</t>
-        </is>
-      </c>
-      <c r="D290" t="inlineStr">
-        <is>
-          <t xml:space="preserve">无法发送指令，请检查设备连接。</t>
-        </is>
-      </c>
-      <c r="E290" t="inlineStr">
-        <is>
-          <t xml:space="preserve">無法傳送指令，請檢查裝置連線。</t>
-        </is>
-      </c>
-      <c r="F290" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Could not send the command. Check device connection.</t>
-        </is>
-      </c>
-      <c r="G290" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Could not send the command. Check device connection.</t>
-        </is>
-      </c>
-    </row>
-    <row r="291">
-      <c r="A291" t="inlineStr">
-        <is>
-          <t xml:space="preserve">device_power_off</t>
-        </is>
-      </c>
-      <c r="B291" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Device is powered off. Tap the power button to turn on.</t>
-        </is>
-      </c>
-      <c r="C291" t="inlineStr">
-        <is>
-          <t xml:space="preserve">電源がオフです。電源ボタンをタップしてオンにしてください。</t>
-        </is>
-      </c>
-      <c r="D291" t="inlineStr">
-        <is>
-          <t xml:space="preserve">设备已关机，请点击电源键开机。</t>
-        </is>
-      </c>
-      <c r="E291" t="inlineStr">
-        <is>
-          <t xml:space="preserve">裝置已關機，請點擊電源鍵開機。</t>
-        </is>
-      </c>
-      <c r="F291" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Device is powered off. Tap the power button to turn on.</t>
-        </is>
-      </c>
-      <c r="G291" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Device is powered off. Tap the power button to turn on.</t>
-        </is>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" t="inlineStr">
-        <is>
-          <t xml:space="preserve">device_settings_unavailable</t>
-        </is>
-      </c>
-      <c r="B292" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Device settings are unavailable.</t>
-        </is>
-      </c>
-      <c r="C292" t="inlineStr">
-        <is>
-          <t xml:space="preserve">デバイス設定を開けません。</t>
-        </is>
-      </c>
-      <c r="D292" t="inlineStr">
-        <is>
-          <t xml:space="preserve">无法打开设备设置。</t>
-        </is>
-      </c>
-      <c r="E292" t="inlineStr">
-        <is>
-          <t xml:space="preserve">無法開啟裝置設定。</t>
-        </is>
-      </c>
-      <c r="F292" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Device settings are unavailable.</t>
-        </is>
-      </c>
-      <c r="G292" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Device settings are unavailable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" t="inlineStr">
-        <is>
-          <t xml:space="preserve">device_settings_open_failed</t>
-        </is>
-      </c>
-      <c r="B293" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Could not open device settings.</t>
-        </is>
-      </c>
-      <c r="C293" t="inlineStr">
-        <is>
-          <t xml:space="preserve">デバイス設定を開けませんでした。</t>
-        </is>
-      </c>
-      <c r="D293" t="inlineStr">
-        <is>
-          <t xml:space="preserve">无法打开设备设置页。</t>
-        </is>
-      </c>
-      <c r="E293" t="inlineStr">
-        <is>
-          <t xml:space="preserve">無法開啟裝置設定頁。</t>
-        </is>
-      </c>
-      <c r="F293" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Could not open device settings.</t>
-        </is>
-      </c>
-      <c r="G293" t="inlineStr">
         <is>
           <t xml:space="preserve">Could not open device settings.</t>
         </is>

</xml_diff>